<commit_message>
Remove artificial data generation - extract only real DOCX values
Co-authored-by: danieljohnconstantine-a11y <229551202+danieljohnconstantine-a11y@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/all_dogs_master.xlsx
+++ b/outputs/all_dogs_master.xlsx
@@ -789,9 +789,7 @@
           <t>PARADISE FLYER</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>62.46385193753615</v>
-      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
@@ -825,15 +823,9 @@
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="n">
-        <v>62.46385193753615</v>
-      </c>
-      <c r="AF3" t="n">
-        <v>62.46385193753615</v>
-      </c>
-      <c r="AG3" t="n">
-        <v>62.46385193753615</v>
-      </c>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
       <c r="AH3" t="inlineStr">
         <is>
           <t>6/11/2025</t>
@@ -977,9 +969,7 @@
           <t>SCELZI</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>62.1195652173913</v>
-      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
@@ -1013,15 +1003,9 @@
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="n">
-        <v>62.1195652173913</v>
-      </c>
-      <c r="AF5" t="n">
-        <v>62.1195652173913</v>
-      </c>
-      <c r="AG5" t="n">
-        <v>62.1195652173913</v>
-      </c>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
       <c r="AH5" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -1165,9 +1149,7 @@
           <t>YUNDERUP TAMMY</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v>61.29398410896709</v>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
@@ -1201,15 +1183,9 @@
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="n">
-        <v>61.29398410896709</v>
-      </c>
-      <c r="AF7" t="n">
-        <v>61.29398410896709</v>
-      </c>
-      <c r="AG7" t="n">
-        <v>61.29398410896709</v>
-      </c>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
       <c r="AH7" t="inlineStr">
         <is>
           <t>16/10/2025</t>
@@ -1433,9 +1409,7 @@
           <t>PANTHERS MAGIC</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>63.10344827586208</v>
-      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
@@ -1469,15 +1443,9 @@
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="inlineStr"/>
-      <c r="AE10" t="n">
-        <v>63.10344827586208</v>
-      </c>
-      <c r="AF10" t="n">
-        <v>63.10344827586208</v>
-      </c>
-      <c r="AG10" t="n">
-        <v>63.10344827586208</v>
-      </c>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr"/>
       <c r="AH10" t="inlineStr">
         <is>
           <t>4/11/2025</t>
@@ -1621,9 +1589,7 @@
           <t>DON'T PLAY GAMES</t>
         </is>
       </c>
-      <c r="E12" t="n">
-        <v>63.85809312638581</v>
-      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
@@ -1657,15 +1623,9 @@
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr"/>
-      <c r="AE12" t="n">
-        <v>63.85809312638581</v>
-      </c>
-      <c r="AF12" t="n">
-        <v>63.85809312638581</v>
-      </c>
-      <c r="AG12" t="n">
-        <v>63.85809312638581</v>
-      </c>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
+      <c r="AG12" t="inlineStr"/>
       <c r="AH12" t="inlineStr">
         <is>
           <t>4/11/2025</t>
@@ -1809,9 +1769,7 @@
           <t>BOILER MAKER</t>
         </is>
       </c>
-      <c r="E14" t="n">
-        <v>62.46385193753615</v>
-      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
@@ -1845,15 +1803,9 @@
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr"/>
       <c r="AD14" t="inlineStr"/>
-      <c r="AE14" t="n">
-        <v>62.46385193753615</v>
-      </c>
-      <c r="AF14" t="n">
-        <v>62.46385193753615</v>
-      </c>
-      <c r="AG14" t="n">
-        <v>62.46385193753615</v>
-      </c>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
+      <c r="AG14" t="inlineStr"/>
       <c r="AH14" t="inlineStr">
         <is>
           <t>6/11/2025</t>
@@ -1997,9 +1949,7 @@
           <t>THANK YOU JOE</t>
         </is>
       </c>
-      <c r="E16" t="n">
-        <v>63.44125809435707</v>
-      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
@@ -2033,15 +1983,9 @@
       <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="inlineStr"/>
-      <c r="AE16" t="n">
-        <v>63.44125809435707</v>
-      </c>
-      <c r="AF16" t="n">
-        <v>63.44125809435707</v>
-      </c>
-      <c r="AG16" t="n">
-        <v>63.44125809435707</v>
-      </c>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr"/>
+      <c r="AG16" t="inlineStr"/>
       <c r="AH16" t="inlineStr">
         <is>
           <t>22/10/2025</t>
@@ -2185,9 +2129,7 @@
           <t>HARMONY RHYTHM</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>62.68738574040219</v>
-      </c>
+      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -2221,15 +2163,9 @@
       <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="inlineStr"/>
       <c r="AD18" t="inlineStr"/>
-      <c r="AE18" t="n">
-        <v>62.68738574040219</v>
-      </c>
-      <c r="AF18" t="n">
-        <v>62.68738574040219</v>
-      </c>
-      <c r="AG18" t="n">
-        <v>62.68738574040219</v>
-      </c>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr"/>
+      <c r="AG18" t="inlineStr"/>
       <c r="AH18" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -2373,9 +2309,7 @@
           <t>SUNSET SKYLIGHT</t>
         </is>
       </c>
-      <c r="E20" t="n">
-        <v>62.46385193753615</v>
-      </c>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
@@ -2409,15 +2343,9 @@
       <c r="AB20" t="inlineStr"/>
       <c r="AC20" t="inlineStr"/>
       <c r="AD20" t="inlineStr"/>
-      <c r="AE20" t="n">
-        <v>62.46385193753615</v>
-      </c>
-      <c r="AF20" t="n">
-        <v>62.46385193753615</v>
-      </c>
-      <c r="AG20" t="n">
-        <v>62.46385193753615</v>
-      </c>
+      <c r="AE20" t="inlineStr"/>
+      <c r="AF20" t="inlineStr"/>
+      <c r="AG20" t="inlineStr"/>
       <c r="AH20" t="inlineStr">
         <is>
           <t>6/11/2025</t>
@@ -2561,9 +2489,7 @@
           <t>KILLER KELLY</t>
         </is>
       </c>
-      <c r="E22" t="n">
-        <v>62.23230490018149</v>
-      </c>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
@@ -2597,15 +2523,9 @@
       <c r="AB22" t="inlineStr"/>
       <c r="AC22" t="inlineStr"/>
       <c r="AD22" t="inlineStr"/>
-      <c r="AE22" t="n">
-        <v>62.23230490018149</v>
-      </c>
-      <c r="AF22" t="n">
-        <v>62.23230490018149</v>
-      </c>
-      <c r="AG22" t="n">
-        <v>62.23230490018149</v>
-      </c>
+      <c r="AE22" t="inlineStr"/>
+      <c r="AF22" t="inlineStr"/>
+      <c r="AG22" t="inlineStr"/>
       <c r="AH22" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -2749,9 +2669,7 @@
           <t>RED HOT BERNIE</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>62.97709923664122</v>
-      </c>
+      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
@@ -2785,15 +2703,9 @@
       <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="inlineStr"/>
       <c r="AD24" t="inlineStr"/>
-      <c r="AE24" t="n">
-        <v>62.97709923664122</v>
-      </c>
-      <c r="AF24" t="n">
-        <v>62.97709923664122</v>
-      </c>
-      <c r="AG24" t="n">
-        <v>62.97709923664122</v>
-      </c>
+      <c r="AE24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr"/>
+      <c r="AG24" t="inlineStr"/>
       <c r="AH24" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -2937,9 +2849,7 @@
           <t>PREDATOR GUNDI</t>
         </is>
       </c>
-      <c r="E26" t="n">
-        <v>60.69895769466586</v>
-      </c>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
@@ -2973,15 +2883,9 @@
       <c r="AB26" t="inlineStr"/>
       <c r="AC26" t="inlineStr"/>
       <c r="AD26" t="inlineStr"/>
-      <c r="AE26" t="n">
-        <v>60.69895769466586</v>
-      </c>
-      <c r="AF26" t="n">
-        <v>60.69895769466586</v>
-      </c>
-      <c r="AG26" t="n">
-        <v>60.69895769466586</v>
-      </c>
+      <c r="AE26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr"/>
+      <c r="AG26" t="inlineStr"/>
       <c r="AH26" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -3125,9 +3029,7 @@
           <t>BERRIGAN DRIVE</t>
         </is>
       </c>
-      <c r="E28" t="n">
-        <v>61.47915732855223</v>
-      </c>
+      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
@@ -3161,15 +3063,9 @@
       <c r="AB28" t="inlineStr"/>
       <c r="AC28" t="inlineStr"/>
       <c r="AD28" t="inlineStr"/>
-      <c r="AE28" t="n">
-        <v>61.47915732855223</v>
-      </c>
-      <c r="AF28" t="n">
-        <v>61.47915732855223</v>
-      </c>
-      <c r="AG28" t="n">
-        <v>61.47915732855223</v>
-      </c>
+      <c r="AE28" t="inlineStr"/>
+      <c r="AF28" t="inlineStr"/>
+      <c r="AG28" t="inlineStr"/>
       <c r="AH28" t="inlineStr">
         <is>
           <t>22/10/2025</t>
@@ -3245,9 +3141,7 @@
           <t>HANNAH'S PASSION</t>
         </is>
       </c>
-      <c r="E29" t="n">
-        <v>62.048392442824</v>
-      </c>
+      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
@@ -3281,15 +3175,9 @@
       <c r="AB29" t="inlineStr"/>
       <c r="AC29" t="inlineStr"/>
       <c r="AD29" t="inlineStr"/>
-      <c r="AE29" t="n">
-        <v>62.048392442824</v>
-      </c>
-      <c r="AF29" t="n">
-        <v>62.048392442824</v>
-      </c>
-      <c r="AG29" t="n">
-        <v>62.048392442824</v>
-      </c>
+      <c r="AE29" t="inlineStr"/>
+      <c r="AF29" t="inlineStr"/>
+      <c r="AG29" t="inlineStr"/>
       <c r="AH29" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -3433,9 +3321,7 @@
           <t>AUREATE</t>
         </is>
       </c>
-      <c r="E31" t="n">
-        <v>62.048392442824</v>
-      </c>
+      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
@@ -3469,15 +3355,9 @@
       <c r="AB31" t="inlineStr"/>
       <c r="AC31" t="inlineStr"/>
       <c r="AD31" t="inlineStr"/>
-      <c r="AE31" t="n">
-        <v>62.048392442824</v>
-      </c>
-      <c r="AF31" t="n">
-        <v>62.048392442824</v>
-      </c>
-      <c r="AG31" t="n">
-        <v>62.048392442824</v>
-      </c>
+      <c r="AE31" t="inlineStr"/>
+      <c r="AF31" t="inlineStr"/>
+      <c r="AG31" t="inlineStr"/>
       <c r="AH31" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -3621,9 +3501,7 @@
           <t>WYONG EL PASO</t>
         </is>
       </c>
-      <c r="E33" t="n">
-        <v>62.17203586848224</v>
-      </c>
+      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
@@ -3657,15 +3535,9 @@
       <c r="AB33" t="inlineStr"/>
       <c r="AC33" t="inlineStr"/>
       <c r="AD33" t="inlineStr"/>
-      <c r="AE33" t="n">
-        <v>62.17203586848224</v>
-      </c>
-      <c r="AF33" t="n">
-        <v>62.17203586848224</v>
-      </c>
-      <c r="AG33" t="n">
-        <v>62.17203586848224</v>
-      </c>
+      <c r="AE33" t="inlineStr"/>
+      <c r="AF33" t="inlineStr"/>
+      <c r="AG33" t="inlineStr"/>
       <c r="AH33" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -3809,9 +3681,7 @@
           <t>LADY FREYA</t>
         </is>
       </c>
-      <c r="E35" t="n">
-        <v>62.74473924977127</v>
-      </c>
+      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
@@ -3845,15 +3715,9 @@
       <c r="AB35" t="inlineStr"/>
       <c r="AC35" t="inlineStr"/>
       <c r="AD35" t="inlineStr"/>
-      <c r="AE35" t="n">
-        <v>62.74473924977127</v>
-      </c>
-      <c r="AF35" t="n">
-        <v>62.74473924977127</v>
-      </c>
-      <c r="AG35" t="n">
-        <v>62.74473924977127</v>
-      </c>
+      <c r="AE35" t="inlineStr"/>
+      <c r="AF35" t="inlineStr"/>
+      <c r="AG35" t="inlineStr"/>
       <c r="AH35" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -3997,9 +3861,7 @@
           <t>CANYA BON BON</t>
         </is>
       </c>
-      <c r="E37" t="n">
-        <v>61.22285332442365</v>
-      </c>
+      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
@@ -4033,15 +3895,9 @@
       <c r="AB37" t="inlineStr"/>
       <c r="AC37" t="inlineStr"/>
       <c r="AD37" t="inlineStr"/>
-      <c r="AE37" t="n">
-        <v>61.22285332442365</v>
-      </c>
-      <c r="AF37" t="n">
-        <v>61.22285332442365</v>
-      </c>
-      <c r="AG37" t="n">
-        <v>61.22285332442365</v>
-      </c>
+      <c r="AE37" t="inlineStr"/>
+      <c r="AF37" t="inlineStr"/>
+      <c r="AG37" t="inlineStr"/>
       <c r="AH37" t="inlineStr">
         <is>
           <t>27/10/2025</t>
@@ -4185,9 +4041,7 @@
           <t>CYCLONIC CLINTON</t>
         </is>
       </c>
-      <c r="E39" t="n">
-        <v>61.9054054054054</v>
-      </c>
+      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
@@ -4221,15 +4075,9 @@
       <c r="AB39" t="inlineStr"/>
       <c r="AC39" t="inlineStr"/>
       <c r="AD39" t="inlineStr"/>
-      <c r="AE39" t="n">
-        <v>61.9054054054054</v>
-      </c>
-      <c r="AF39" t="n">
-        <v>61.9054054054054</v>
-      </c>
-      <c r="AG39" t="n">
-        <v>61.9054054054054</v>
-      </c>
+      <c r="AE39" t="inlineStr"/>
+      <c r="AF39" t="inlineStr"/>
+      <c r="AG39" t="inlineStr"/>
       <c r="AH39" t="inlineStr">
         <is>
           <t>13/10/2025</t>
@@ -4373,9 +4221,7 @@
           <t>TRUNKEY FRANK</t>
         </is>
       </c>
-      <c r="E41" t="n">
-        <v>62.23404255319149</v>
-      </c>
+      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
@@ -4409,15 +4255,9 @@
       <c r="AB41" t="inlineStr"/>
       <c r="AC41" t="inlineStr"/>
       <c r="AD41" t="inlineStr"/>
-      <c r="AE41" t="n">
-        <v>62.23404255319149</v>
-      </c>
-      <c r="AF41" t="n">
-        <v>62.23404255319149</v>
-      </c>
-      <c r="AG41" t="n">
-        <v>62.23404255319149</v>
-      </c>
+      <c r="AE41" t="inlineStr"/>
+      <c r="AF41" t="inlineStr"/>
+      <c r="AG41" t="inlineStr"/>
       <c r="AH41" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -4561,9 +4401,7 @@
           <t>TRUNKEY REBEL</t>
         </is>
       </c>
-      <c r="E43" t="n">
-        <v>62.97709923664122</v>
-      </c>
+      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
@@ -4597,15 +4435,9 @@
       <c r="AB43" t="inlineStr"/>
       <c r="AC43" t="inlineStr"/>
       <c r="AD43" t="inlineStr"/>
-      <c r="AE43" t="n">
-        <v>62.97709923664122</v>
-      </c>
-      <c r="AF43" t="n">
-        <v>62.97709923664122</v>
-      </c>
-      <c r="AG43" t="n">
-        <v>62.97709923664122</v>
-      </c>
+      <c r="AE43" t="inlineStr"/>
+      <c r="AF43" t="inlineStr"/>
+      <c r="AG43" t="inlineStr"/>
       <c r="AH43" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -4749,9 +4581,7 @@
           <t>SPEEDY DEVILLE</t>
         </is>
       </c>
-      <c r="E45" t="n">
-        <v>62.23230490018149</v>
-      </c>
+      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
@@ -4785,15 +4615,9 @@
       <c r="AB45" t="inlineStr"/>
       <c r="AC45" t="inlineStr"/>
       <c r="AD45" t="inlineStr"/>
-      <c r="AE45" t="n">
-        <v>62.23230490018149</v>
-      </c>
-      <c r="AF45" t="n">
-        <v>62.23230490018149</v>
-      </c>
-      <c r="AG45" t="n">
-        <v>62.23230490018149</v>
-      </c>
+      <c r="AE45" t="inlineStr"/>
+      <c r="AF45" t="inlineStr"/>
+      <c r="AG45" t="inlineStr"/>
       <c r="AH45" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -4937,9 +4761,7 @@
           <t>PECORINO MONELLI</t>
         </is>
       </c>
-      <c r="E47" t="n">
-        <v>63.41637010676158</v>
-      </c>
+      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
@@ -4973,15 +4795,9 @@
       <c r="AB47" t="inlineStr"/>
       <c r="AC47" t="inlineStr"/>
       <c r="AD47" t="inlineStr"/>
-      <c r="AE47" t="n">
-        <v>63.41637010676158</v>
-      </c>
-      <c r="AF47" t="n">
-        <v>63.41637010676158</v>
-      </c>
-      <c r="AG47" t="n">
-        <v>63.41637010676158</v>
-      </c>
+      <c r="AE47" t="inlineStr"/>
+      <c r="AF47" t="inlineStr"/>
+      <c r="AG47" t="inlineStr"/>
       <c r="AH47" t="inlineStr">
         <is>
           <t>13/10/2025</t>
@@ -5125,9 +4941,7 @@
           <t>DON'T TURN</t>
         </is>
       </c>
-      <c r="E49" t="n">
-        <v>59.63190184049079</v>
-      </c>
+      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
@@ -5161,15 +4975,9 @@
       <c r="AB49" t="inlineStr"/>
       <c r="AC49" t="inlineStr"/>
       <c r="AD49" t="inlineStr"/>
-      <c r="AE49" t="n">
-        <v>59.63190184049079</v>
-      </c>
-      <c r="AF49" t="n">
-        <v>59.63190184049079</v>
-      </c>
-      <c r="AG49" t="n">
-        <v>59.63190184049079</v>
-      </c>
+      <c r="AE49" t="inlineStr"/>
+      <c r="AF49" t="inlineStr"/>
+      <c r="AG49" t="inlineStr"/>
       <c r="AH49" t="inlineStr">
         <is>
           <t>13/10/2025</t>
@@ -5313,9 +5121,7 @@
           <t>CHAMPAGNE CATHY</t>
         </is>
       </c>
-      <c r="E51" t="n">
-        <v>62.1195652173913</v>
-      </c>
+      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
@@ -5349,15 +5155,9 @@
       <c r="AB51" t="inlineStr"/>
       <c r="AC51" t="inlineStr"/>
       <c r="AD51" t="inlineStr"/>
-      <c r="AE51" t="n">
-        <v>62.1195652173913</v>
-      </c>
-      <c r="AF51" t="n">
-        <v>62.1195652173913</v>
-      </c>
-      <c r="AG51" t="n">
-        <v>62.1195652173913</v>
-      </c>
+      <c r="AE51" t="inlineStr"/>
+      <c r="AF51" t="inlineStr"/>
+      <c r="AG51" t="inlineStr"/>
       <c r="AH51" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -5501,9 +5301,7 @@
           <t>ON RED ALERT</t>
         </is>
       </c>
-      <c r="E53" t="n">
-        <v>62.048392442824</v>
-      </c>
+      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
@@ -5537,15 +5335,9 @@
       <c r="AB53" t="inlineStr"/>
       <c r="AC53" t="inlineStr"/>
       <c r="AD53" t="inlineStr"/>
-      <c r="AE53" t="n">
-        <v>62.048392442824</v>
-      </c>
-      <c r="AF53" t="n">
-        <v>62.048392442824</v>
-      </c>
-      <c r="AG53" t="n">
-        <v>62.048392442824</v>
-      </c>
+      <c r="AE53" t="inlineStr"/>
+      <c r="AF53" t="inlineStr"/>
+      <c r="AG53" t="inlineStr"/>
       <c r="AH53" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -5689,9 +5481,7 @@
           <t>HUNTER</t>
         </is>
       </c>
-      <c r="E55" t="n">
-        <v>61.63977609483042</v>
-      </c>
+      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
@@ -5725,15 +5515,9 @@
       <c r="AB55" t="inlineStr"/>
       <c r="AC55" t="inlineStr"/>
       <c r="AD55" t="inlineStr"/>
-      <c r="AE55" t="n">
-        <v>61.63977609483042</v>
-      </c>
-      <c r="AF55" t="n">
-        <v>61.63977609483042</v>
-      </c>
-      <c r="AG55" t="n">
-        <v>61.63977609483042</v>
-      </c>
+      <c r="AE55" t="inlineStr"/>
+      <c r="AF55" t="inlineStr"/>
+      <c r="AG55" t="inlineStr"/>
       <c r="AH55" t="inlineStr">
         <is>
           <t>29/10/2025</t>
@@ -5877,9 +5661,7 @@
           <t>CYNTHIA KEEPING</t>
         </is>
       </c>
-      <c r="E57" t="n">
-        <v>62.17203586848224</v>
-      </c>
+      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
@@ -5913,15 +5695,9 @@
       <c r="AB57" t="inlineStr"/>
       <c r="AC57" t="inlineStr"/>
       <c r="AD57" t="inlineStr"/>
-      <c r="AE57" t="n">
-        <v>62.17203586848224</v>
-      </c>
-      <c r="AF57" t="n">
-        <v>62.17203586848224</v>
-      </c>
-      <c r="AG57" t="n">
-        <v>62.17203586848224</v>
-      </c>
+      <c r="AE57" t="inlineStr"/>
+      <c r="AF57" t="inlineStr"/>
+      <c r="AG57" t="inlineStr"/>
       <c r="AH57" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -6065,9 +5841,7 @@
           <t>SEND IT COCO</t>
         </is>
       </c>
-      <c r="E59" t="n">
-        <v>61.75596578117965</v>
-      </c>
+      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
@@ -6101,15 +5875,9 @@
       <c r="AB59" t="inlineStr"/>
       <c r="AC59" t="inlineStr"/>
       <c r="AD59" t="inlineStr"/>
-      <c r="AE59" t="n">
-        <v>61.75596578117965</v>
-      </c>
-      <c r="AF59" t="n">
-        <v>61.75596578117965</v>
-      </c>
-      <c r="AG59" t="n">
-        <v>61.75596578117965</v>
-      </c>
+      <c r="AE59" t="inlineStr"/>
+      <c r="AF59" t="inlineStr"/>
+      <c r="AG59" t="inlineStr"/>
       <c r="AH59" t="inlineStr">
         <is>
           <t>8/10/2025</t>
@@ -6253,9 +6021,7 @@
           <t>JUST A BABE</t>
         </is>
       </c>
-      <c r="E61" t="n">
-        <v>62.23404255319149</v>
-      </c>
+      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr"/>
@@ -6289,15 +6055,9 @@
       <c r="AB61" t="inlineStr"/>
       <c r="AC61" t="inlineStr"/>
       <c r="AD61" t="inlineStr"/>
-      <c r="AE61" t="n">
-        <v>62.23404255319149</v>
-      </c>
-      <c r="AF61" t="n">
-        <v>62.23404255319149</v>
-      </c>
-      <c r="AG61" t="n">
-        <v>62.23404255319149</v>
-      </c>
+      <c r="AE61" t="inlineStr"/>
+      <c r="AF61" t="inlineStr"/>
+      <c r="AG61" t="inlineStr"/>
       <c r="AH61" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -6441,9 +6201,7 @@
           <t>FEARLESS PARKER</t>
         </is>
       </c>
-      <c r="E63" t="n">
-        <v>64.34316353887401</v>
-      </c>
+      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
@@ -6477,15 +6235,9 @@
       <c r="AB63" t="inlineStr"/>
       <c r="AC63" t="inlineStr"/>
       <c r="AD63" t="inlineStr"/>
-      <c r="AE63" t="n">
-        <v>64.34316353887401</v>
-      </c>
-      <c r="AF63" t="n">
-        <v>64.34316353887401</v>
-      </c>
-      <c r="AG63" t="n">
-        <v>64.34316353887401</v>
-      </c>
+      <c r="AE63" t="inlineStr"/>
+      <c r="AF63" t="inlineStr"/>
+      <c r="AG63" t="inlineStr"/>
       <c r="AH63" t="inlineStr">
         <is>
           <t>4/11/2025</t>
@@ -6629,9 +6381,7 @@
           <t>REINA</t>
         </is>
       </c>
-      <c r="E65" t="n">
-        <v>62.68738574040219</v>
-      </c>
+      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
@@ -6665,15 +6415,9 @@
       <c r="AB65" t="inlineStr"/>
       <c r="AC65" t="inlineStr"/>
       <c r="AD65" t="inlineStr"/>
-      <c r="AE65" t="n">
-        <v>62.68738574040219</v>
-      </c>
-      <c r="AF65" t="n">
-        <v>62.68738574040219</v>
-      </c>
-      <c r="AG65" t="n">
-        <v>62.68738574040219</v>
-      </c>
+      <c r="AE65" t="inlineStr"/>
+      <c r="AF65" t="inlineStr"/>
+      <c r="AG65" t="inlineStr"/>
       <c r="AH65" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -6817,9 +6561,7 @@
           <t>RAPIDO MYSTIQUE</t>
         </is>
       </c>
-      <c r="E67" t="n">
-        <v>60.92307692307693</v>
-      </c>
+      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr"/>
@@ -6853,15 +6595,9 @@
       <c r="AB67" t="inlineStr"/>
       <c r="AC67" t="inlineStr"/>
       <c r="AD67" t="inlineStr"/>
-      <c r="AE67" t="n">
-        <v>60.92307692307693</v>
-      </c>
-      <c r="AF67" t="n">
-        <v>60.92307692307693</v>
-      </c>
-      <c r="AG67" t="n">
-        <v>60.92307692307693</v>
-      </c>
+      <c r="AE67" t="inlineStr"/>
+      <c r="AF67" t="inlineStr"/>
+      <c r="AG67" t="inlineStr"/>
       <c r="AH67" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -7005,9 +6741,7 @@
           <t>BRUISER MY UNCLE</t>
         </is>
       </c>
-      <c r="E69" t="n">
-        <v>62.90956749672346</v>
-      </c>
+      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr"/>
@@ -7041,15 +6775,9 @@
       <c r="AB69" t="inlineStr"/>
       <c r="AC69" t="inlineStr"/>
       <c r="AD69" t="inlineStr"/>
-      <c r="AE69" t="n">
-        <v>62.90956749672346</v>
-      </c>
-      <c r="AF69" t="n">
-        <v>62.90956749672346</v>
-      </c>
-      <c r="AG69" t="n">
-        <v>62.90956749672346</v>
-      </c>
+      <c r="AE69" t="inlineStr"/>
+      <c r="AF69" t="inlineStr"/>
+      <c r="AG69" t="inlineStr"/>
       <c r="AH69" t="inlineStr">
         <is>
           <t>3/11/2025</t>
@@ -7193,9 +6921,7 @@
           <t>WOODBURN GRACE</t>
         </is>
       </c>
-      <c r="E71" t="n">
-        <v>60.92307692307693</v>
-      </c>
+      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
@@ -7229,15 +6955,9 @@
       <c r="AB71" t="inlineStr"/>
       <c r="AC71" t="inlineStr"/>
       <c r="AD71" t="inlineStr"/>
-      <c r="AE71" t="n">
-        <v>60.92307692307693</v>
-      </c>
-      <c r="AF71" t="n">
-        <v>60.92307692307693</v>
-      </c>
-      <c r="AG71" t="n">
-        <v>60.92307692307693</v>
-      </c>
+      <c r="AE71" t="inlineStr"/>
+      <c r="AF71" t="inlineStr"/>
+      <c r="AG71" t="inlineStr"/>
       <c r="AH71" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -7313,9 +7033,7 @@
           <t>SUMMER SWELL</t>
         </is>
       </c>
-      <c r="E72" t="n">
-        <v>62.1195652173913</v>
-      </c>
+      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
@@ -7349,15 +7067,9 @@
       <c r="AB72" t="inlineStr"/>
       <c r="AC72" t="inlineStr"/>
       <c r="AD72" t="inlineStr"/>
-      <c r="AE72" t="n">
-        <v>62.1195652173913</v>
-      </c>
-      <c r="AF72" t="n">
-        <v>62.1195652173913</v>
-      </c>
-      <c r="AG72" t="n">
-        <v>62.1195652173913</v>
-      </c>
+      <c r="AE72" t="inlineStr"/>
+      <c r="AF72" t="inlineStr"/>
+      <c r="AG72" t="inlineStr"/>
       <c r="AH72" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -7433,9 +7145,7 @@
           <t>ARIEL'S DRIVE</t>
         </is>
       </c>
-      <c r="E73" t="n">
-        <v>62.048392442824</v>
-      </c>
+      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr"/>
@@ -7469,15 +7179,9 @@
       <c r="AB73" t="inlineStr"/>
       <c r="AC73" t="inlineStr"/>
       <c r="AD73" t="inlineStr"/>
-      <c r="AE73" t="n">
-        <v>62.048392442824</v>
-      </c>
-      <c r="AF73" t="n">
-        <v>62.048392442824</v>
-      </c>
-      <c r="AG73" t="n">
-        <v>62.048392442824</v>
-      </c>
+      <c r="AE73" t="inlineStr"/>
+      <c r="AF73" t="inlineStr"/>
+      <c r="AG73" t="inlineStr"/>
       <c r="AH73" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -7553,9 +7257,7 @@
           <t>IMPRESS NEMO</t>
         </is>
       </c>
-      <c r="E74" t="n">
-        <v>62.048392442824</v>
-      </c>
+      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr"/>
@@ -7589,15 +7291,9 @@
       <c r="AB74" t="inlineStr"/>
       <c r="AC74" t="inlineStr"/>
       <c r="AD74" t="inlineStr"/>
-      <c r="AE74" t="n">
-        <v>62.048392442824</v>
-      </c>
-      <c r="AF74" t="n">
-        <v>62.048392442824</v>
-      </c>
-      <c r="AG74" t="n">
-        <v>62.048392442824</v>
-      </c>
+      <c r="AE74" t="inlineStr"/>
+      <c r="AF74" t="inlineStr"/>
+      <c r="AG74" t="inlineStr"/>
       <c r="AH74" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -7741,9 +7437,7 @@
           <t>SPEED CHELLER</t>
         </is>
       </c>
-      <c r="E76" t="n">
-        <v>62.17203586848224</v>
-      </c>
+      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr"/>
@@ -7777,15 +7471,9 @@
       <c r="AB76" t="inlineStr"/>
       <c r="AC76" t="inlineStr"/>
       <c r="AD76" t="inlineStr"/>
-      <c r="AE76" t="n">
-        <v>62.17203586848224</v>
-      </c>
-      <c r="AF76" t="n">
-        <v>62.17203586848224</v>
-      </c>
-      <c r="AG76" t="n">
-        <v>62.17203586848224</v>
-      </c>
+      <c r="AE76" t="inlineStr"/>
+      <c r="AF76" t="inlineStr"/>
+      <c r="AG76" t="inlineStr"/>
       <c r="AH76" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -7929,9 +7617,7 @@
           <t>RIPPIN' BLUE</t>
         </is>
       </c>
-      <c r="E78" t="n">
-        <v>62.74473924977127</v>
-      </c>
+      <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr"/>
@@ -7965,15 +7651,9 @@
       <c r="AB78" t="inlineStr"/>
       <c r="AC78" t="inlineStr"/>
       <c r="AD78" t="inlineStr"/>
-      <c r="AE78" t="n">
-        <v>62.74473924977127</v>
-      </c>
-      <c r="AF78" t="n">
-        <v>62.74473924977127</v>
-      </c>
-      <c r="AG78" t="n">
-        <v>62.74473924977127</v>
-      </c>
+      <c r="AE78" t="inlineStr"/>
+      <c r="AF78" t="inlineStr"/>
+      <c r="AG78" t="inlineStr"/>
       <c r="AH78" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -8117,9 +7797,7 @@
           <t>FERNDALE FLYER</t>
         </is>
       </c>
-      <c r="E80" t="n">
-        <v>62.882096069869</v>
-      </c>
+      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr"/>
@@ -8153,15 +7831,9 @@
       <c r="AB80" t="inlineStr"/>
       <c r="AC80" t="inlineStr"/>
       <c r="AD80" t="inlineStr"/>
-      <c r="AE80" t="n">
-        <v>62.882096069869</v>
-      </c>
-      <c r="AF80" t="n">
-        <v>62.882096069869</v>
-      </c>
-      <c r="AG80" t="n">
-        <v>62.882096069869</v>
-      </c>
+      <c r="AE80" t="inlineStr"/>
+      <c r="AF80" t="inlineStr"/>
+      <c r="AG80" t="inlineStr"/>
       <c r="AH80" t="inlineStr">
         <is>
           <t>1/11/2025</t>
@@ -8305,9 +7977,7 @@
           <t>MR</t>
         </is>
       </c>
-      <c r="E82" t="n">
-        <v>62.9004076878276</v>
-      </c>
+      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr"/>
@@ -8341,15 +8011,9 @@
       <c r="AB82" t="inlineStr"/>
       <c r="AC82" t="inlineStr"/>
       <c r="AD82" t="inlineStr"/>
-      <c r="AE82" t="n">
-        <v>62.9004076878276</v>
-      </c>
-      <c r="AF82" t="n">
-        <v>62.9004076878276</v>
-      </c>
-      <c r="AG82" t="n">
-        <v>62.9004076878276</v>
-      </c>
+      <c r="AE82" t="inlineStr"/>
+      <c r="AF82" t="inlineStr"/>
+      <c r="AG82" t="inlineStr"/>
       <c r="AH82" t="inlineStr">
         <is>
           <t>30/10/2025</t>
@@ -8493,9 +8157,7 @@
           <t>JUDGE JEBRYNAH</t>
         </is>
       </c>
-      <c r="E84" t="n">
-        <v>60.69895769466586</v>
-      </c>
+      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr"/>
@@ -8529,15 +8191,9 @@
       <c r="AB84" t="inlineStr"/>
       <c r="AC84" t="inlineStr"/>
       <c r="AD84" t="inlineStr"/>
-      <c r="AE84" t="n">
-        <v>60.69895769466586</v>
-      </c>
-      <c r="AF84" t="n">
-        <v>60.69895769466586</v>
-      </c>
-      <c r="AG84" t="n">
-        <v>60.69895769466586</v>
-      </c>
+      <c r="AE84" t="inlineStr"/>
+      <c r="AF84" t="inlineStr"/>
+      <c r="AG84" t="inlineStr"/>
       <c r="AH84" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -8681,9 +8337,7 @@
           <t>INFRARED GEM</t>
         </is>
       </c>
-      <c r="E86" t="n">
-        <v>60.69895769466586</v>
-      </c>
+      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr"/>
@@ -8717,15 +8371,9 @@
       <c r="AB86" t="inlineStr"/>
       <c r="AC86" t="inlineStr"/>
       <c r="AD86" t="inlineStr"/>
-      <c r="AE86" t="n">
-        <v>60.69895769466586</v>
-      </c>
-      <c r="AF86" t="n">
-        <v>60.69895769466586</v>
-      </c>
-      <c r="AG86" t="n">
-        <v>60.69895769466586</v>
-      </c>
+      <c r="AE86" t="inlineStr"/>
+      <c r="AF86" t="inlineStr"/>
+      <c r="AG86" t="inlineStr"/>
       <c r="AH86" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -8869,9 +8517,7 @@
           <t>DAIKOKU FLYER</t>
         </is>
       </c>
-      <c r="E88" t="n">
-        <v>61.51898734177216</v>
-      </c>
+      <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr"/>
@@ -8905,15 +8551,9 @@
       <c r="AB88" t="inlineStr"/>
       <c r="AC88" t="inlineStr"/>
       <c r="AD88" t="inlineStr"/>
-      <c r="AE88" t="n">
-        <v>61.51898734177216</v>
-      </c>
-      <c r="AF88" t="n">
-        <v>61.51898734177216</v>
-      </c>
-      <c r="AG88" t="n">
-        <v>61.51898734177216</v>
-      </c>
+      <c r="AE88" t="inlineStr"/>
+      <c r="AF88" t="inlineStr"/>
+      <c r="AG88" t="inlineStr"/>
       <c r="AH88" t="inlineStr">
         <is>
           <t>15/09/2025</t>
@@ -9057,9 +8697,7 @@
           <t>CAKE IN TUMMY</t>
         </is>
       </c>
-      <c r="E90" t="n">
-        <v>62.97709923664122</v>
-      </c>
+      <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr"/>
@@ -9093,15 +8731,9 @@
       <c r="AB90" t="inlineStr"/>
       <c r="AC90" t="inlineStr"/>
       <c r="AD90" t="inlineStr"/>
-      <c r="AE90" t="n">
-        <v>62.97709923664122</v>
-      </c>
-      <c r="AF90" t="n">
-        <v>62.97709923664122</v>
-      </c>
-      <c r="AG90" t="n">
-        <v>62.97709923664122</v>
-      </c>
+      <c r="AE90" t="inlineStr"/>
+      <c r="AF90" t="inlineStr"/>
+      <c r="AG90" t="inlineStr"/>
       <c r="AH90" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -9245,9 +8877,7 @@
           <t>POPPY TAHLEIA</t>
         </is>
       </c>
-      <c r="E92" t="n">
-        <v>63.94316163410302</v>
-      </c>
+      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr"/>
@@ -9281,15 +8911,9 @@
       <c r="AB92" t="inlineStr"/>
       <c r="AC92" t="inlineStr"/>
       <c r="AD92" t="inlineStr"/>
-      <c r="AE92" t="n">
-        <v>63.94316163410302</v>
-      </c>
-      <c r="AF92" t="n">
-        <v>63.94316163410302</v>
-      </c>
-      <c r="AG92" t="n">
-        <v>63.94316163410302</v>
-      </c>
+      <c r="AE92" t="inlineStr"/>
+      <c r="AF92" t="inlineStr"/>
+      <c r="AG92" t="inlineStr"/>
       <c r="AH92" t="inlineStr">
         <is>
           <t>28/10/2025</t>
@@ -9433,9 +9057,7 @@
           <t>KING POTATO</t>
         </is>
       </c>
-      <c r="E94" t="n">
-        <v>63.43612334801763</v>
-      </c>
+      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr"/>
@@ -9469,15 +9091,9 @@
       <c r="AB94" t="inlineStr"/>
       <c r="AC94" t="inlineStr"/>
       <c r="AD94" t="inlineStr"/>
-      <c r="AE94" t="n">
-        <v>63.43612334801763</v>
-      </c>
-      <c r="AF94" t="n">
-        <v>63.43612334801763</v>
-      </c>
-      <c r="AG94" t="n">
-        <v>63.43612334801763</v>
-      </c>
+      <c r="AE94" t="inlineStr"/>
+      <c r="AF94" t="inlineStr"/>
+      <c r="AG94" t="inlineStr"/>
       <c r="AH94" t="inlineStr">
         <is>
           <t>4/11/2025</t>
@@ -9621,9 +9237,7 @@
           <t>CROCODILE CRAWL</t>
         </is>
       </c>
-      <c r="E96" t="n">
-        <v>61.94573130377233</v>
-      </c>
+      <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr"/>
@@ -9657,15 +9271,9 @@
       <c r="AB96" t="inlineStr"/>
       <c r="AC96" t="inlineStr"/>
       <c r="AD96" t="inlineStr"/>
-      <c r="AE96" t="n">
-        <v>61.94573130377233</v>
-      </c>
-      <c r="AF96" t="n">
-        <v>61.94573130377233</v>
-      </c>
-      <c r="AG96" t="n">
-        <v>61.94573130377233</v>
-      </c>
+      <c r="AE96" t="inlineStr"/>
+      <c r="AF96" t="inlineStr"/>
+      <c r="AG96" t="inlineStr"/>
       <c r="AH96" t="inlineStr">
         <is>
           <t>8/11/2025</t>
@@ -9809,9 +9417,7 @@
           <t>JUST A PRINCESS</t>
         </is>
       </c>
-      <c r="E98" t="n">
-        <v>63.10344827586208</v>
-      </c>
+      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr"/>
@@ -9845,15 +9451,9 @@
       <c r="AB98" t="inlineStr"/>
       <c r="AC98" t="inlineStr"/>
       <c r="AD98" t="inlineStr"/>
-      <c r="AE98" t="n">
-        <v>63.10344827586208</v>
-      </c>
-      <c r="AF98" t="n">
-        <v>63.10344827586208</v>
-      </c>
-      <c r="AG98" t="n">
-        <v>63.10344827586208</v>
-      </c>
+      <c r="AE98" t="inlineStr"/>
+      <c r="AF98" t="inlineStr"/>
+      <c r="AG98" t="inlineStr"/>
       <c r="AH98" t="inlineStr">
         <is>
           <t>4/11/2025</t>
@@ -9997,9 +9597,7 @@
           <t>FOOT FALCON</t>
         </is>
       </c>
-      <c r="E100" t="n">
-        <v>62.17203586848224</v>
-      </c>
+      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr"/>
@@ -10033,15 +9631,9 @@
       <c r="AB100" t="inlineStr"/>
       <c r="AC100" t="inlineStr"/>
       <c r="AD100" t="inlineStr"/>
-      <c r="AE100" t="n">
-        <v>62.17203586848224</v>
-      </c>
-      <c r="AF100" t="n">
-        <v>62.17203586848224</v>
-      </c>
-      <c r="AG100" t="n">
-        <v>62.17203586848224</v>
-      </c>
+      <c r="AE100" t="inlineStr"/>
+      <c r="AF100" t="inlineStr"/>
+      <c r="AG100" t="inlineStr"/>
       <c r="AH100" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -10185,9 +9777,7 @@
           <t>MY MOET</t>
         </is>
       </c>
-      <c r="E102" t="n">
-        <v>63.74455732946299</v>
-      </c>
+      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr"/>
@@ -10221,15 +9811,9 @@
       <c r="AB102" t="inlineStr"/>
       <c r="AC102" t="inlineStr"/>
       <c r="AD102" t="inlineStr"/>
-      <c r="AE102" t="n">
-        <v>63.74455732946299</v>
-      </c>
-      <c r="AF102" t="n">
-        <v>63.74455732946299</v>
-      </c>
-      <c r="AG102" t="n">
-        <v>63.74455732946299</v>
-      </c>
+      <c r="AE102" t="inlineStr"/>
+      <c r="AF102" t="inlineStr"/>
+      <c r="AG102" t="inlineStr"/>
       <c r="AH102" t="inlineStr">
         <is>
           <t>31/10/2025</t>
@@ -10373,9 +9957,7 @@
           <t>ASTON FLORIN</t>
         </is>
       </c>
-      <c r="E104" t="n">
-        <v>64.02845709204091</v>
-      </c>
+      <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr"/>
@@ -10409,15 +9991,9 @@
       <c r="AB104" t="inlineStr"/>
       <c r="AC104" t="inlineStr"/>
       <c r="AD104" t="inlineStr"/>
-      <c r="AE104" t="n">
-        <v>64.02845709204091</v>
-      </c>
-      <c r="AF104" t="n">
-        <v>64.02845709204091</v>
-      </c>
-      <c r="AG104" t="n">
-        <v>64.02845709204091</v>
-      </c>
+      <c r="AE104" t="inlineStr"/>
+      <c r="AF104" t="inlineStr"/>
+      <c r="AG104" t="inlineStr"/>
       <c r="AH104" t="inlineStr">
         <is>
           <t>31/10/2025</t>
@@ -10561,9 +10137,7 @@
           <t>PRIDE AND POWER</t>
         </is>
       </c>
-      <c r="E106" t="n">
-        <v>63.82978723404256</v>
-      </c>
+      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr"/>
@@ -10597,15 +10171,9 @@
       <c r="AB106" t="inlineStr"/>
       <c r="AC106" t="inlineStr"/>
       <c r="AD106" t="inlineStr"/>
-      <c r="AE106" t="n">
-        <v>63.82978723404256</v>
-      </c>
-      <c r="AF106" t="n">
-        <v>63.82978723404256</v>
-      </c>
-      <c r="AG106" t="n">
-        <v>63.82978723404256</v>
-      </c>
+      <c r="AE106" t="inlineStr"/>
+      <c r="AF106" t="inlineStr"/>
+      <c r="AG106" t="inlineStr"/>
       <c r="AH106" t="inlineStr">
         <is>
           <t>30/10/2025</t>
@@ -10749,9 +10317,7 @@
           <t>OUTSIDE THE FIRE</t>
         </is>
       </c>
-      <c r="E108" t="n">
-        <v>61.59327731092437</v>
-      </c>
+      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr"/>
@@ -10785,15 +10351,9 @@
       <c r="AB108" t="inlineStr"/>
       <c r="AC108" t="inlineStr"/>
       <c r="AD108" t="inlineStr"/>
-      <c r="AE108" t="n">
-        <v>61.59327731092437</v>
-      </c>
-      <c r="AF108" t="n">
-        <v>61.59327731092437</v>
-      </c>
-      <c r="AG108" t="n">
-        <v>61.59327731092437</v>
-      </c>
+      <c r="AE108" t="inlineStr"/>
+      <c r="AF108" t="inlineStr"/>
+      <c r="AG108" t="inlineStr"/>
       <c r="AH108" t="inlineStr">
         <is>
           <t>6/10/2025</t>
@@ -10937,9 +10497,7 @@
           <t>PAID IN FULL</t>
         </is>
       </c>
-      <c r="E110" t="n">
-        <v>62.23230490018149</v>
-      </c>
+      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr"/>
@@ -10973,15 +10531,9 @@
       <c r="AB110" t="inlineStr"/>
       <c r="AC110" t="inlineStr"/>
       <c r="AD110" t="inlineStr"/>
-      <c r="AE110" t="n">
-        <v>62.23230490018149</v>
-      </c>
-      <c r="AF110" t="n">
-        <v>62.23230490018149</v>
-      </c>
-      <c r="AG110" t="n">
-        <v>62.23230490018149</v>
-      </c>
+      <c r="AE110" t="inlineStr"/>
+      <c r="AF110" t="inlineStr"/>
+      <c r="AG110" t="inlineStr"/>
       <c r="AH110" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -11125,9 +10677,7 @@
           <t>INVESTED</t>
         </is>
       </c>
-      <c r="E112" t="n">
-        <v>63.75442739079102</v>
-      </c>
+      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr"/>
@@ -11161,15 +10711,9 @@
       <c r="AB112" t="inlineStr"/>
       <c r="AC112" t="inlineStr"/>
       <c r="AD112" t="inlineStr"/>
-      <c r="AE112" t="n">
-        <v>63.75442739079102</v>
-      </c>
-      <c r="AF112" t="n">
-        <v>63.75442739079102</v>
-      </c>
-      <c r="AG112" t="n">
-        <v>63.75442739079102</v>
-      </c>
+      <c r="AE112" t="inlineStr"/>
+      <c r="AF112" t="inlineStr"/>
+      <c r="AG112" t="inlineStr"/>
       <c r="AH112" t="inlineStr">
         <is>
           <t>6/11/2025</t>
@@ -11313,9 +10857,7 @@
           <t>GOLDEN HANDCUFFS</t>
         </is>
       </c>
-      <c r="E114" t="n">
-        <v>62.60869565217391</v>
-      </c>
+      <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr"/>
@@ -11349,15 +10891,9 @@
       <c r="AB114" t="inlineStr"/>
       <c r="AC114" t="inlineStr"/>
       <c r="AD114" t="inlineStr"/>
-      <c r="AE114" t="n">
-        <v>62.60869565217391</v>
-      </c>
-      <c r="AF114" t="n">
-        <v>62.60869565217391</v>
-      </c>
-      <c r="AG114" t="n">
-        <v>62.60869565217391</v>
-      </c>
+      <c r="AE114" t="inlineStr"/>
+      <c r="AF114" t="inlineStr"/>
+      <c r="AG114" t="inlineStr"/>
       <c r="AH114" t="inlineStr">
         <is>
           <t>31/10/2025</t>
@@ -11581,9 +11117,7 @@
           <t>ELECTRA STARR</t>
         </is>
       </c>
-      <c r="E117" t="n">
-        <v>62.048392442824</v>
-      </c>
+      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
@@ -11617,15 +11151,9 @@
       <c r="AB117" t="inlineStr"/>
       <c r="AC117" t="inlineStr"/>
       <c r="AD117" t="inlineStr"/>
-      <c r="AE117" t="n">
-        <v>62.048392442824</v>
-      </c>
-      <c r="AF117" t="n">
-        <v>62.048392442824</v>
-      </c>
-      <c r="AG117" t="n">
-        <v>62.048392442824</v>
-      </c>
+      <c r="AE117" t="inlineStr"/>
+      <c r="AF117" t="inlineStr"/>
+      <c r="AG117" t="inlineStr"/>
       <c r="AH117" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -11701,9 +11229,7 @@
           <t>RED HOT BONNIE</t>
         </is>
       </c>
-      <c r="E118" t="n">
-        <v>62.048392442824</v>
-      </c>
+      <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="inlineStr"/>
@@ -11737,15 +11263,9 @@
       <c r="AB118" t="inlineStr"/>
       <c r="AC118" t="inlineStr"/>
       <c r="AD118" t="inlineStr"/>
-      <c r="AE118" t="n">
-        <v>62.048392442824</v>
-      </c>
-      <c r="AF118" t="n">
-        <v>62.048392442824</v>
-      </c>
-      <c r="AG118" t="n">
-        <v>62.048392442824</v>
-      </c>
+      <c r="AE118" t="inlineStr"/>
+      <c r="AF118" t="inlineStr"/>
+      <c r="AG118" t="inlineStr"/>
       <c r="AH118" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -11889,9 +11409,7 @@
           <t>ZERO SURF</t>
         </is>
       </c>
-      <c r="E120" t="n">
-        <v>62.17203586848224</v>
-      </c>
+      <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="inlineStr"/>
@@ -11925,15 +11443,9 @@
       <c r="AB120" t="inlineStr"/>
       <c r="AC120" t="inlineStr"/>
       <c r="AD120" t="inlineStr"/>
-      <c r="AE120" t="n">
-        <v>62.17203586848224</v>
-      </c>
-      <c r="AF120" t="n">
-        <v>62.17203586848224</v>
-      </c>
-      <c r="AG120" t="n">
-        <v>62.17203586848224</v>
-      </c>
+      <c r="AE120" t="inlineStr"/>
+      <c r="AF120" t="inlineStr"/>
+      <c r="AG120" t="inlineStr"/>
       <c r="AH120" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -12077,9 +11589,7 @@
           <t>ELITE ARNOTT</t>
         </is>
       </c>
-      <c r="E122" t="n">
-        <v>61.83949504057711</v>
-      </c>
+      <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr"/>
@@ -12113,15 +11623,9 @@
       <c r="AB122" t="inlineStr"/>
       <c r="AC122" t="inlineStr"/>
       <c r="AD122" t="inlineStr"/>
-      <c r="AE122" t="n">
-        <v>61.83949504057711</v>
-      </c>
-      <c r="AF122" t="n">
-        <v>61.83949504057711</v>
-      </c>
-      <c r="AG122" t="n">
-        <v>61.83949504057711</v>
-      </c>
+      <c r="AE122" t="inlineStr"/>
+      <c r="AF122" t="inlineStr"/>
+      <c r="AG122" t="inlineStr"/>
       <c r="AH122" t="inlineStr">
         <is>
           <t>22/10/2025</t>
@@ -12265,9 +11769,7 @@
           <t>WEST ON BURNIE</t>
         </is>
       </c>
-      <c r="E124" t="n">
-        <v>62.23404255319149</v>
-      </c>
+      <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr"/>
@@ -12301,15 +11803,9 @@
       <c r="AB124" t="inlineStr"/>
       <c r="AC124" t="inlineStr"/>
       <c r="AD124" t="inlineStr"/>
-      <c r="AE124" t="n">
-        <v>62.23404255319149</v>
-      </c>
-      <c r="AF124" t="n">
-        <v>62.23404255319149</v>
-      </c>
-      <c r="AG124" t="n">
-        <v>62.23404255319149</v>
-      </c>
+      <c r="AE124" t="inlineStr"/>
+      <c r="AF124" t="inlineStr"/>
+      <c r="AG124" t="inlineStr"/>
       <c r="AH124" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -12453,9 +11949,7 @@
           <t>HELLO BAILEY</t>
         </is>
       </c>
-      <c r="E126" t="n">
-        <v>62.97709923664122</v>
-      </c>
+      <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr"/>
@@ -12489,15 +11983,9 @@
       <c r="AB126" t="inlineStr"/>
       <c r="AC126" t="inlineStr"/>
       <c r="AD126" t="inlineStr"/>
-      <c r="AE126" t="n">
-        <v>62.97709923664122</v>
-      </c>
-      <c r="AF126" t="n">
-        <v>62.97709923664122</v>
-      </c>
-      <c r="AG126" t="n">
-        <v>62.97709923664122</v>
-      </c>
+      <c r="AE126" t="inlineStr"/>
+      <c r="AF126" t="inlineStr"/>
+      <c r="AG126" t="inlineStr"/>
       <c r="AH126" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -12641,9 +12129,7 @@
           <t>PURE LOVE</t>
         </is>
       </c>
-      <c r="E128" t="n">
-        <v>62.8021978021978</v>
-      </c>
+      <c r="E128" t="inlineStr"/>
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr"/>
@@ -12677,15 +12163,9 @@
       <c r="AB128" t="inlineStr"/>
       <c r="AC128" t="inlineStr"/>
       <c r="AD128" t="inlineStr"/>
-      <c r="AE128" t="n">
-        <v>62.8021978021978</v>
-      </c>
-      <c r="AF128" t="n">
-        <v>62.8021978021978</v>
-      </c>
-      <c r="AG128" t="n">
-        <v>62.8021978021978</v>
-      </c>
+      <c r="AE128" t="inlineStr"/>
+      <c r="AF128" t="inlineStr"/>
+      <c r="AG128" t="inlineStr"/>
       <c r="AH128" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -12829,9 +12309,7 @@
           <t>FOUND THE BRAKE</t>
         </is>
       </c>
-      <c r="E130" t="n">
-        <v>61.56716417910449</v>
-      </c>
+      <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr"/>
@@ -12865,15 +12343,9 @@
       <c r="AB130" t="inlineStr"/>
       <c r="AC130" t="inlineStr"/>
       <c r="AD130" t="inlineStr"/>
-      <c r="AE130" t="n">
-        <v>61.56716417910449</v>
-      </c>
-      <c r="AF130" t="n">
-        <v>61.56716417910449</v>
-      </c>
-      <c r="AG130" t="n">
-        <v>61.56716417910449</v>
-      </c>
+      <c r="AE130" t="inlineStr"/>
+      <c r="AF130" t="inlineStr"/>
+      <c r="AG130" t="inlineStr"/>
       <c r="AH130" t="inlineStr">
         <is>
           <t>8/10/2025</t>
@@ -13017,9 +12489,7 @@
           <t>ARMED FOR ACTION</t>
         </is>
       </c>
-      <c r="E132" t="n">
-        <v>62.8021978021978</v>
-      </c>
+      <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr"/>
@@ -13053,15 +12523,9 @@
       <c r="AB132" t="inlineStr"/>
       <c r="AC132" t="inlineStr"/>
       <c r="AD132" t="inlineStr"/>
-      <c r="AE132" t="n">
-        <v>62.8021978021978</v>
-      </c>
-      <c r="AF132" t="n">
-        <v>62.8021978021978</v>
-      </c>
-      <c r="AG132" t="n">
-        <v>62.8021978021978</v>
-      </c>
+      <c r="AE132" t="inlineStr"/>
+      <c r="AF132" t="inlineStr"/>
+      <c r="AG132" t="inlineStr"/>
       <c r="AH132" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -13205,9 +12669,7 @@
           <t>TINY TWIST</t>
         </is>
       </c>
-      <c r="E134" t="n">
-        <v>61.52889993784959</v>
-      </c>
+      <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr"/>
@@ -13241,15 +12703,9 @@
       <c r="AB134" t="inlineStr"/>
       <c r="AC134" t="inlineStr"/>
       <c r="AD134" t="inlineStr"/>
-      <c r="AE134" t="n">
-        <v>61.52889993784959</v>
-      </c>
-      <c r="AF134" t="n">
-        <v>61.52889993784959</v>
-      </c>
-      <c r="AG134" t="n">
-        <v>61.52889993784959</v>
-      </c>
+      <c r="AE134" t="inlineStr"/>
+      <c r="AF134" t="inlineStr"/>
+      <c r="AG134" t="inlineStr"/>
       <c r="AH134" t="inlineStr">
         <is>
           <t>29/10/2025</t>
@@ -13393,9 +12849,7 @@
           <t>JUNGLE DELUXE</t>
         </is>
       </c>
-      <c r="E136" t="n">
-        <v>61.84340931615461</v>
-      </c>
+      <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="inlineStr"/>
@@ -13429,15 +12883,9 @@
       <c r="AB136" t="inlineStr"/>
       <c r="AC136" t="inlineStr"/>
       <c r="AD136" t="inlineStr"/>
-      <c r="AE136" t="n">
-        <v>61.84340931615461</v>
-      </c>
-      <c r="AF136" t="n">
-        <v>61.84340931615461</v>
-      </c>
-      <c r="AG136" t="n">
-        <v>61.84340931615461</v>
-      </c>
+      <c r="AE136" t="inlineStr"/>
+      <c r="AF136" t="inlineStr"/>
+      <c r="AG136" t="inlineStr"/>
       <c r="AH136" t="inlineStr">
         <is>
           <t>10/09/2025</t>
@@ -13877,9 +13325,7 @@
           <t>FROTHING</t>
         </is>
       </c>
-      <c r="E142" t="n">
-        <v>62.048392442824</v>
-      </c>
+      <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr"/>
@@ -13913,15 +13359,9 @@
       <c r="AB142" t="inlineStr"/>
       <c r="AC142" t="inlineStr"/>
       <c r="AD142" t="inlineStr"/>
-      <c r="AE142" t="n">
-        <v>62.048392442824</v>
-      </c>
-      <c r="AF142" t="n">
-        <v>62.048392442824</v>
-      </c>
-      <c r="AG142" t="n">
-        <v>62.048392442824</v>
-      </c>
+      <c r="AE142" t="inlineStr"/>
+      <c r="AF142" t="inlineStr"/>
+      <c r="AG142" t="inlineStr"/>
       <c r="AH142" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -14065,9 +13505,7 @@
           <t>RIPPIN' PIKE</t>
         </is>
       </c>
-      <c r="E144" t="n">
-        <v>62.74473924977127</v>
-      </c>
+      <c r="E144" t="inlineStr"/>
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr"/>
@@ -14101,15 +13539,9 @@
       <c r="AB144" t="inlineStr"/>
       <c r="AC144" t="inlineStr"/>
       <c r="AD144" t="inlineStr"/>
-      <c r="AE144" t="n">
-        <v>62.74473924977127</v>
-      </c>
-      <c r="AF144" t="n">
-        <v>62.74473924977127</v>
-      </c>
-      <c r="AG144" t="n">
-        <v>62.74473924977127</v>
-      </c>
+      <c r="AE144" t="inlineStr"/>
+      <c r="AF144" t="inlineStr"/>
+      <c r="AG144" t="inlineStr"/>
       <c r="AH144" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -14253,9 +13685,7 @@
           <t>RAPIDO WARRIOR</t>
         </is>
       </c>
-      <c r="E146" t="n">
-        <v>62.23404255319149</v>
-      </c>
+      <c r="E146" t="inlineStr"/>
       <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="inlineStr"/>
@@ -14289,15 +13719,9 @@
       <c r="AB146" t="inlineStr"/>
       <c r="AC146" t="inlineStr"/>
       <c r="AD146" t="inlineStr"/>
-      <c r="AE146" t="n">
-        <v>62.23404255319149</v>
-      </c>
-      <c r="AF146" t="n">
-        <v>62.23404255319149</v>
-      </c>
-      <c r="AG146" t="n">
-        <v>62.23404255319149</v>
-      </c>
+      <c r="AE146" t="inlineStr"/>
+      <c r="AF146" t="inlineStr"/>
+      <c r="AG146" t="inlineStr"/>
       <c r="AH146" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -14441,9 +13865,7 @@
           <t>REGGAE MELODY</t>
         </is>
       </c>
-      <c r="E148" t="n">
-        <v>63.06206896551724</v>
-      </c>
+      <c r="E148" t="inlineStr"/>
       <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr"/>
@@ -14477,15 +13899,9 @@
       <c r="AB148" t="inlineStr"/>
       <c r="AC148" t="inlineStr"/>
       <c r="AD148" t="inlineStr"/>
-      <c r="AE148" t="n">
-        <v>63.06206896551724</v>
-      </c>
-      <c r="AF148" t="n">
-        <v>63.06206896551724</v>
-      </c>
-      <c r="AG148" t="n">
-        <v>63.06206896551724</v>
-      </c>
+      <c r="AE148" t="inlineStr"/>
+      <c r="AF148" t="inlineStr"/>
+      <c r="AG148" t="inlineStr"/>
       <c r="AH148" t="inlineStr">
         <is>
           <t>29/10/2025</t>
@@ -14629,9 +14045,7 @@
           <t>JANA BLADE</t>
         </is>
       </c>
-      <c r="E150" t="n">
-        <v>62.23230490018149</v>
-      </c>
+      <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr"/>
@@ -14665,15 +14079,9 @@
       <c r="AB150" t="inlineStr"/>
       <c r="AC150" t="inlineStr"/>
       <c r="AD150" t="inlineStr"/>
-      <c r="AE150" t="n">
-        <v>62.23230490018149</v>
-      </c>
-      <c r="AF150" t="n">
-        <v>62.23230490018149</v>
-      </c>
-      <c r="AG150" t="n">
-        <v>62.23230490018149</v>
-      </c>
+      <c r="AE150" t="inlineStr"/>
+      <c r="AF150" t="inlineStr"/>
+      <c r="AG150" t="inlineStr"/>
       <c r="AH150" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -14817,9 +14225,7 @@
           <t>CHEDDAR MONELLI</t>
         </is>
       </c>
-      <c r="E152" t="n">
-        <v>60.88560885608856</v>
-      </c>
+      <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr"/>
       <c r="H152" t="inlineStr"/>
@@ -14853,15 +14259,9 @@
       <c r="AB152" t="inlineStr"/>
       <c r="AC152" t="inlineStr"/>
       <c r="AD152" t="inlineStr"/>
-      <c r="AE152" t="n">
-        <v>60.88560885608856</v>
-      </c>
-      <c r="AF152" t="n">
-        <v>60.88560885608856</v>
-      </c>
-      <c r="AG152" t="n">
-        <v>60.88560885608856</v>
-      </c>
+      <c r="AE152" t="inlineStr"/>
+      <c r="AF152" t="inlineStr"/>
+      <c r="AG152" t="inlineStr"/>
       <c r="AH152" t="inlineStr">
         <is>
           <t>29/10/2025</t>
@@ -15005,9 +14405,7 @@
           <t>RIPPIN' PEDRO</t>
         </is>
       </c>
-      <c r="E154" t="n">
-        <v>62.8021978021978</v>
-      </c>
+      <c r="E154" t="inlineStr"/>
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr"/>
@@ -15041,15 +14439,9 @@
       <c r="AB154" t="inlineStr"/>
       <c r="AC154" t="inlineStr"/>
       <c r="AD154" t="inlineStr"/>
-      <c r="AE154" t="n">
-        <v>62.8021978021978</v>
-      </c>
-      <c r="AF154" t="n">
-        <v>62.8021978021978</v>
-      </c>
-      <c r="AG154" t="n">
-        <v>62.8021978021978</v>
-      </c>
+      <c r="AE154" t="inlineStr"/>
+      <c r="AF154" t="inlineStr"/>
+      <c r="AG154" t="inlineStr"/>
       <c r="AH154" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -15193,9 +14585,7 @@
           <t>NOT MUCH KUNA</t>
         </is>
       </c>
-      <c r="E156" t="n">
-        <v>62.46056782334384</v>
-      </c>
+      <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr"/>
@@ -15229,15 +14619,9 @@
       <c r="AB156" t="inlineStr"/>
       <c r="AC156" t="inlineStr"/>
       <c r="AD156" t="inlineStr"/>
-      <c r="AE156" t="n">
-        <v>62.46056782334384</v>
-      </c>
-      <c r="AF156" t="n">
-        <v>62.46056782334384</v>
-      </c>
-      <c r="AG156" t="n">
-        <v>62.46056782334384</v>
-      </c>
+      <c r="AE156" t="inlineStr"/>
+      <c r="AF156" t="inlineStr"/>
+      <c r="AG156" t="inlineStr"/>
       <c r="AH156" t="inlineStr">
         <is>
           <t>22/10/2025</t>
@@ -15381,9 +14765,7 @@
           <t>TEMPTING LULU</t>
         </is>
       </c>
-      <c r="E158" t="n">
-        <v>60.69895769466586</v>
-      </c>
+      <c r="E158" t="inlineStr"/>
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="inlineStr"/>
@@ -15417,15 +14799,9 @@
       <c r="AB158" t="inlineStr"/>
       <c r="AC158" t="inlineStr"/>
       <c r="AD158" t="inlineStr"/>
-      <c r="AE158" t="n">
-        <v>60.69895769466586</v>
-      </c>
-      <c r="AF158" t="n">
-        <v>60.69895769466586</v>
-      </c>
-      <c r="AG158" t="n">
-        <v>60.69895769466586</v>
-      </c>
+      <c r="AE158" t="inlineStr"/>
+      <c r="AF158" t="inlineStr"/>
+      <c r="AG158" t="inlineStr"/>
       <c r="AH158" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -15569,9 +14945,7 @@
           <t>SMILE TIME</t>
         </is>
       </c>
-      <c r="E160" t="n">
-        <v>62.52713851498045</v>
-      </c>
+      <c r="E160" t="inlineStr"/>
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr"/>
       <c r="H160" t="inlineStr"/>
@@ -15605,15 +14979,9 @@
       <c r="AB160" t="inlineStr"/>
       <c r="AC160" t="inlineStr"/>
       <c r="AD160" t="inlineStr"/>
-      <c r="AE160" t="n">
-        <v>62.52713851498045</v>
-      </c>
-      <c r="AF160" t="n">
-        <v>62.52713851498045</v>
-      </c>
-      <c r="AG160" t="n">
-        <v>62.52713851498045</v>
-      </c>
+      <c r="AE160" t="inlineStr"/>
+      <c r="AF160" t="inlineStr"/>
+      <c r="AG160" t="inlineStr"/>
       <c r="AH160" t="inlineStr">
         <is>
           <t>28/10/2025</t>
@@ -15757,9 +15125,7 @@
           <t>RIPPIN' RUBY</t>
         </is>
       </c>
-      <c r="E162" t="n">
-        <v>62.28882833787466</v>
-      </c>
+      <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr"/>
       <c r="H162" t="inlineStr"/>
@@ -15793,15 +15159,9 @@
       <c r="AB162" t="inlineStr"/>
       <c r="AC162" t="inlineStr"/>
       <c r="AD162" t="inlineStr"/>
-      <c r="AE162" t="n">
-        <v>62.28882833787466</v>
-      </c>
-      <c r="AF162" t="n">
-        <v>62.28882833787466</v>
-      </c>
-      <c r="AG162" t="n">
-        <v>62.28882833787466</v>
-      </c>
+      <c r="AE162" t="inlineStr"/>
+      <c r="AF162" t="inlineStr"/>
+      <c r="AG162" t="inlineStr"/>
       <c r="AH162" t="inlineStr">
         <is>
           <t>17/09/2025</t>
@@ -16093,9 +15453,7 @@
           <t>HOLLY CAN BROWSE</t>
         </is>
       </c>
-      <c r="E166" t="n">
-        <v>62.17203586848224</v>
-      </c>
+      <c r="E166" t="inlineStr"/>
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr"/>
       <c r="H166" t="inlineStr"/>
@@ -16129,15 +15487,9 @@
       <c r="AB166" t="inlineStr"/>
       <c r="AC166" t="inlineStr"/>
       <c r="AD166" t="inlineStr"/>
-      <c r="AE166" t="n">
-        <v>62.17203586848224</v>
-      </c>
-      <c r="AF166" t="n">
-        <v>62.17203586848224</v>
-      </c>
-      <c r="AG166" t="n">
-        <v>62.17203586848224</v>
-      </c>
+      <c r="AE166" t="inlineStr"/>
+      <c r="AF166" t="inlineStr"/>
+      <c r="AG166" t="inlineStr"/>
       <c r="AH166" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -16281,9 +15633,7 @@
           <t>MILKY BAR KID</t>
         </is>
       </c>
-      <c r="E168" t="n">
-        <v>62.74473924977127</v>
-      </c>
+      <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="inlineStr"/>
@@ -16317,15 +15667,9 @@
       <c r="AB168" t="inlineStr"/>
       <c r="AC168" t="inlineStr"/>
       <c r="AD168" t="inlineStr"/>
-      <c r="AE168" t="n">
-        <v>62.74473924977127</v>
-      </c>
-      <c r="AF168" t="n">
-        <v>62.74473924977127</v>
-      </c>
-      <c r="AG168" t="n">
-        <v>62.74473924977127</v>
-      </c>
+      <c r="AE168" t="inlineStr"/>
+      <c r="AF168" t="inlineStr"/>
+      <c r="AG168" t="inlineStr"/>
       <c r="AH168" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -16469,9 +15813,7 @@
           <t>MERL'S LAD</t>
         </is>
       </c>
-      <c r="E170" t="n">
-        <v>62.17203586848224</v>
-      </c>
+      <c r="E170" t="inlineStr"/>
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="inlineStr"/>
@@ -16505,15 +15847,9 @@
       <c r="AB170" t="inlineStr"/>
       <c r="AC170" t="inlineStr"/>
       <c r="AD170" t="inlineStr"/>
-      <c r="AE170" t="n">
-        <v>62.17203586848224</v>
-      </c>
-      <c r="AF170" t="n">
-        <v>62.17203586848224</v>
-      </c>
-      <c r="AG170" t="n">
-        <v>62.17203586848224</v>
-      </c>
+      <c r="AE170" t="inlineStr"/>
+      <c r="AF170" t="inlineStr"/>
+      <c r="AG170" t="inlineStr"/>
       <c r="AH170" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -16657,9 +15993,7 @@
           <t>SUNSET AMANDA</t>
         </is>
       </c>
-      <c r="E172" t="n">
-        <v>61.8392134181608</v>
-      </c>
+      <c r="E172" t="inlineStr"/>
       <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr"/>
       <c r="H172" t="inlineStr"/>
@@ -16693,15 +16027,9 @@
       <c r="AB172" t="inlineStr"/>
       <c r="AC172" t="inlineStr"/>
       <c r="AD172" t="inlineStr"/>
-      <c r="AE172" t="n">
-        <v>61.8392134181608</v>
-      </c>
-      <c r="AF172" t="n">
-        <v>61.8392134181608</v>
-      </c>
-      <c r="AG172" t="n">
-        <v>61.8392134181608</v>
-      </c>
+      <c r="AE172" t="inlineStr"/>
+      <c r="AF172" t="inlineStr"/>
+      <c r="AG172" t="inlineStr"/>
       <c r="AH172" t="inlineStr">
         <is>
           <t>6/10/2025</t>
@@ -16845,9 +16173,7 @@
           <t>FEARLESS COBRA</t>
         </is>
       </c>
-      <c r="E174" t="n">
-        <v>62.8021978021978</v>
-      </c>
+      <c r="E174" t="inlineStr"/>
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr"/>
       <c r="H174" t="inlineStr"/>
@@ -16881,15 +16207,9 @@
       <c r="AB174" t="inlineStr"/>
       <c r="AC174" t="inlineStr"/>
       <c r="AD174" t="inlineStr"/>
-      <c r="AE174" t="n">
-        <v>62.8021978021978</v>
-      </c>
-      <c r="AF174" t="n">
-        <v>62.8021978021978</v>
-      </c>
-      <c r="AG174" t="n">
-        <v>62.8021978021978</v>
-      </c>
+      <c r="AE174" t="inlineStr"/>
+      <c r="AF174" t="inlineStr"/>
+      <c r="AG174" t="inlineStr"/>
       <c r="AH174" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -17033,9 +16353,7 @@
           <t>VIVID LOVE</t>
         </is>
       </c>
-      <c r="E176" t="n">
-        <v>63.82978723404256</v>
-      </c>
+      <c r="E176" t="inlineStr"/>
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr"/>
       <c r="H176" t="inlineStr"/>
@@ -17069,15 +16387,9 @@
       <c r="AB176" t="inlineStr"/>
       <c r="AC176" t="inlineStr"/>
       <c r="AD176" t="inlineStr"/>
-      <c r="AE176" t="n">
-        <v>63.82978723404256</v>
-      </c>
-      <c r="AF176" t="n">
-        <v>63.82978723404256</v>
-      </c>
-      <c r="AG176" t="n">
-        <v>63.82978723404256</v>
-      </c>
+      <c r="AE176" t="inlineStr"/>
+      <c r="AF176" t="inlineStr"/>
+      <c r="AG176" t="inlineStr"/>
       <c r="AH176" t="inlineStr">
         <is>
           <t>30/10/2025</t>
@@ -17221,9 +16533,7 @@
           <t>RAPIDO PRONTO</t>
         </is>
       </c>
-      <c r="E178" t="n">
-        <v>62.68738574040219</v>
-      </c>
+      <c r="E178" t="inlineStr"/>
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr"/>
       <c r="H178" t="inlineStr"/>
@@ -17257,15 +16567,9 @@
       <c r="AB178" t="inlineStr"/>
       <c r="AC178" t="inlineStr"/>
       <c r="AD178" t="inlineStr"/>
-      <c r="AE178" t="n">
-        <v>62.68738574040219</v>
-      </c>
-      <c r="AF178" t="n">
-        <v>62.68738574040219</v>
-      </c>
-      <c r="AG178" t="n">
-        <v>62.68738574040219</v>
-      </c>
+      <c r="AE178" t="inlineStr"/>
+      <c r="AF178" t="inlineStr"/>
+      <c r="AG178" t="inlineStr"/>
       <c r="AH178" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -17409,9 +16713,7 @@
           <t>DOREEN KEEPING</t>
         </is>
       </c>
-      <c r="E180" t="n">
-        <v>62.97709923664122</v>
-      </c>
+      <c r="E180" t="inlineStr"/>
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr"/>
       <c r="H180" t="inlineStr"/>
@@ -17445,15 +16747,9 @@
       <c r="AB180" t="inlineStr"/>
       <c r="AC180" t="inlineStr"/>
       <c r="AD180" t="inlineStr"/>
-      <c r="AE180" t="n">
-        <v>62.97709923664122</v>
-      </c>
-      <c r="AF180" t="n">
-        <v>62.97709923664122</v>
-      </c>
-      <c r="AG180" t="n">
-        <v>62.97709923664122</v>
-      </c>
+      <c r="AE180" t="inlineStr"/>
+      <c r="AF180" t="inlineStr"/>
+      <c r="AG180" t="inlineStr"/>
       <c r="AH180" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -17597,9 +16893,7 @@
           <t>WIZARD'S NERO</t>
         </is>
       </c>
-      <c r="E182" t="n">
-        <v>62.10465784933871</v>
-      </c>
+      <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr"/>
       <c r="H182" t="inlineStr"/>
@@ -17633,15 +16927,9 @@
       <c r="AB182" t="inlineStr"/>
       <c r="AC182" t="inlineStr"/>
       <c r="AD182" t="inlineStr"/>
-      <c r="AE182" t="n">
-        <v>62.10465784933871</v>
-      </c>
-      <c r="AF182" t="n">
-        <v>62.10465784933871</v>
-      </c>
-      <c r="AG182" t="n">
-        <v>62.10465784933871</v>
-      </c>
+      <c r="AE182" t="inlineStr"/>
+      <c r="AF182" t="inlineStr"/>
+      <c r="AG182" t="inlineStr"/>
       <c r="AH182" t="inlineStr">
         <is>
           <t>3/11/2025</t>
@@ -17717,9 +17005,7 @@
           <t>NO ROLE MODELS</t>
         </is>
       </c>
-      <c r="E183" t="n">
-        <v>62.1195652173913</v>
-      </c>
+      <c r="E183" t="inlineStr"/>
       <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr"/>
       <c r="H183" t="inlineStr"/>
@@ -17753,15 +17039,9 @@
       <c r="AB183" t="inlineStr"/>
       <c r="AC183" t="inlineStr"/>
       <c r="AD183" t="inlineStr"/>
-      <c r="AE183" t="n">
-        <v>62.1195652173913</v>
-      </c>
-      <c r="AF183" t="n">
-        <v>62.1195652173913</v>
-      </c>
-      <c r="AG183" t="n">
-        <v>62.1195652173913</v>
-      </c>
+      <c r="AE183" t="inlineStr"/>
+      <c r="AF183" t="inlineStr"/>
+      <c r="AG183" t="inlineStr"/>
       <c r="AH183" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -17905,9 +17185,7 @@
           <t>NAUGHTY EVIE</t>
         </is>
       </c>
-      <c r="E185" t="n">
-        <v>61.94573130377233</v>
-      </c>
+      <c r="E185" t="inlineStr"/>
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr"/>
       <c r="H185" t="inlineStr"/>
@@ -17941,15 +17219,9 @@
       <c r="AB185" t="inlineStr"/>
       <c r="AC185" t="inlineStr"/>
       <c r="AD185" t="inlineStr"/>
-      <c r="AE185" t="n">
-        <v>61.94573130377233</v>
-      </c>
-      <c r="AF185" t="n">
-        <v>61.94573130377233</v>
-      </c>
-      <c r="AG185" t="n">
-        <v>61.94573130377233</v>
-      </c>
+      <c r="AE185" t="inlineStr"/>
+      <c r="AF185" t="inlineStr"/>
+      <c r="AG185" t="inlineStr"/>
       <c r="AH185" t="inlineStr">
         <is>
           <t>8/11/2025</t>
@@ -18093,9 +17365,7 @@
           <t>OFF SHORE</t>
         </is>
       </c>
-      <c r="E187" t="n">
-        <v>62.1195652173913</v>
-      </c>
+      <c r="E187" t="inlineStr"/>
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr"/>
       <c r="H187" t="inlineStr"/>
@@ -18129,15 +17399,9 @@
       <c r="AB187" t="inlineStr"/>
       <c r="AC187" t="inlineStr"/>
       <c r="AD187" t="inlineStr"/>
-      <c r="AE187" t="n">
-        <v>62.1195652173913</v>
-      </c>
-      <c r="AF187" t="n">
-        <v>62.1195652173913</v>
-      </c>
-      <c r="AG187" t="n">
-        <v>62.1195652173913</v>
-      </c>
+      <c r="AE187" t="inlineStr"/>
+      <c r="AF187" t="inlineStr"/>
+      <c r="AG187" t="inlineStr"/>
       <c r="AH187" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -18281,9 +17545,7 @@
           <t>ROCKIN' KINLOCH</t>
         </is>
       </c>
-      <c r="E189" t="n">
-        <v>62.1195652173913</v>
-      </c>
+      <c r="E189" t="inlineStr"/>
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr"/>
       <c r="H189" t="inlineStr"/>
@@ -18317,15 +17579,9 @@
       <c r="AB189" t="inlineStr"/>
       <c r="AC189" t="inlineStr"/>
       <c r="AD189" t="inlineStr"/>
-      <c r="AE189" t="n">
-        <v>62.1195652173913</v>
-      </c>
-      <c r="AF189" t="n">
-        <v>62.1195652173913</v>
-      </c>
-      <c r="AG189" t="n">
-        <v>62.1195652173913</v>
-      </c>
+      <c r="AE189" t="inlineStr"/>
+      <c r="AF189" t="inlineStr"/>
+      <c r="AG189" t="inlineStr"/>
       <c r="AH189" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -18469,9 +17725,7 @@
           <t>CITY OF LOVE</t>
         </is>
       </c>
-      <c r="E191" t="n">
-        <v>61.78378378378378</v>
-      </c>
+      <c r="E191" t="inlineStr"/>
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr"/>
       <c r="H191" t="inlineStr"/>
@@ -18505,15 +17759,9 @@
       <c r="AB191" t="inlineStr"/>
       <c r="AC191" t="inlineStr"/>
       <c r="AD191" t="inlineStr"/>
-      <c r="AE191" t="n">
-        <v>61.78378378378378</v>
-      </c>
-      <c r="AF191" t="n">
-        <v>61.78378378378378</v>
-      </c>
-      <c r="AG191" t="n">
-        <v>61.78378378378378</v>
-      </c>
+      <c r="AE191" t="inlineStr"/>
+      <c r="AF191" t="inlineStr"/>
+      <c r="AG191" t="inlineStr"/>
       <c r="AH191" t="inlineStr">
         <is>
           <t>8/11/2025</t>
@@ -18657,9 +17905,7 @@
           <t>MUST BE SPEEDY</t>
         </is>
       </c>
-      <c r="E193" t="n">
-        <v>63.74455732946299</v>
-      </c>
+      <c r="E193" t="inlineStr"/>
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr"/>
       <c r="H193" t="inlineStr"/>
@@ -18693,15 +17939,9 @@
       <c r="AB193" t="inlineStr"/>
       <c r="AC193" t="inlineStr"/>
       <c r="AD193" t="inlineStr"/>
-      <c r="AE193" t="n">
-        <v>63.74455732946299</v>
-      </c>
-      <c r="AF193" t="n">
-        <v>63.74455732946299</v>
-      </c>
-      <c r="AG193" t="n">
-        <v>63.74455732946299</v>
-      </c>
+      <c r="AE193" t="inlineStr"/>
+      <c r="AF193" t="inlineStr"/>
+      <c r="AG193" t="inlineStr"/>
       <c r="AH193" t="inlineStr">
         <is>
           <t>7/11/2025</t>
@@ -18845,9 +18085,7 @@
           <t>FIDEL PRONTO</t>
         </is>
       </c>
-      <c r="E195" t="n">
-        <v>62.68738574040219</v>
-      </c>
+      <c r="E195" t="inlineStr"/>
       <c r="F195" t="inlineStr"/>
       <c r="G195" t="inlineStr"/>
       <c r="H195" t="inlineStr"/>
@@ -18881,15 +18119,9 @@
       <c r="AB195" t="inlineStr"/>
       <c r="AC195" t="inlineStr"/>
       <c r="AD195" t="inlineStr"/>
-      <c r="AE195" t="n">
-        <v>62.68738574040219</v>
-      </c>
-      <c r="AF195" t="n">
-        <v>62.68738574040219</v>
-      </c>
-      <c r="AG195" t="n">
-        <v>62.68738574040219</v>
-      </c>
+      <c r="AE195" t="inlineStr"/>
+      <c r="AF195" t="inlineStr"/>
+      <c r="AG195" t="inlineStr"/>
       <c r="AH195" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -19033,9 +18265,7 @@
           <t>SHINBONER PIXIE</t>
         </is>
       </c>
-      <c r="E197" t="n">
-        <v>62.23230490018149</v>
-      </c>
+      <c r="E197" t="inlineStr"/>
       <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr"/>
       <c r="H197" t="inlineStr"/>
@@ -19069,15 +18299,9 @@
       <c r="AB197" t="inlineStr"/>
       <c r="AC197" t="inlineStr"/>
       <c r="AD197" t="inlineStr"/>
-      <c r="AE197" t="n">
-        <v>62.23230490018149</v>
-      </c>
-      <c r="AF197" t="n">
-        <v>62.23230490018149</v>
-      </c>
-      <c r="AG197" t="n">
-        <v>62.23230490018149</v>
-      </c>
+      <c r="AE197" t="inlineStr"/>
+      <c r="AF197" t="inlineStr"/>
+      <c r="AG197" t="inlineStr"/>
       <c r="AH197" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -19221,9 +18445,7 @@
           <t>POP'S ANGEL</t>
         </is>
       </c>
-      <c r="E199" t="n">
-        <v>61.08597285067874</v>
-      </c>
+      <c r="E199" t="inlineStr"/>
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr"/>
       <c r="H199" t="inlineStr"/>
@@ -19257,15 +18479,9 @@
       <c r="AB199" t="inlineStr"/>
       <c r="AC199" t="inlineStr"/>
       <c r="AD199" t="inlineStr"/>
-      <c r="AE199" t="n">
-        <v>61.08597285067874</v>
-      </c>
-      <c r="AF199" t="n">
-        <v>61.08597285067874</v>
-      </c>
-      <c r="AG199" t="n">
-        <v>61.08597285067874</v>
-      </c>
+      <c r="AE199" t="inlineStr"/>
+      <c r="AF199" t="inlineStr"/>
+      <c r="AG199" t="inlineStr"/>
       <c r="AH199" t="inlineStr">
         <is>
           <t>3/11/2025</t>
@@ -19409,9 +18625,7 @@
           <t>LIGHTNING BOLT</t>
         </is>
       </c>
-      <c r="E201" t="n">
-        <v>62.1195652173913</v>
-      </c>
+      <c r="E201" t="inlineStr"/>
       <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="inlineStr"/>
@@ -19445,15 +18659,9 @@
       <c r="AB201" t="inlineStr"/>
       <c r="AC201" t="inlineStr"/>
       <c r="AD201" t="inlineStr"/>
-      <c r="AE201" t="n">
-        <v>62.1195652173913</v>
-      </c>
-      <c r="AF201" t="n">
-        <v>62.1195652173913</v>
-      </c>
-      <c r="AG201" t="n">
-        <v>62.1195652173913</v>
-      </c>
+      <c r="AE201" t="inlineStr"/>
+      <c r="AF201" t="inlineStr"/>
+      <c r="AG201" t="inlineStr"/>
       <c r="AH201" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -19529,9 +18737,7 @@
           <t>OFF SHORE</t>
         </is>
       </c>
-      <c r="E202" t="n">
-        <v>62.1195652173913</v>
-      </c>
+      <c r="E202" t="inlineStr"/>
       <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr"/>
       <c r="H202" t="inlineStr"/>
@@ -19565,15 +18771,9 @@
       <c r="AB202" t="inlineStr"/>
       <c r="AC202" t="inlineStr"/>
       <c r="AD202" t="inlineStr"/>
-      <c r="AE202" t="n">
-        <v>62.1195652173913</v>
-      </c>
-      <c r="AF202" t="n">
-        <v>62.1195652173913</v>
-      </c>
-      <c r="AG202" t="n">
-        <v>62.1195652173913</v>
-      </c>
+      <c r="AE202" t="inlineStr"/>
+      <c r="AF202" t="inlineStr"/>
+      <c r="AG202" t="inlineStr"/>
       <c r="AH202" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -19717,9 +18917,7 @@
           <t>NAUGHTY EVIE</t>
         </is>
       </c>
-      <c r="E204" t="n">
-        <v>61.94573130377233</v>
-      </c>
+      <c r="E204" t="inlineStr"/>
       <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr"/>
       <c r="H204" t="inlineStr"/>
@@ -19753,15 +18951,9 @@
       <c r="AB204" t="inlineStr"/>
       <c r="AC204" t="inlineStr"/>
       <c r="AD204" t="inlineStr"/>
-      <c r="AE204" t="n">
-        <v>61.94573130377233</v>
-      </c>
-      <c r="AF204" t="n">
-        <v>61.94573130377233</v>
-      </c>
-      <c r="AG204" t="n">
-        <v>61.94573130377233</v>
-      </c>
+      <c r="AE204" t="inlineStr"/>
+      <c r="AF204" t="inlineStr"/>
+      <c r="AG204" t="inlineStr"/>
       <c r="AH204" t="inlineStr">
         <is>
           <t>8/11/2025</t>
@@ -19905,9 +19097,7 @@
           <t>MAKUTZ</t>
         </is>
       </c>
-      <c r="E206" t="n">
-        <v>62.74473924977127</v>
-      </c>
+      <c r="E206" t="inlineStr"/>
       <c r="F206" t="inlineStr"/>
       <c r="G206" t="inlineStr"/>
       <c r="H206" t="inlineStr"/>
@@ -19941,15 +19131,9 @@
       <c r="AB206" t="inlineStr"/>
       <c r="AC206" t="inlineStr"/>
       <c r="AD206" t="inlineStr"/>
-      <c r="AE206" t="n">
-        <v>62.74473924977127</v>
-      </c>
-      <c r="AF206" t="n">
-        <v>62.74473924977127</v>
-      </c>
-      <c r="AG206" t="n">
-        <v>62.74473924977127</v>
-      </c>
+      <c r="AE206" t="inlineStr"/>
+      <c r="AF206" t="inlineStr"/>
+      <c r="AG206" t="inlineStr"/>
       <c r="AH206" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -20093,9 +19277,7 @@
           <t>CHAMBERLAIN</t>
         </is>
       </c>
-      <c r="E208" t="n">
-        <v>64.02845709204091</v>
-      </c>
+      <c r="E208" t="inlineStr"/>
       <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr"/>
       <c r="H208" t="inlineStr"/>
@@ -20129,15 +19311,9 @@
       <c r="AB208" t="inlineStr"/>
       <c r="AC208" t="inlineStr"/>
       <c r="AD208" t="inlineStr"/>
-      <c r="AE208" t="n">
-        <v>64.02845709204091</v>
-      </c>
-      <c r="AF208" t="n">
-        <v>64.02845709204091</v>
-      </c>
-      <c r="AG208" t="n">
-        <v>64.02845709204091</v>
-      </c>
+      <c r="AE208" t="inlineStr"/>
+      <c r="AF208" t="inlineStr"/>
+      <c r="AG208" t="inlineStr"/>
       <c r="AH208" t="inlineStr">
         <is>
           <t>10/10/2025</t>
@@ -20281,9 +19457,7 @@
           <t>BISCOTTI BLAST</t>
         </is>
       </c>
-      <c r="E210" t="n">
-        <v>62.96670030272453</v>
-      </c>
+      <c r="E210" t="inlineStr"/>
       <c r="F210" t="inlineStr"/>
       <c r="G210" t="inlineStr"/>
       <c r="H210" t="inlineStr"/>
@@ -20317,15 +19491,9 @@
       <c r="AB210" t="inlineStr"/>
       <c r="AC210" t="inlineStr"/>
       <c r="AD210" t="inlineStr"/>
-      <c r="AE210" t="n">
-        <v>62.96670030272453</v>
-      </c>
-      <c r="AF210" t="n">
-        <v>62.96670030272453</v>
-      </c>
-      <c r="AG210" t="n">
-        <v>62.96670030272453</v>
-      </c>
+      <c r="AE210" t="inlineStr"/>
+      <c r="AF210" t="inlineStr"/>
+      <c r="AG210" t="inlineStr"/>
       <c r="AH210" t="inlineStr">
         <is>
           <t>1/11/2025</t>
@@ -20469,9 +19637,7 @@
           <t>CONCORD GUNDI</t>
         </is>
       </c>
-      <c r="E212" t="n">
-        <v>62.68738574040219</v>
-      </c>
+      <c r="E212" t="inlineStr"/>
       <c r="F212" t="inlineStr"/>
       <c r="G212" t="inlineStr"/>
       <c r="H212" t="inlineStr"/>
@@ -20505,15 +19671,9 @@
       <c r="AB212" t="inlineStr"/>
       <c r="AC212" t="inlineStr"/>
       <c r="AD212" t="inlineStr"/>
-      <c r="AE212" t="n">
-        <v>62.68738574040219</v>
-      </c>
-      <c r="AF212" t="n">
-        <v>62.68738574040219</v>
-      </c>
-      <c r="AG212" t="n">
-        <v>62.68738574040219</v>
-      </c>
+      <c r="AE212" t="inlineStr"/>
+      <c r="AF212" t="inlineStr"/>
+      <c r="AG212" t="inlineStr"/>
       <c r="AH212" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -20657,9 +19817,7 @@
           <t>WEST ON HALO</t>
         </is>
       </c>
-      <c r="E214" t="n">
-        <v>62.23230490018149</v>
-      </c>
+      <c r="E214" t="inlineStr"/>
       <c r="F214" t="inlineStr"/>
       <c r="G214" t="inlineStr"/>
       <c r="H214" t="inlineStr"/>
@@ -20693,15 +19851,9 @@
       <c r="AB214" t="inlineStr"/>
       <c r="AC214" t="inlineStr"/>
       <c r="AD214" t="inlineStr"/>
-      <c r="AE214" t="n">
-        <v>62.23230490018149</v>
-      </c>
-      <c r="AF214" t="n">
-        <v>62.23230490018149</v>
-      </c>
-      <c r="AG214" t="n">
-        <v>62.23230490018149</v>
-      </c>
+      <c r="AE214" t="inlineStr"/>
+      <c r="AF214" t="inlineStr"/>
+      <c r="AG214" t="inlineStr"/>
       <c r="AH214" t="inlineStr">
         <is>
           <t>5/11/2025</t>

</xml_diff>

<commit_message>
Add speed computation and consistency validation per Phase 7 requirements
Co-authored-by: danieljohnconstantine-a11y <229551202+danieljohnconstantine-a11y@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/all_dogs_master.xlsx
+++ b/outputs/all_dogs_master.xlsx
@@ -808,9 +808,15 @@
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
+      <c r="AD3" t="n">
+        <v>62.46385193753615</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>62.46385193753615</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>62.46385193753615</v>
+      </c>
       <c r="AG3" t="inlineStr">
         <is>
           <t>6/11/2025</t>
@@ -839,7 +845,9 @@
         </is>
       </c>
       <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
+      <c r="AO3" t="n">
+        <v>62.46385193753615</v>
+      </c>
       <c r="AP3" t="inlineStr"/>
       <c r="AQ3" t="inlineStr"/>
       <c r="AR3" t="inlineStr">
@@ -978,9 +986,15 @@
       <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
+      <c r="AD5" t="n">
+        <v>62.1195652173913</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>62.1195652173913</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>62.1195652173913</v>
+      </c>
       <c r="AG5" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -1009,7 +1023,9 @@
         </is>
       </c>
       <c r="AN5" t="inlineStr"/>
-      <c r="AO5" t="inlineStr"/>
+      <c r="AO5" t="n">
+        <v>62.1195652173913</v>
+      </c>
       <c r="AP5" t="inlineStr"/>
       <c r="AQ5" t="inlineStr"/>
       <c r="AR5" t="inlineStr">
@@ -1148,9 +1164,15 @@
       <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
-      <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr"/>
+      <c r="AD7" t="n">
+        <v>61.29398410896709</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>61.29398410896709</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>61.29398410896709</v>
+      </c>
       <c r="AG7" t="inlineStr">
         <is>
           <t>16/10/2025</t>
@@ -1179,7 +1201,9 @@
         </is>
       </c>
       <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr"/>
+      <c r="AO7" t="n">
+        <v>61.29398410896709</v>
+      </c>
       <c r="AP7" t="inlineStr"/>
       <c r="AQ7" t="inlineStr"/>
       <c r="AR7" t="inlineStr">
@@ -1393,9 +1417,15 @@
       <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
-      <c r="AD10" t="inlineStr"/>
-      <c r="AE10" t="inlineStr"/>
-      <c r="AF10" t="inlineStr"/>
+      <c r="AD10" t="n">
+        <v>63.10344827586208</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>63.10344827586208</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>63.10344827586208</v>
+      </c>
       <c r="AG10" t="inlineStr">
         <is>
           <t>4/11/2025</t>
@@ -1424,7 +1454,9 @@
         </is>
       </c>
       <c r="AN10" t="inlineStr"/>
-      <c r="AO10" t="inlineStr"/>
+      <c r="AO10" t="n">
+        <v>63.10344827586208</v>
+      </c>
       <c r="AP10" t="inlineStr"/>
       <c r="AQ10" t="inlineStr"/>
       <c r="AR10" t="inlineStr">
@@ -1563,9 +1595,15 @@
       <c r="AA12" t="inlineStr"/>
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
-      <c r="AD12" t="inlineStr"/>
-      <c r="AE12" t="inlineStr"/>
-      <c r="AF12" t="inlineStr"/>
+      <c r="AD12" t="n">
+        <v>63.85809312638581</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>63.85809312638581</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>63.85809312638581</v>
+      </c>
       <c r="AG12" t="inlineStr">
         <is>
           <t>4/11/2025</t>
@@ -1594,7 +1632,9 @@
         </is>
       </c>
       <c r="AN12" t="inlineStr"/>
-      <c r="AO12" t="inlineStr"/>
+      <c r="AO12" t="n">
+        <v>63.85809312638581</v>
+      </c>
       <c r="AP12" t="inlineStr"/>
       <c r="AQ12" t="inlineStr"/>
       <c r="AR12" t="inlineStr">
@@ -1733,9 +1773,15 @@
       <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr"/>
-      <c r="AD14" t="inlineStr"/>
-      <c r="AE14" t="inlineStr"/>
-      <c r="AF14" t="inlineStr"/>
+      <c r="AD14" t="n">
+        <v>62.46385193753615</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>62.46385193753615</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>62.46385193753615</v>
+      </c>
       <c r="AG14" t="inlineStr">
         <is>
           <t>6/11/2025</t>
@@ -1764,7 +1810,9 @@
         </is>
       </c>
       <c r="AN14" t="inlineStr"/>
-      <c r="AO14" t="inlineStr"/>
+      <c r="AO14" t="n">
+        <v>62.46385193753615</v>
+      </c>
       <c r="AP14" t="inlineStr"/>
       <c r="AQ14" t="inlineStr"/>
       <c r="AR14" t="inlineStr">
@@ -1903,9 +1951,15 @@
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr"/>
-      <c r="AD16" t="inlineStr"/>
-      <c r="AE16" t="inlineStr"/>
-      <c r="AF16" t="inlineStr"/>
+      <c r="AD16" t="n">
+        <v>63.44125809435707</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>63.44125809435707</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>63.44125809435707</v>
+      </c>
       <c r="AG16" t="inlineStr">
         <is>
           <t>22/10/2025</t>
@@ -1934,7 +1988,9 @@
         </is>
       </c>
       <c r="AN16" t="inlineStr"/>
-      <c r="AO16" t="inlineStr"/>
+      <c r="AO16" t="n">
+        <v>63.44125809435707</v>
+      </c>
       <c r="AP16" t="inlineStr"/>
       <c r="AQ16" t="inlineStr"/>
       <c r="AR16" t="inlineStr">
@@ -2073,9 +2129,15 @@
       <c r="AA18" t="inlineStr"/>
       <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="inlineStr"/>
-      <c r="AD18" t="inlineStr"/>
-      <c r="AE18" t="inlineStr"/>
-      <c r="AF18" t="inlineStr"/>
+      <c r="AD18" t="n">
+        <v>62.68738574040219</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>62.68738574040219</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>62.68738574040219</v>
+      </c>
       <c r="AG18" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -2104,7 +2166,9 @@
         </is>
       </c>
       <c r="AN18" t="inlineStr"/>
-      <c r="AO18" t="inlineStr"/>
+      <c r="AO18" t="n">
+        <v>62.68738574040219</v>
+      </c>
       <c r="AP18" t="inlineStr"/>
       <c r="AQ18" t="inlineStr"/>
       <c r="AR18" t="inlineStr">
@@ -2243,9 +2307,15 @@
       <c r="AA20" t="inlineStr"/>
       <c r="AB20" t="inlineStr"/>
       <c r="AC20" t="inlineStr"/>
-      <c r="AD20" t="inlineStr"/>
-      <c r="AE20" t="inlineStr"/>
-      <c r="AF20" t="inlineStr"/>
+      <c r="AD20" t="n">
+        <v>62.46385193753615</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>62.46385193753615</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>62.46385193753615</v>
+      </c>
       <c r="AG20" t="inlineStr">
         <is>
           <t>6/11/2025</t>
@@ -2274,7 +2344,9 @@
         </is>
       </c>
       <c r="AN20" t="inlineStr"/>
-      <c r="AO20" t="inlineStr"/>
+      <c r="AO20" t="n">
+        <v>62.46385193753615</v>
+      </c>
       <c r="AP20" t="inlineStr"/>
       <c r="AQ20" t="inlineStr"/>
       <c r="AR20" t="inlineStr">
@@ -2413,9 +2485,15 @@
       <c r="AA22" t="inlineStr"/>
       <c r="AB22" t="inlineStr"/>
       <c r="AC22" t="inlineStr"/>
-      <c r="AD22" t="inlineStr"/>
-      <c r="AE22" t="inlineStr"/>
-      <c r="AF22" t="inlineStr"/>
+      <c r="AD22" t="n">
+        <v>62.23230490018149</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>62.23230490018149</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>62.23230490018149</v>
+      </c>
       <c r="AG22" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -2444,7 +2522,9 @@
         </is>
       </c>
       <c r="AN22" t="inlineStr"/>
-      <c r="AO22" t="inlineStr"/>
+      <c r="AO22" t="n">
+        <v>62.23230490018149</v>
+      </c>
       <c r="AP22" t="inlineStr"/>
       <c r="AQ22" t="inlineStr"/>
       <c r="AR22" t="inlineStr">
@@ -2583,9 +2663,15 @@
       <c r="AA24" t="inlineStr"/>
       <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="inlineStr"/>
-      <c r="AD24" t="inlineStr"/>
-      <c r="AE24" t="inlineStr"/>
-      <c r="AF24" t="inlineStr"/>
+      <c r="AD24" t="n">
+        <v>62.97709923664122</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>62.97709923664122</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>62.97709923664122</v>
+      </c>
       <c r="AG24" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -2614,7 +2700,9 @@
         </is>
       </c>
       <c r="AN24" t="inlineStr"/>
-      <c r="AO24" t="inlineStr"/>
+      <c r="AO24" t="n">
+        <v>62.97709923664122</v>
+      </c>
       <c r="AP24" t="inlineStr"/>
       <c r="AQ24" t="inlineStr"/>
       <c r="AR24" t="inlineStr">
@@ -2753,9 +2841,15 @@
       <c r="AA26" t="inlineStr"/>
       <c r="AB26" t="inlineStr"/>
       <c r="AC26" t="inlineStr"/>
-      <c r="AD26" t="inlineStr"/>
-      <c r="AE26" t="inlineStr"/>
-      <c r="AF26" t="inlineStr"/>
+      <c r="AD26" t="n">
+        <v>60.69895769466586</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>60.69895769466586</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>60.69895769466586</v>
+      </c>
       <c r="AG26" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -2784,7 +2878,9 @@
         </is>
       </c>
       <c r="AN26" t="inlineStr"/>
-      <c r="AO26" t="inlineStr"/>
+      <c r="AO26" t="n">
+        <v>60.69895769466586</v>
+      </c>
       <c r="AP26" t="inlineStr"/>
       <c r="AQ26" t="inlineStr"/>
       <c r="AR26" t="inlineStr">
@@ -2923,9 +3019,15 @@
       <c r="AA28" t="inlineStr"/>
       <c r="AB28" t="inlineStr"/>
       <c r="AC28" t="inlineStr"/>
-      <c r="AD28" t="inlineStr"/>
-      <c r="AE28" t="inlineStr"/>
-      <c r="AF28" t="inlineStr"/>
+      <c r="AD28" t="n">
+        <v>61.47915732855223</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>61.47915732855223</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>61.47915732855223</v>
+      </c>
       <c r="AG28" t="inlineStr">
         <is>
           <t>22/10/2025</t>
@@ -2954,7 +3056,9 @@
         </is>
       </c>
       <c r="AN28" t="inlineStr"/>
-      <c r="AO28" t="inlineStr"/>
+      <c r="AO28" t="n">
+        <v>61.47915732855223</v>
+      </c>
       <c r="AP28" t="inlineStr"/>
       <c r="AQ28" t="inlineStr"/>
       <c r="AR28" t="inlineStr">
@@ -3030,9 +3134,15 @@
       <c r="AA29" t="inlineStr"/>
       <c r="AB29" t="inlineStr"/>
       <c r="AC29" t="inlineStr"/>
-      <c r="AD29" t="inlineStr"/>
-      <c r="AE29" t="inlineStr"/>
-      <c r="AF29" t="inlineStr"/>
+      <c r="AD29" t="n">
+        <v>62.048392442824</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>62.048392442824</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>62.048392442824</v>
+      </c>
       <c r="AG29" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -3061,7 +3171,9 @@
         </is>
       </c>
       <c r="AN29" t="inlineStr"/>
-      <c r="AO29" t="inlineStr"/>
+      <c r="AO29" t="n">
+        <v>62.048392442824</v>
+      </c>
       <c r="AP29" t="inlineStr"/>
       <c r="AQ29" t="inlineStr"/>
       <c r="AR29" t="inlineStr">
@@ -3200,9 +3312,15 @@
       <c r="AA31" t="inlineStr"/>
       <c r="AB31" t="inlineStr"/>
       <c r="AC31" t="inlineStr"/>
-      <c r="AD31" t="inlineStr"/>
-      <c r="AE31" t="inlineStr"/>
-      <c r="AF31" t="inlineStr"/>
+      <c r="AD31" t="n">
+        <v>62.048392442824</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>62.048392442824</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>62.048392442824</v>
+      </c>
       <c r="AG31" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -3231,7 +3349,9 @@
         </is>
       </c>
       <c r="AN31" t="inlineStr"/>
-      <c r="AO31" t="inlineStr"/>
+      <c r="AO31" t="n">
+        <v>62.048392442824</v>
+      </c>
       <c r="AP31" t="inlineStr"/>
       <c r="AQ31" t="inlineStr"/>
       <c r="AR31" t="inlineStr">
@@ -3370,9 +3490,15 @@
       <c r="AA33" t="inlineStr"/>
       <c r="AB33" t="inlineStr"/>
       <c r="AC33" t="inlineStr"/>
-      <c r="AD33" t="inlineStr"/>
-      <c r="AE33" t="inlineStr"/>
-      <c r="AF33" t="inlineStr"/>
+      <c r="AD33" t="n">
+        <v>62.17203586848224</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>62.17203586848224</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>62.17203586848224</v>
+      </c>
       <c r="AG33" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -3401,7 +3527,9 @@
         </is>
       </c>
       <c r="AN33" t="inlineStr"/>
-      <c r="AO33" t="inlineStr"/>
+      <c r="AO33" t="n">
+        <v>62.17203586848224</v>
+      </c>
       <c r="AP33" t="inlineStr"/>
       <c r="AQ33" t="inlineStr"/>
       <c r="AR33" t="inlineStr">
@@ -3540,9 +3668,15 @@
       <c r="AA35" t="inlineStr"/>
       <c r="AB35" t="inlineStr"/>
       <c r="AC35" t="inlineStr"/>
-      <c r="AD35" t="inlineStr"/>
-      <c r="AE35" t="inlineStr"/>
-      <c r="AF35" t="inlineStr"/>
+      <c r="AD35" t="n">
+        <v>62.74473924977127</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>62.74473924977127</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>62.74473924977127</v>
+      </c>
       <c r="AG35" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -3571,7 +3705,9 @@
         </is>
       </c>
       <c r="AN35" t="inlineStr"/>
-      <c r="AO35" t="inlineStr"/>
+      <c r="AO35" t="n">
+        <v>62.74473924977127</v>
+      </c>
       <c r="AP35" t="inlineStr"/>
       <c r="AQ35" t="inlineStr"/>
       <c r="AR35" t="inlineStr">
@@ -3710,9 +3846,15 @@
       <c r="AA37" t="inlineStr"/>
       <c r="AB37" t="inlineStr"/>
       <c r="AC37" t="inlineStr"/>
-      <c r="AD37" t="inlineStr"/>
-      <c r="AE37" t="inlineStr"/>
-      <c r="AF37" t="inlineStr"/>
+      <c r="AD37" t="n">
+        <v>61.22285332442365</v>
+      </c>
+      <c r="AE37" t="n">
+        <v>61.22285332442365</v>
+      </c>
+      <c r="AF37" t="n">
+        <v>61.22285332442365</v>
+      </c>
       <c r="AG37" t="inlineStr">
         <is>
           <t>27/10/2025</t>
@@ -3741,7 +3883,9 @@
         </is>
       </c>
       <c r="AN37" t="inlineStr"/>
-      <c r="AO37" t="inlineStr"/>
+      <c r="AO37" t="n">
+        <v>61.22285332442365</v>
+      </c>
       <c r="AP37" t="inlineStr"/>
       <c r="AQ37" t="inlineStr"/>
       <c r="AR37" t="inlineStr">
@@ -3880,9 +4024,15 @@
       <c r="AA39" t="inlineStr"/>
       <c r="AB39" t="inlineStr"/>
       <c r="AC39" t="inlineStr"/>
-      <c r="AD39" t="inlineStr"/>
-      <c r="AE39" t="inlineStr"/>
-      <c r="AF39" t="inlineStr"/>
+      <c r="AD39" t="n">
+        <v>61.9054054054054</v>
+      </c>
+      <c r="AE39" t="n">
+        <v>61.9054054054054</v>
+      </c>
+      <c r="AF39" t="n">
+        <v>61.9054054054054</v>
+      </c>
       <c r="AG39" t="inlineStr">
         <is>
           <t>13/10/2025</t>
@@ -3911,7 +4061,9 @@
         </is>
       </c>
       <c r="AN39" t="inlineStr"/>
-      <c r="AO39" t="inlineStr"/>
+      <c r="AO39" t="n">
+        <v>61.9054054054054</v>
+      </c>
       <c r="AP39" t="inlineStr"/>
       <c r="AQ39" t="inlineStr"/>
       <c r="AR39" t="inlineStr">
@@ -4050,9 +4202,15 @@
       <c r="AA41" t="inlineStr"/>
       <c r="AB41" t="inlineStr"/>
       <c r="AC41" t="inlineStr"/>
-      <c r="AD41" t="inlineStr"/>
-      <c r="AE41" t="inlineStr"/>
-      <c r="AF41" t="inlineStr"/>
+      <c r="AD41" t="n">
+        <v>62.23404255319149</v>
+      </c>
+      <c r="AE41" t="n">
+        <v>62.23404255319149</v>
+      </c>
+      <c r="AF41" t="n">
+        <v>62.23404255319149</v>
+      </c>
       <c r="AG41" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -4081,7 +4239,9 @@
         </is>
       </c>
       <c r="AN41" t="inlineStr"/>
-      <c r="AO41" t="inlineStr"/>
+      <c r="AO41" t="n">
+        <v>62.23404255319149</v>
+      </c>
       <c r="AP41" t="inlineStr"/>
       <c r="AQ41" t="inlineStr"/>
       <c r="AR41" t="inlineStr">
@@ -4220,9 +4380,15 @@
       <c r="AA43" t="inlineStr"/>
       <c r="AB43" t="inlineStr"/>
       <c r="AC43" t="inlineStr"/>
-      <c r="AD43" t="inlineStr"/>
-      <c r="AE43" t="inlineStr"/>
-      <c r="AF43" t="inlineStr"/>
+      <c r="AD43" t="n">
+        <v>62.97709923664122</v>
+      </c>
+      <c r="AE43" t="n">
+        <v>62.97709923664122</v>
+      </c>
+      <c r="AF43" t="n">
+        <v>62.97709923664122</v>
+      </c>
       <c r="AG43" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -4251,7 +4417,9 @@
         </is>
       </c>
       <c r="AN43" t="inlineStr"/>
-      <c r="AO43" t="inlineStr"/>
+      <c r="AO43" t="n">
+        <v>62.97709923664122</v>
+      </c>
       <c r="AP43" t="inlineStr"/>
       <c r="AQ43" t="inlineStr"/>
       <c r="AR43" t="inlineStr">
@@ -4390,9 +4558,15 @@
       <c r="AA45" t="inlineStr"/>
       <c r="AB45" t="inlineStr"/>
       <c r="AC45" t="inlineStr"/>
-      <c r="AD45" t="inlineStr"/>
-      <c r="AE45" t="inlineStr"/>
-      <c r="AF45" t="inlineStr"/>
+      <c r="AD45" t="n">
+        <v>62.23230490018149</v>
+      </c>
+      <c r="AE45" t="n">
+        <v>62.23230490018149</v>
+      </c>
+      <c r="AF45" t="n">
+        <v>62.23230490018149</v>
+      </c>
       <c r="AG45" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -4421,7 +4595,9 @@
         </is>
       </c>
       <c r="AN45" t="inlineStr"/>
-      <c r="AO45" t="inlineStr"/>
+      <c r="AO45" t="n">
+        <v>62.23230490018149</v>
+      </c>
       <c r="AP45" t="inlineStr"/>
       <c r="AQ45" t="inlineStr"/>
       <c r="AR45" t="inlineStr">
@@ -4560,9 +4736,15 @@
       <c r="AA47" t="inlineStr"/>
       <c r="AB47" t="inlineStr"/>
       <c r="AC47" t="inlineStr"/>
-      <c r="AD47" t="inlineStr"/>
-      <c r="AE47" t="inlineStr"/>
-      <c r="AF47" t="inlineStr"/>
+      <c r="AD47" t="n">
+        <v>63.41637010676158</v>
+      </c>
+      <c r="AE47" t="n">
+        <v>63.41637010676158</v>
+      </c>
+      <c r="AF47" t="n">
+        <v>63.41637010676158</v>
+      </c>
       <c r="AG47" t="inlineStr">
         <is>
           <t>13/10/2025</t>
@@ -4591,7 +4773,9 @@
         </is>
       </c>
       <c r="AN47" t="inlineStr"/>
-      <c r="AO47" t="inlineStr"/>
+      <c r="AO47" t="n">
+        <v>63.41637010676158</v>
+      </c>
       <c r="AP47" t="inlineStr"/>
       <c r="AQ47" t="inlineStr"/>
       <c r="AR47" t="inlineStr">
@@ -4730,9 +4914,15 @@
       <c r="AA49" t="inlineStr"/>
       <c r="AB49" t="inlineStr"/>
       <c r="AC49" t="inlineStr"/>
-      <c r="AD49" t="inlineStr"/>
-      <c r="AE49" t="inlineStr"/>
-      <c r="AF49" t="inlineStr"/>
+      <c r="AD49" t="n">
+        <v>59.63190184049079</v>
+      </c>
+      <c r="AE49" t="n">
+        <v>59.63190184049079</v>
+      </c>
+      <c r="AF49" t="n">
+        <v>59.63190184049079</v>
+      </c>
       <c r="AG49" t="inlineStr">
         <is>
           <t>13/10/2025</t>
@@ -4761,7 +4951,9 @@
         </is>
       </c>
       <c r="AN49" t="inlineStr"/>
-      <c r="AO49" t="inlineStr"/>
+      <c r="AO49" t="n">
+        <v>59.63190184049079</v>
+      </c>
       <c r="AP49" t="inlineStr"/>
       <c r="AQ49" t="inlineStr"/>
       <c r="AR49" t="inlineStr">
@@ -4900,9 +5092,15 @@
       <c r="AA51" t="inlineStr"/>
       <c r="AB51" t="inlineStr"/>
       <c r="AC51" t="inlineStr"/>
-      <c r="AD51" t="inlineStr"/>
-      <c r="AE51" t="inlineStr"/>
-      <c r="AF51" t="inlineStr"/>
+      <c r="AD51" t="n">
+        <v>62.1195652173913</v>
+      </c>
+      <c r="AE51" t="n">
+        <v>62.1195652173913</v>
+      </c>
+      <c r="AF51" t="n">
+        <v>62.1195652173913</v>
+      </c>
       <c r="AG51" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -4931,7 +5129,9 @@
         </is>
       </c>
       <c r="AN51" t="inlineStr"/>
-      <c r="AO51" t="inlineStr"/>
+      <c r="AO51" t="n">
+        <v>62.1195652173913</v>
+      </c>
       <c r="AP51" t="inlineStr"/>
       <c r="AQ51" t="inlineStr"/>
       <c r="AR51" t="inlineStr">
@@ -5070,9 +5270,15 @@
       <c r="AA53" t="inlineStr"/>
       <c r="AB53" t="inlineStr"/>
       <c r="AC53" t="inlineStr"/>
-      <c r="AD53" t="inlineStr"/>
-      <c r="AE53" t="inlineStr"/>
-      <c r="AF53" t="inlineStr"/>
+      <c r="AD53" t="n">
+        <v>62.048392442824</v>
+      </c>
+      <c r="AE53" t="n">
+        <v>62.048392442824</v>
+      </c>
+      <c r="AF53" t="n">
+        <v>62.048392442824</v>
+      </c>
       <c r="AG53" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -5101,7 +5307,9 @@
         </is>
       </c>
       <c r="AN53" t="inlineStr"/>
-      <c r="AO53" t="inlineStr"/>
+      <c r="AO53" t="n">
+        <v>62.048392442824</v>
+      </c>
       <c r="AP53" t="inlineStr"/>
       <c r="AQ53" t="inlineStr"/>
       <c r="AR53" t="inlineStr">
@@ -5240,9 +5448,15 @@
       <c r="AA55" t="inlineStr"/>
       <c r="AB55" t="inlineStr"/>
       <c r="AC55" t="inlineStr"/>
-      <c r="AD55" t="inlineStr"/>
-      <c r="AE55" t="inlineStr"/>
-      <c r="AF55" t="inlineStr"/>
+      <c r="AD55" t="n">
+        <v>61.63977609483042</v>
+      </c>
+      <c r="AE55" t="n">
+        <v>61.63977609483042</v>
+      </c>
+      <c r="AF55" t="n">
+        <v>61.63977609483042</v>
+      </c>
       <c r="AG55" t="inlineStr">
         <is>
           <t>29/10/2025</t>
@@ -5271,7 +5485,9 @@
         </is>
       </c>
       <c r="AN55" t="inlineStr"/>
-      <c r="AO55" t="inlineStr"/>
+      <c r="AO55" t="n">
+        <v>61.63977609483042</v>
+      </c>
       <c r="AP55" t="inlineStr"/>
       <c r="AQ55" t="inlineStr"/>
       <c r="AR55" t="inlineStr">
@@ -5410,9 +5626,15 @@
       <c r="AA57" t="inlineStr"/>
       <c r="AB57" t="inlineStr"/>
       <c r="AC57" t="inlineStr"/>
-      <c r="AD57" t="inlineStr"/>
-      <c r="AE57" t="inlineStr"/>
-      <c r="AF57" t="inlineStr"/>
+      <c r="AD57" t="n">
+        <v>62.17203586848224</v>
+      </c>
+      <c r="AE57" t="n">
+        <v>62.17203586848224</v>
+      </c>
+      <c r="AF57" t="n">
+        <v>62.17203586848224</v>
+      </c>
       <c r="AG57" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -5441,7 +5663,9 @@
         </is>
       </c>
       <c r="AN57" t="inlineStr"/>
-      <c r="AO57" t="inlineStr"/>
+      <c r="AO57" t="n">
+        <v>62.17203586848224</v>
+      </c>
       <c r="AP57" t="inlineStr"/>
       <c r="AQ57" t="inlineStr"/>
       <c r="AR57" t="inlineStr">
@@ -5580,9 +5804,15 @@
       <c r="AA59" t="inlineStr"/>
       <c r="AB59" t="inlineStr"/>
       <c r="AC59" t="inlineStr"/>
-      <c r="AD59" t="inlineStr"/>
-      <c r="AE59" t="inlineStr"/>
-      <c r="AF59" t="inlineStr"/>
+      <c r="AD59" t="n">
+        <v>61.75596578117965</v>
+      </c>
+      <c r="AE59" t="n">
+        <v>61.75596578117965</v>
+      </c>
+      <c r="AF59" t="n">
+        <v>61.75596578117965</v>
+      </c>
       <c r="AG59" t="inlineStr">
         <is>
           <t>8/10/2025</t>
@@ -5611,7 +5841,9 @@
         </is>
       </c>
       <c r="AN59" t="inlineStr"/>
-      <c r="AO59" t="inlineStr"/>
+      <c r="AO59" t="n">
+        <v>61.75596578117965</v>
+      </c>
       <c r="AP59" t="inlineStr"/>
       <c r="AQ59" t="inlineStr"/>
       <c r="AR59" t="inlineStr">
@@ -5750,9 +5982,15 @@
       <c r="AA61" t="inlineStr"/>
       <c r="AB61" t="inlineStr"/>
       <c r="AC61" t="inlineStr"/>
-      <c r="AD61" t="inlineStr"/>
-      <c r="AE61" t="inlineStr"/>
-      <c r="AF61" t="inlineStr"/>
+      <c r="AD61" t="n">
+        <v>62.23404255319149</v>
+      </c>
+      <c r="AE61" t="n">
+        <v>62.23404255319149</v>
+      </c>
+      <c r="AF61" t="n">
+        <v>62.23404255319149</v>
+      </c>
       <c r="AG61" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -5781,7 +6019,9 @@
         </is>
       </c>
       <c r="AN61" t="inlineStr"/>
-      <c r="AO61" t="inlineStr"/>
+      <c r="AO61" t="n">
+        <v>62.23404255319149</v>
+      </c>
       <c r="AP61" t="inlineStr"/>
       <c r="AQ61" t="inlineStr"/>
       <c r="AR61" t="inlineStr">
@@ -5920,9 +6160,15 @@
       <c r="AA63" t="inlineStr"/>
       <c r="AB63" t="inlineStr"/>
       <c r="AC63" t="inlineStr"/>
-      <c r="AD63" t="inlineStr"/>
-      <c r="AE63" t="inlineStr"/>
-      <c r="AF63" t="inlineStr"/>
+      <c r="AD63" t="n">
+        <v>64.34316353887401</v>
+      </c>
+      <c r="AE63" t="n">
+        <v>64.34316353887401</v>
+      </c>
+      <c r="AF63" t="n">
+        <v>64.34316353887401</v>
+      </c>
       <c r="AG63" t="inlineStr">
         <is>
           <t>4/11/2025</t>
@@ -5951,7 +6197,9 @@
         </is>
       </c>
       <c r="AN63" t="inlineStr"/>
-      <c r="AO63" t="inlineStr"/>
+      <c r="AO63" t="n">
+        <v>64.34316353887401</v>
+      </c>
       <c r="AP63" t="inlineStr"/>
       <c r="AQ63" t="inlineStr"/>
       <c r="AR63" t="inlineStr">
@@ -6090,9 +6338,15 @@
       <c r="AA65" t="inlineStr"/>
       <c r="AB65" t="inlineStr"/>
       <c r="AC65" t="inlineStr"/>
-      <c r="AD65" t="inlineStr"/>
-      <c r="AE65" t="inlineStr"/>
-      <c r="AF65" t="inlineStr"/>
+      <c r="AD65" t="n">
+        <v>62.68738574040219</v>
+      </c>
+      <c r="AE65" t="n">
+        <v>62.68738574040219</v>
+      </c>
+      <c r="AF65" t="n">
+        <v>62.68738574040219</v>
+      </c>
       <c r="AG65" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -6121,7 +6375,9 @@
         </is>
       </c>
       <c r="AN65" t="inlineStr"/>
-      <c r="AO65" t="inlineStr"/>
+      <c r="AO65" t="n">
+        <v>62.68738574040219</v>
+      </c>
       <c r="AP65" t="inlineStr"/>
       <c r="AQ65" t="inlineStr"/>
       <c r="AR65" t="inlineStr">
@@ -6260,9 +6516,15 @@
       <c r="AA67" t="inlineStr"/>
       <c r="AB67" t="inlineStr"/>
       <c r="AC67" t="inlineStr"/>
-      <c r="AD67" t="inlineStr"/>
-      <c r="AE67" t="inlineStr"/>
-      <c r="AF67" t="inlineStr"/>
+      <c r="AD67" t="n">
+        <v>60.92307692307693</v>
+      </c>
+      <c r="AE67" t="n">
+        <v>60.92307692307693</v>
+      </c>
+      <c r="AF67" t="n">
+        <v>60.92307692307693</v>
+      </c>
       <c r="AG67" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -6291,7 +6553,9 @@
         </is>
       </c>
       <c r="AN67" t="inlineStr"/>
-      <c r="AO67" t="inlineStr"/>
+      <c r="AO67" t="n">
+        <v>60.92307692307693</v>
+      </c>
       <c r="AP67" t="inlineStr"/>
       <c r="AQ67" t="inlineStr"/>
       <c r="AR67" t="inlineStr">
@@ -6430,9 +6694,15 @@
       <c r="AA69" t="inlineStr"/>
       <c r="AB69" t="inlineStr"/>
       <c r="AC69" t="inlineStr"/>
-      <c r="AD69" t="inlineStr"/>
-      <c r="AE69" t="inlineStr"/>
-      <c r="AF69" t="inlineStr"/>
+      <c r="AD69" t="n">
+        <v>62.90956749672346</v>
+      </c>
+      <c r="AE69" t="n">
+        <v>62.90956749672346</v>
+      </c>
+      <c r="AF69" t="n">
+        <v>62.90956749672346</v>
+      </c>
       <c r="AG69" t="inlineStr">
         <is>
           <t>3/11/2025</t>
@@ -6461,7 +6731,9 @@
         </is>
       </c>
       <c r="AN69" t="inlineStr"/>
-      <c r="AO69" t="inlineStr"/>
+      <c r="AO69" t="n">
+        <v>62.90956749672346</v>
+      </c>
       <c r="AP69" t="inlineStr"/>
       <c r="AQ69" t="inlineStr"/>
       <c r="AR69" t="inlineStr">
@@ -6600,9 +6872,15 @@
       <c r="AA71" t="inlineStr"/>
       <c r="AB71" t="inlineStr"/>
       <c r="AC71" t="inlineStr"/>
-      <c r="AD71" t="inlineStr"/>
-      <c r="AE71" t="inlineStr"/>
-      <c r="AF71" t="inlineStr"/>
+      <c r="AD71" t="n">
+        <v>60.92307692307693</v>
+      </c>
+      <c r="AE71" t="n">
+        <v>60.92307692307693</v>
+      </c>
+      <c r="AF71" t="n">
+        <v>60.92307692307693</v>
+      </c>
       <c r="AG71" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -6631,7 +6909,9 @@
         </is>
       </c>
       <c r="AN71" t="inlineStr"/>
-      <c r="AO71" t="inlineStr"/>
+      <c r="AO71" t="n">
+        <v>60.92307692307693</v>
+      </c>
       <c r="AP71" t="inlineStr"/>
       <c r="AQ71" t="inlineStr"/>
       <c r="AR71" t="inlineStr">
@@ -6707,9 +6987,15 @@
       <c r="AA72" t="inlineStr"/>
       <c r="AB72" t="inlineStr"/>
       <c r="AC72" t="inlineStr"/>
-      <c r="AD72" t="inlineStr"/>
-      <c r="AE72" t="inlineStr"/>
-      <c r="AF72" t="inlineStr"/>
+      <c r="AD72" t="n">
+        <v>62.1195652173913</v>
+      </c>
+      <c r="AE72" t="n">
+        <v>62.1195652173913</v>
+      </c>
+      <c r="AF72" t="n">
+        <v>62.1195652173913</v>
+      </c>
       <c r="AG72" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -6738,7 +7024,9 @@
         </is>
       </c>
       <c r="AN72" t="inlineStr"/>
-      <c r="AO72" t="inlineStr"/>
+      <c r="AO72" t="n">
+        <v>62.1195652173913</v>
+      </c>
       <c r="AP72" t="inlineStr"/>
       <c r="AQ72" t="inlineStr"/>
       <c r="AR72" t="inlineStr">
@@ -6814,9 +7102,15 @@
       <c r="AA73" t="inlineStr"/>
       <c r="AB73" t="inlineStr"/>
       <c r="AC73" t="inlineStr"/>
-      <c r="AD73" t="inlineStr"/>
-      <c r="AE73" t="inlineStr"/>
-      <c r="AF73" t="inlineStr"/>
+      <c r="AD73" t="n">
+        <v>62.048392442824</v>
+      </c>
+      <c r="AE73" t="n">
+        <v>62.048392442824</v>
+      </c>
+      <c r="AF73" t="n">
+        <v>62.048392442824</v>
+      </c>
       <c r="AG73" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -6845,7 +7139,9 @@
         </is>
       </c>
       <c r="AN73" t="inlineStr"/>
-      <c r="AO73" t="inlineStr"/>
+      <c r="AO73" t="n">
+        <v>62.048392442824</v>
+      </c>
       <c r="AP73" t="inlineStr"/>
       <c r="AQ73" t="inlineStr"/>
       <c r="AR73" t="inlineStr">
@@ -6921,9 +7217,15 @@
       <c r="AA74" t="inlineStr"/>
       <c r="AB74" t="inlineStr"/>
       <c r="AC74" t="inlineStr"/>
-      <c r="AD74" t="inlineStr"/>
-      <c r="AE74" t="inlineStr"/>
-      <c r="AF74" t="inlineStr"/>
+      <c r="AD74" t="n">
+        <v>62.048392442824</v>
+      </c>
+      <c r="AE74" t="n">
+        <v>62.048392442824</v>
+      </c>
+      <c r="AF74" t="n">
+        <v>62.048392442824</v>
+      </c>
       <c r="AG74" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -6952,7 +7254,9 @@
         </is>
       </c>
       <c r="AN74" t="inlineStr"/>
-      <c r="AO74" t="inlineStr"/>
+      <c r="AO74" t="n">
+        <v>62.048392442824</v>
+      </c>
       <c r="AP74" t="inlineStr"/>
       <c r="AQ74" t="inlineStr"/>
       <c r="AR74" t="inlineStr">
@@ -7091,9 +7395,15 @@
       <c r="AA76" t="inlineStr"/>
       <c r="AB76" t="inlineStr"/>
       <c r="AC76" t="inlineStr"/>
-      <c r="AD76" t="inlineStr"/>
-      <c r="AE76" t="inlineStr"/>
-      <c r="AF76" t="inlineStr"/>
+      <c r="AD76" t="n">
+        <v>62.17203586848224</v>
+      </c>
+      <c r="AE76" t="n">
+        <v>62.17203586848224</v>
+      </c>
+      <c r="AF76" t="n">
+        <v>62.17203586848224</v>
+      </c>
       <c r="AG76" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -7122,7 +7432,9 @@
         </is>
       </c>
       <c r="AN76" t="inlineStr"/>
-      <c r="AO76" t="inlineStr"/>
+      <c r="AO76" t="n">
+        <v>62.17203586848224</v>
+      </c>
       <c r="AP76" t="inlineStr"/>
       <c r="AQ76" t="inlineStr"/>
       <c r="AR76" t="inlineStr">
@@ -7261,9 +7573,15 @@
       <c r="AA78" t="inlineStr"/>
       <c r="AB78" t="inlineStr"/>
       <c r="AC78" t="inlineStr"/>
-      <c r="AD78" t="inlineStr"/>
-      <c r="AE78" t="inlineStr"/>
-      <c r="AF78" t="inlineStr"/>
+      <c r="AD78" t="n">
+        <v>62.74473924977127</v>
+      </c>
+      <c r="AE78" t="n">
+        <v>62.74473924977127</v>
+      </c>
+      <c r="AF78" t="n">
+        <v>62.74473924977127</v>
+      </c>
       <c r="AG78" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -7292,7 +7610,9 @@
         </is>
       </c>
       <c r="AN78" t="inlineStr"/>
-      <c r="AO78" t="inlineStr"/>
+      <c r="AO78" t="n">
+        <v>62.74473924977127</v>
+      </c>
       <c r="AP78" t="inlineStr"/>
       <c r="AQ78" t="inlineStr"/>
       <c r="AR78" t="inlineStr">
@@ -7431,9 +7751,15 @@
       <c r="AA80" t="inlineStr"/>
       <c r="AB80" t="inlineStr"/>
       <c r="AC80" t="inlineStr"/>
-      <c r="AD80" t="inlineStr"/>
-      <c r="AE80" t="inlineStr"/>
-      <c r="AF80" t="inlineStr"/>
+      <c r="AD80" t="n">
+        <v>62.882096069869</v>
+      </c>
+      <c r="AE80" t="n">
+        <v>62.882096069869</v>
+      </c>
+      <c r="AF80" t="n">
+        <v>62.882096069869</v>
+      </c>
       <c r="AG80" t="inlineStr">
         <is>
           <t>1/11/2025</t>
@@ -7462,7 +7788,9 @@
         </is>
       </c>
       <c r="AN80" t="inlineStr"/>
-      <c r="AO80" t="inlineStr"/>
+      <c r="AO80" t="n">
+        <v>62.882096069869</v>
+      </c>
       <c r="AP80" t="inlineStr"/>
       <c r="AQ80" t="inlineStr"/>
       <c r="AR80" t="inlineStr">
@@ -7601,9 +7929,15 @@
       <c r="AA82" t="inlineStr"/>
       <c r="AB82" t="inlineStr"/>
       <c r="AC82" t="inlineStr"/>
-      <c r="AD82" t="inlineStr"/>
-      <c r="AE82" t="inlineStr"/>
-      <c r="AF82" t="inlineStr"/>
+      <c r="AD82" t="n">
+        <v>62.9004076878276</v>
+      </c>
+      <c r="AE82" t="n">
+        <v>62.9004076878276</v>
+      </c>
+      <c r="AF82" t="n">
+        <v>62.9004076878276</v>
+      </c>
       <c r="AG82" t="inlineStr">
         <is>
           <t>30/10/2025</t>
@@ -7632,7 +7966,9 @@
         </is>
       </c>
       <c r="AN82" t="inlineStr"/>
-      <c r="AO82" t="inlineStr"/>
+      <c r="AO82" t="n">
+        <v>62.9004076878276</v>
+      </c>
       <c r="AP82" t="inlineStr"/>
       <c r="AQ82" t="inlineStr"/>
       <c r="AR82" t="inlineStr">
@@ -7771,9 +8107,15 @@
       <c r="AA84" t="inlineStr"/>
       <c r="AB84" t="inlineStr"/>
       <c r="AC84" t="inlineStr"/>
-      <c r="AD84" t="inlineStr"/>
-      <c r="AE84" t="inlineStr"/>
-      <c r="AF84" t="inlineStr"/>
+      <c r="AD84" t="n">
+        <v>60.69895769466586</v>
+      </c>
+      <c r="AE84" t="n">
+        <v>60.69895769466586</v>
+      </c>
+      <c r="AF84" t="n">
+        <v>60.69895769466586</v>
+      </c>
       <c r="AG84" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -7802,7 +8144,9 @@
         </is>
       </c>
       <c r="AN84" t="inlineStr"/>
-      <c r="AO84" t="inlineStr"/>
+      <c r="AO84" t="n">
+        <v>60.69895769466586</v>
+      </c>
       <c r="AP84" t="inlineStr"/>
       <c r="AQ84" t="inlineStr"/>
       <c r="AR84" t="inlineStr">
@@ -7941,9 +8285,15 @@
       <c r="AA86" t="inlineStr"/>
       <c r="AB86" t="inlineStr"/>
       <c r="AC86" t="inlineStr"/>
-      <c r="AD86" t="inlineStr"/>
-      <c r="AE86" t="inlineStr"/>
-      <c r="AF86" t="inlineStr"/>
+      <c r="AD86" t="n">
+        <v>60.69895769466586</v>
+      </c>
+      <c r="AE86" t="n">
+        <v>60.69895769466586</v>
+      </c>
+      <c r="AF86" t="n">
+        <v>60.69895769466586</v>
+      </c>
       <c r="AG86" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -7972,7 +8322,9 @@
         </is>
       </c>
       <c r="AN86" t="inlineStr"/>
-      <c r="AO86" t="inlineStr"/>
+      <c r="AO86" t="n">
+        <v>60.69895769466586</v>
+      </c>
       <c r="AP86" t="inlineStr"/>
       <c r="AQ86" t="inlineStr"/>
       <c r="AR86" t="inlineStr">
@@ -8111,9 +8463,15 @@
       <c r="AA88" t="inlineStr"/>
       <c r="AB88" t="inlineStr"/>
       <c r="AC88" t="inlineStr"/>
-      <c r="AD88" t="inlineStr"/>
-      <c r="AE88" t="inlineStr"/>
-      <c r="AF88" t="inlineStr"/>
+      <c r="AD88" t="n">
+        <v>61.51898734177216</v>
+      </c>
+      <c r="AE88" t="n">
+        <v>61.51898734177216</v>
+      </c>
+      <c r="AF88" t="n">
+        <v>61.51898734177216</v>
+      </c>
       <c r="AG88" t="inlineStr">
         <is>
           <t>15/09/2025</t>
@@ -8142,7 +8500,9 @@
         </is>
       </c>
       <c r="AN88" t="inlineStr"/>
-      <c r="AO88" t="inlineStr"/>
+      <c r="AO88" t="n">
+        <v>61.51898734177216</v>
+      </c>
       <c r="AP88" t="inlineStr"/>
       <c r="AQ88" t="inlineStr"/>
       <c r="AR88" t="inlineStr">
@@ -8281,9 +8641,15 @@
       <c r="AA90" t="inlineStr"/>
       <c r="AB90" t="inlineStr"/>
       <c r="AC90" t="inlineStr"/>
-      <c r="AD90" t="inlineStr"/>
-      <c r="AE90" t="inlineStr"/>
-      <c r="AF90" t="inlineStr"/>
+      <c r="AD90" t="n">
+        <v>62.97709923664122</v>
+      </c>
+      <c r="AE90" t="n">
+        <v>62.97709923664122</v>
+      </c>
+      <c r="AF90" t="n">
+        <v>62.97709923664122</v>
+      </c>
       <c r="AG90" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -8312,7 +8678,9 @@
         </is>
       </c>
       <c r="AN90" t="inlineStr"/>
-      <c r="AO90" t="inlineStr"/>
+      <c r="AO90" t="n">
+        <v>62.97709923664122</v>
+      </c>
       <c r="AP90" t="inlineStr"/>
       <c r="AQ90" t="inlineStr"/>
       <c r="AR90" t="inlineStr">
@@ -8451,9 +8819,15 @@
       <c r="AA92" t="inlineStr"/>
       <c r="AB92" t="inlineStr"/>
       <c r="AC92" t="inlineStr"/>
-      <c r="AD92" t="inlineStr"/>
-      <c r="AE92" t="inlineStr"/>
-      <c r="AF92" t="inlineStr"/>
+      <c r="AD92" t="n">
+        <v>63.94316163410302</v>
+      </c>
+      <c r="AE92" t="n">
+        <v>63.94316163410302</v>
+      </c>
+      <c r="AF92" t="n">
+        <v>63.94316163410302</v>
+      </c>
       <c r="AG92" t="inlineStr">
         <is>
           <t>28/10/2025</t>
@@ -8482,7 +8856,9 @@
         </is>
       </c>
       <c r="AN92" t="inlineStr"/>
-      <c r="AO92" t="inlineStr"/>
+      <c r="AO92" t="n">
+        <v>63.94316163410302</v>
+      </c>
       <c r="AP92" t="inlineStr"/>
       <c r="AQ92" t="inlineStr"/>
       <c r="AR92" t="inlineStr">
@@ -8621,9 +8997,15 @@
       <c r="AA94" t="inlineStr"/>
       <c r="AB94" t="inlineStr"/>
       <c r="AC94" t="inlineStr"/>
-      <c r="AD94" t="inlineStr"/>
-      <c r="AE94" t="inlineStr"/>
-      <c r="AF94" t="inlineStr"/>
+      <c r="AD94" t="n">
+        <v>63.43612334801763</v>
+      </c>
+      <c r="AE94" t="n">
+        <v>63.43612334801763</v>
+      </c>
+      <c r="AF94" t="n">
+        <v>63.43612334801763</v>
+      </c>
       <c r="AG94" t="inlineStr">
         <is>
           <t>4/11/2025</t>
@@ -8652,7 +9034,9 @@
         </is>
       </c>
       <c r="AN94" t="inlineStr"/>
-      <c r="AO94" t="inlineStr"/>
+      <c r="AO94" t="n">
+        <v>63.43612334801763</v>
+      </c>
       <c r="AP94" t="inlineStr"/>
       <c r="AQ94" t="inlineStr"/>
       <c r="AR94" t="inlineStr">
@@ -8791,9 +9175,15 @@
       <c r="AA96" t="inlineStr"/>
       <c r="AB96" t="inlineStr"/>
       <c r="AC96" t="inlineStr"/>
-      <c r="AD96" t="inlineStr"/>
-      <c r="AE96" t="inlineStr"/>
-      <c r="AF96" t="inlineStr"/>
+      <c r="AD96" t="n">
+        <v>61.94573130377233</v>
+      </c>
+      <c r="AE96" t="n">
+        <v>61.94573130377233</v>
+      </c>
+      <c r="AF96" t="n">
+        <v>61.94573130377233</v>
+      </c>
       <c r="AG96" t="inlineStr">
         <is>
           <t>8/11/2025</t>
@@ -8822,7 +9212,9 @@
         </is>
       </c>
       <c r="AN96" t="inlineStr"/>
-      <c r="AO96" t="inlineStr"/>
+      <c r="AO96" t="n">
+        <v>61.94573130377233</v>
+      </c>
       <c r="AP96" t="inlineStr"/>
       <c r="AQ96" t="inlineStr"/>
       <c r="AR96" t="inlineStr">
@@ -8961,9 +9353,15 @@
       <c r="AA98" t="inlineStr"/>
       <c r="AB98" t="inlineStr"/>
       <c r="AC98" t="inlineStr"/>
-      <c r="AD98" t="inlineStr"/>
-      <c r="AE98" t="inlineStr"/>
-      <c r="AF98" t="inlineStr"/>
+      <c r="AD98" t="n">
+        <v>63.10344827586208</v>
+      </c>
+      <c r="AE98" t="n">
+        <v>63.10344827586208</v>
+      </c>
+      <c r="AF98" t="n">
+        <v>63.10344827586208</v>
+      </c>
       <c r="AG98" t="inlineStr">
         <is>
           <t>4/11/2025</t>
@@ -8992,7 +9390,9 @@
         </is>
       </c>
       <c r="AN98" t="inlineStr"/>
-      <c r="AO98" t="inlineStr"/>
+      <c r="AO98" t="n">
+        <v>63.10344827586208</v>
+      </c>
       <c r="AP98" t="inlineStr"/>
       <c r="AQ98" t="inlineStr"/>
       <c r="AR98" t="inlineStr">
@@ -9131,9 +9531,15 @@
       <c r="AA100" t="inlineStr"/>
       <c r="AB100" t="inlineStr"/>
       <c r="AC100" t="inlineStr"/>
-      <c r="AD100" t="inlineStr"/>
-      <c r="AE100" t="inlineStr"/>
-      <c r="AF100" t="inlineStr"/>
+      <c r="AD100" t="n">
+        <v>62.17203586848224</v>
+      </c>
+      <c r="AE100" t="n">
+        <v>62.17203586848224</v>
+      </c>
+      <c r="AF100" t="n">
+        <v>62.17203586848224</v>
+      </c>
       <c r="AG100" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -9162,7 +9568,9 @@
         </is>
       </c>
       <c r="AN100" t="inlineStr"/>
-      <c r="AO100" t="inlineStr"/>
+      <c r="AO100" t="n">
+        <v>62.17203586848224</v>
+      </c>
       <c r="AP100" t="inlineStr"/>
       <c r="AQ100" t="inlineStr"/>
       <c r="AR100" t="inlineStr">
@@ -9301,9 +9709,15 @@
       <c r="AA102" t="inlineStr"/>
       <c r="AB102" t="inlineStr"/>
       <c r="AC102" t="inlineStr"/>
-      <c r="AD102" t="inlineStr"/>
-      <c r="AE102" t="inlineStr"/>
-      <c r="AF102" t="inlineStr"/>
+      <c r="AD102" t="n">
+        <v>63.74455732946299</v>
+      </c>
+      <c r="AE102" t="n">
+        <v>63.74455732946299</v>
+      </c>
+      <c r="AF102" t="n">
+        <v>63.74455732946299</v>
+      </c>
       <c r="AG102" t="inlineStr">
         <is>
           <t>31/10/2025</t>
@@ -9332,7 +9746,9 @@
         </is>
       </c>
       <c r="AN102" t="inlineStr"/>
-      <c r="AO102" t="inlineStr"/>
+      <c r="AO102" t="n">
+        <v>63.74455732946299</v>
+      </c>
       <c r="AP102" t="inlineStr"/>
       <c r="AQ102" t="inlineStr"/>
       <c r="AR102" t="inlineStr">
@@ -9471,9 +9887,15 @@
       <c r="AA104" t="inlineStr"/>
       <c r="AB104" t="inlineStr"/>
       <c r="AC104" t="inlineStr"/>
-      <c r="AD104" t="inlineStr"/>
-      <c r="AE104" t="inlineStr"/>
-      <c r="AF104" t="inlineStr"/>
+      <c r="AD104" t="n">
+        <v>64.02845709204091</v>
+      </c>
+      <c r="AE104" t="n">
+        <v>64.02845709204091</v>
+      </c>
+      <c r="AF104" t="n">
+        <v>64.02845709204091</v>
+      </c>
       <c r="AG104" t="inlineStr">
         <is>
           <t>31/10/2025</t>
@@ -9502,7 +9924,9 @@
         </is>
       </c>
       <c r="AN104" t="inlineStr"/>
-      <c r="AO104" t="inlineStr"/>
+      <c r="AO104" t="n">
+        <v>64.02845709204091</v>
+      </c>
       <c r="AP104" t="inlineStr"/>
       <c r="AQ104" t="inlineStr"/>
       <c r="AR104" t="inlineStr">
@@ -9641,9 +10065,15 @@
       <c r="AA106" t="inlineStr"/>
       <c r="AB106" t="inlineStr"/>
       <c r="AC106" t="inlineStr"/>
-      <c r="AD106" t="inlineStr"/>
-      <c r="AE106" t="inlineStr"/>
-      <c r="AF106" t="inlineStr"/>
+      <c r="AD106" t="n">
+        <v>63.82978723404256</v>
+      </c>
+      <c r="AE106" t="n">
+        <v>63.82978723404256</v>
+      </c>
+      <c r="AF106" t="n">
+        <v>63.82978723404256</v>
+      </c>
       <c r="AG106" t="inlineStr">
         <is>
           <t>30/10/2025</t>
@@ -9672,7 +10102,9 @@
         </is>
       </c>
       <c r="AN106" t="inlineStr"/>
-      <c r="AO106" t="inlineStr"/>
+      <c r="AO106" t="n">
+        <v>63.82978723404256</v>
+      </c>
       <c r="AP106" t="inlineStr"/>
       <c r="AQ106" t="inlineStr"/>
       <c r="AR106" t="inlineStr">
@@ -9811,9 +10243,15 @@
       <c r="AA108" t="inlineStr"/>
       <c r="AB108" t="inlineStr"/>
       <c r="AC108" t="inlineStr"/>
-      <c r="AD108" t="inlineStr"/>
-      <c r="AE108" t="inlineStr"/>
-      <c r="AF108" t="inlineStr"/>
+      <c r="AD108" t="n">
+        <v>61.59327731092437</v>
+      </c>
+      <c r="AE108" t="n">
+        <v>61.59327731092437</v>
+      </c>
+      <c r="AF108" t="n">
+        <v>61.59327731092437</v>
+      </c>
       <c r="AG108" t="inlineStr">
         <is>
           <t>6/10/2025</t>
@@ -9842,7 +10280,9 @@
         </is>
       </c>
       <c r="AN108" t="inlineStr"/>
-      <c r="AO108" t="inlineStr"/>
+      <c r="AO108" t="n">
+        <v>61.59327731092437</v>
+      </c>
       <c r="AP108" t="inlineStr"/>
       <c r="AQ108" t="inlineStr"/>
       <c r="AR108" t="inlineStr">
@@ -9981,9 +10421,15 @@
       <c r="AA110" t="inlineStr"/>
       <c r="AB110" t="inlineStr"/>
       <c r="AC110" t="inlineStr"/>
-      <c r="AD110" t="inlineStr"/>
-      <c r="AE110" t="inlineStr"/>
-      <c r="AF110" t="inlineStr"/>
+      <c r="AD110" t="n">
+        <v>62.23230490018149</v>
+      </c>
+      <c r="AE110" t="n">
+        <v>62.23230490018149</v>
+      </c>
+      <c r="AF110" t="n">
+        <v>62.23230490018149</v>
+      </c>
       <c r="AG110" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -10012,7 +10458,9 @@
         </is>
       </c>
       <c r="AN110" t="inlineStr"/>
-      <c r="AO110" t="inlineStr"/>
+      <c r="AO110" t="n">
+        <v>62.23230490018149</v>
+      </c>
       <c r="AP110" t="inlineStr"/>
       <c r="AQ110" t="inlineStr"/>
       <c r="AR110" t="inlineStr">
@@ -10151,9 +10599,15 @@
       <c r="AA112" t="inlineStr"/>
       <c r="AB112" t="inlineStr"/>
       <c r="AC112" t="inlineStr"/>
-      <c r="AD112" t="inlineStr"/>
-      <c r="AE112" t="inlineStr"/>
-      <c r="AF112" t="inlineStr"/>
+      <c r="AD112" t="n">
+        <v>63.75442739079102</v>
+      </c>
+      <c r="AE112" t="n">
+        <v>63.75442739079102</v>
+      </c>
+      <c r="AF112" t="n">
+        <v>63.75442739079102</v>
+      </c>
       <c r="AG112" t="inlineStr">
         <is>
           <t>6/11/2025</t>
@@ -10182,7 +10636,9 @@
         </is>
       </c>
       <c r="AN112" t="inlineStr"/>
-      <c r="AO112" t="inlineStr"/>
+      <c r="AO112" t="n">
+        <v>63.75442739079102</v>
+      </c>
       <c r="AP112" t="inlineStr"/>
       <c r="AQ112" t="inlineStr"/>
       <c r="AR112" t="inlineStr">
@@ -10321,9 +10777,15 @@
       <c r="AA114" t="inlineStr"/>
       <c r="AB114" t="inlineStr"/>
       <c r="AC114" t="inlineStr"/>
-      <c r="AD114" t="inlineStr"/>
-      <c r="AE114" t="inlineStr"/>
-      <c r="AF114" t="inlineStr"/>
+      <c r="AD114" t="n">
+        <v>62.60869565217391</v>
+      </c>
+      <c r="AE114" t="n">
+        <v>62.60869565217391</v>
+      </c>
+      <c r="AF114" t="n">
+        <v>62.60869565217391</v>
+      </c>
       <c r="AG114" t="inlineStr">
         <is>
           <t>31/10/2025</t>
@@ -10352,7 +10814,9 @@
         </is>
       </c>
       <c r="AN114" t="inlineStr"/>
-      <c r="AO114" t="inlineStr"/>
+      <c r="AO114" t="n">
+        <v>62.60869565217391</v>
+      </c>
       <c r="AP114" t="inlineStr"/>
       <c r="AQ114" t="inlineStr"/>
       <c r="AR114" t="inlineStr">
@@ -10566,9 +11030,15 @@
       <c r="AA117" t="inlineStr"/>
       <c r="AB117" t="inlineStr"/>
       <c r="AC117" t="inlineStr"/>
-      <c r="AD117" t="inlineStr"/>
-      <c r="AE117" t="inlineStr"/>
-      <c r="AF117" t="inlineStr"/>
+      <c r="AD117" t="n">
+        <v>62.048392442824</v>
+      </c>
+      <c r="AE117" t="n">
+        <v>62.048392442824</v>
+      </c>
+      <c r="AF117" t="n">
+        <v>62.048392442824</v>
+      </c>
       <c r="AG117" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -10597,7 +11067,9 @@
         </is>
       </c>
       <c r="AN117" t="inlineStr"/>
-      <c r="AO117" t="inlineStr"/>
+      <c r="AO117" t="n">
+        <v>62.048392442824</v>
+      </c>
       <c r="AP117" t="inlineStr"/>
       <c r="AQ117" t="inlineStr"/>
       <c r="AR117" t="inlineStr">
@@ -10673,9 +11145,15 @@
       <c r="AA118" t="inlineStr"/>
       <c r="AB118" t="inlineStr"/>
       <c r="AC118" t="inlineStr"/>
-      <c r="AD118" t="inlineStr"/>
-      <c r="AE118" t="inlineStr"/>
-      <c r="AF118" t="inlineStr"/>
+      <c r="AD118" t="n">
+        <v>62.048392442824</v>
+      </c>
+      <c r="AE118" t="n">
+        <v>62.048392442824</v>
+      </c>
+      <c r="AF118" t="n">
+        <v>62.048392442824</v>
+      </c>
       <c r="AG118" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -10704,7 +11182,9 @@
         </is>
       </c>
       <c r="AN118" t="inlineStr"/>
-      <c r="AO118" t="inlineStr"/>
+      <c r="AO118" t="n">
+        <v>62.048392442824</v>
+      </c>
       <c r="AP118" t="inlineStr"/>
       <c r="AQ118" t="inlineStr"/>
       <c r="AR118" t="inlineStr">
@@ -10843,9 +11323,15 @@
       <c r="AA120" t="inlineStr"/>
       <c r="AB120" t="inlineStr"/>
       <c r="AC120" t="inlineStr"/>
-      <c r="AD120" t="inlineStr"/>
-      <c r="AE120" t="inlineStr"/>
-      <c r="AF120" t="inlineStr"/>
+      <c r="AD120" t="n">
+        <v>62.17203586848224</v>
+      </c>
+      <c r="AE120" t="n">
+        <v>62.17203586848224</v>
+      </c>
+      <c r="AF120" t="n">
+        <v>62.17203586848224</v>
+      </c>
       <c r="AG120" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -10874,7 +11360,9 @@
         </is>
       </c>
       <c r="AN120" t="inlineStr"/>
-      <c r="AO120" t="inlineStr"/>
+      <c r="AO120" t="n">
+        <v>62.17203586848224</v>
+      </c>
       <c r="AP120" t="inlineStr"/>
       <c r="AQ120" t="inlineStr"/>
       <c r="AR120" t="inlineStr">
@@ -11013,9 +11501,15 @@
       <c r="AA122" t="inlineStr"/>
       <c r="AB122" t="inlineStr"/>
       <c r="AC122" t="inlineStr"/>
-      <c r="AD122" t="inlineStr"/>
-      <c r="AE122" t="inlineStr"/>
-      <c r="AF122" t="inlineStr"/>
+      <c r="AD122" t="n">
+        <v>61.83949504057711</v>
+      </c>
+      <c r="AE122" t="n">
+        <v>61.83949504057711</v>
+      </c>
+      <c r="AF122" t="n">
+        <v>61.83949504057711</v>
+      </c>
       <c r="AG122" t="inlineStr">
         <is>
           <t>22/10/2025</t>
@@ -11044,7 +11538,9 @@
         </is>
       </c>
       <c r="AN122" t="inlineStr"/>
-      <c r="AO122" t="inlineStr"/>
+      <c r="AO122" t="n">
+        <v>61.83949504057711</v>
+      </c>
       <c r="AP122" t="inlineStr"/>
       <c r="AQ122" t="inlineStr"/>
       <c r="AR122" t="inlineStr">
@@ -11183,9 +11679,15 @@
       <c r="AA124" t="inlineStr"/>
       <c r="AB124" t="inlineStr"/>
       <c r="AC124" t="inlineStr"/>
-      <c r="AD124" t="inlineStr"/>
-      <c r="AE124" t="inlineStr"/>
-      <c r="AF124" t="inlineStr"/>
+      <c r="AD124" t="n">
+        <v>62.23404255319149</v>
+      </c>
+      <c r="AE124" t="n">
+        <v>62.23404255319149</v>
+      </c>
+      <c r="AF124" t="n">
+        <v>62.23404255319149</v>
+      </c>
       <c r="AG124" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -11214,7 +11716,9 @@
         </is>
       </c>
       <c r="AN124" t="inlineStr"/>
-      <c r="AO124" t="inlineStr"/>
+      <c r="AO124" t="n">
+        <v>62.23404255319149</v>
+      </c>
       <c r="AP124" t="inlineStr"/>
       <c r="AQ124" t="inlineStr"/>
       <c r="AR124" t="inlineStr">
@@ -11353,9 +11857,15 @@
       <c r="AA126" t="inlineStr"/>
       <c r="AB126" t="inlineStr"/>
       <c r="AC126" t="inlineStr"/>
-      <c r="AD126" t="inlineStr"/>
-      <c r="AE126" t="inlineStr"/>
-      <c r="AF126" t="inlineStr"/>
+      <c r="AD126" t="n">
+        <v>62.97709923664122</v>
+      </c>
+      <c r="AE126" t="n">
+        <v>62.97709923664122</v>
+      </c>
+      <c r="AF126" t="n">
+        <v>62.97709923664122</v>
+      </c>
       <c r="AG126" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -11384,7 +11894,9 @@
         </is>
       </c>
       <c r="AN126" t="inlineStr"/>
-      <c r="AO126" t="inlineStr"/>
+      <c r="AO126" t="n">
+        <v>62.97709923664122</v>
+      </c>
       <c r="AP126" t="inlineStr"/>
       <c r="AQ126" t="inlineStr"/>
       <c r="AR126" t="inlineStr">
@@ -11523,9 +12035,15 @@
       <c r="AA128" t="inlineStr"/>
       <c r="AB128" t="inlineStr"/>
       <c r="AC128" t="inlineStr"/>
-      <c r="AD128" t="inlineStr"/>
-      <c r="AE128" t="inlineStr"/>
-      <c r="AF128" t="inlineStr"/>
+      <c r="AD128" t="n">
+        <v>62.8021978021978</v>
+      </c>
+      <c r="AE128" t="n">
+        <v>62.8021978021978</v>
+      </c>
+      <c r="AF128" t="n">
+        <v>62.8021978021978</v>
+      </c>
       <c r="AG128" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -11554,7 +12072,9 @@
         </is>
       </c>
       <c r="AN128" t="inlineStr"/>
-      <c r="AO128" t="inlineStr"/>
+      <c r="AO128" t="n">
+        <v>62.8021978021978</v>
+      </c>
       <c r="AP128" t="inlineStr"/>
       <c r="AQ128" t="inlineStr"/>
       <c r="AR128" t="inlineStr">
@@ -11693,9 +12213,15 @@
       <c r="AA130" t="inlineStr"/>
       <c r="AB130" t="inlineStr"/>
       <c r="AC130" t="inlineStr"/>
-      <c r="AD130" t="inlineStr"/>
-      <c r="AE130" t="inlineStr"/>
-      <c r="AF130" t="inlineStr"/>
+      <c r="AD130" t="n">
+        <v>61.56716417910449</v>
+      </c>
+      <c r="AE130" t="n">
+        <v>61.56716417910449</v>
+      </c>
+      <c r="AF130" t="n">
+        <v>61.56716417910449</v>
+      </c>
       <c r="AG130" t="inlineStr">
         <is>
           <t>8/10/2025</t>
@@ -11724,7 +12250,9 @@
         </is>
       </c>
       <c r="AN130" t="inlineStr"/>
-      <c r="AO130" t="inlineStr"/>
+      <c r="AO130" t="n">
+        <v>61.56716417910449</v>
+      </c>
       <c r="AP130" t="inlineStr"/>
       <c r="AQ130" t="inlineStr"/>
       <c r="AR130" t="inlineStr">
@@ -11863,9 +12391,15 @@
       <c r="AA132" t="inlineStr"/>
       <c r="AB132" t="inlineStr"/>
       <c r="AC132" t="inlineStr"/>
-      <c r="AD132" t="inlineStr"/>
-      <c r="AE132" t="inlineStr"/>
-      <c r="AF132" t="inlineStr"/>
+      <c r="AD132" t="n">
+        <v>62.8021978021978</v>
+      </c>
+      <c r="AE132" t="n">
+        <v>62.8021978021978</v>
+      </c>
+      <c r="AF132" t="n">
+        <v>62.8021978021978</v>
+      </c>
       <c r="AG132" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -11894,7 +12428,9 @@
         </is>
       </c>
       <c r="AN132" t="inlineStr"/>
-      <c r="AO132" t="inlineStr"/>
+      <c r="AO132" t="n">
+        <v>62.8021978021978</v>
+      </c>
       <c r="AP132" t="inlineStr"/>
       <c r="AQ132" t="inlineStr"/>
       <c r="AR132" t="inlineStr">
@@ -12033,9 +12569,15 @@
       <c r="AA134" t="inlineStr"/>
       <c r="AB134" t="inlineStr"/>
       <c r="AC134" t="inlineStr"/>
-      <c r="AD134" t="inlineStr"/>
-      <c r="AE134" t="inlineStr"/>
-      <c r="AF134" t="inlineStr"/>
+      <c r="AD134" t="n">
+        <v>61.52889993784959</v>
+      </c>
+      <c r="AE134" t="n">
+        <v>61.52889993784959</v>
+      </c>
+      <c r="AF134" t="n">
+        <v>61.52889993784959</v>
+      </c>
       <c r="AG134" t="inlineStr">
         <is>
           <t>29/10/2025</t>
@@ -12064,7 +12606,9 @@
         </is>
       </c>
       <c r="AN134" t="inlineStr"/>
-      <c r="AO134" t="inlineStr"/>
+      <c r="AO134" t="n">
+        <v>61.52889993784959</v>
+      </c>
       <c r="AP134" t="inlineStr"/>
       <c r="AQ134" t="inlineStr"/>
       <c r="AR134" t="inlineStr">
@@ -12203,9 +12747,15 @@
       <c r="AA136" t="inlineStr"/>
       <c r="AB136" t="inlineStr"/>
       <c r="AC136" t="inlineStr"/>
-      <c r="AD136" t="inlineStr"/>
-      <c r="AE136" t="inlineStr"/>
-      <c r="AF136" t="inlineStr"/>
+      <c r="AD136" t="n">
+        <v>61.84340931615461</v>
+      </c>
+      <c r="AE136" t="n">
+        <v>61.84340931615461</v>
+      </c>
+      <c r="AF136" t="n">
+        <v>61.84340931615461</v>
+      </c>
       <c r="AG136" t="inlineStr">
         <is>
           <t>10/09/2025</t>
@@ -12234,7 +12784,9 @@
         </is>
       </c>
       <c r="AN136" t="inlineStr"/>
-      <c r="AO136" t="inlineStr"/>
+      <c r="AO136" t="n">
+        <v>61.84340931615461</v>
+      </c>
       <c r="AP136" t="inlineStr"/>
       <c r="AQ136" t="inlineStr"/>
       <c r="AR136" t="inlineStr">
@@ -12649,9 +13201,15 @@
       <c r="AA142" t="inlineStr"/>
       <c r="AB142" t="inlineStr"/>
       <c r="AC142" t="inlineStr"/>
-      <c r="AD142" t="inlineStr"/>
-      <c r="AE142" t="inlineStr"/>
-      <c r="AF142" t="inlineStr"/>
+      <c r="AD142" t="n">
+        <v>62.048392442824</v>
+      </c>
+      <c r="AE142" t="n">
+        <v>62.048392442824</v>
+      </c>
+      <c r="AF142" t="n">
+        <v>62.048392442824</v>
+      </c>
       <c r="AG142" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -12680,7 +13238,9 @@
         </is>
       </c>
       <c r="AN142" t="inlineStr"/>
-      <c r="AO142" t="inlineStr"/>
+      <c r="AO142" t="n">
+        <v>62.048392442824</v>
+      </c>
       <c r="AP142" t="inlineStr"/>
       <c r="AQ142" t="inlineStr"/>
       <c r="AR142" t="inlineStr">
@@ -12819,9 +13379,15 @@
       <c r="AA144" t="inlineStr"/>
       <c r="AB144" t="inlineStr"/>
       <c r="AC144" t="inlineStr"/>
-      <c r="AD144" t="inlineStr"/>
-      <c r="AE144" t="inlineStr"/>
-      <c r="AF144" t="inlineStr"/>
+      <c r="AD144" t="n">
+        <v>62.74473924977127</v>
+      </c>
+      <c r="AE144" t="n">
+        <v>62.74473924977127</v>
+      </c>
+      <c r="AF144" t="n">
+        <v>62.74473924977127</v>
+      </c>
       <c r="AG144" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -12850,7 +13416,9 @@
         </is>
       </c>
       <c r="AN144" t="inlineStr"/>
-      <c r="AO144" t="inlineStr"/>
+      <c r="AO144" t="n">
+        <v>62.74473924977127</v>
+      </c>
       <c r="AP144" t="inlineStr"/>
       <c r="AQ144" t="inlineStr"/>
       <c r="AR144" t="inlineStr">
@@ -12989,9 +13557,15 @@
       <c r="AA146" t="inlineStr"/>
       <c r="AB146" t="inlineStr"/>
       <c r="AC146" t="inlineStr"/>
-      <c r="AD146" t="inlineStr"/>
-      <c r="AE146" t="inlineStr"/>
-      <c r="AF146" t="inlineStr"/>
+      <c r="AD146" t="n">
+        <v>62.23404255319149</v>
+      </c>
+      <c r="AE146" t="n">
+        <v>62.23404255319149</v>
+      </c>
+      <c r="AF146" t="n">
+        <v>62.23404255319149</v>
+      </c>
       <c r="AG146" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -13020,7 +13594,9 @@
         </is>
       </c>
       <c r="AN146" t="inlineStr"/>
-      <c r="AO146" t="inlineStr"/>
+      <c r="AO146" t="n">
+        <v>62.23404255319149</v>
+      </c>
       <c r="AP146" t="inlineStr"/>
       <c r="AQ146" t="inlineStr"/>
       <c r="AR146" t="inlineStr">
@@ -13159,9 +13735,15 @@
       <c r="AA148" t="inlineStr"/>
       <c r="AB148" t="inlineStr"/>
       <c r="AC148" t="inlineStr"/>
-      <c r="AD148" t="inlineStr"/>
-      <c r="AE148" t="inlineStr"/>
-      <c r="AF148" t="inlineStr"/>
+      <c r="AD148" t="n">
+        <v>63.06206896551724</v>
+      </c>
+      <c r="AE148" t="n">
+        <v>63.06206896551724</v>
+      </c>
+      <c r="AF148" t="n">
+        <v>63.06206896551724</v>
+      </c>
       <c r="AG148" t="inlineStr">
         <is>
           <t>29/10/2025</t>
@@ -13190,7 +13772,9 @@
         </is>
       </c>
       <c r="AN148" t="inlineStr"/>
-      <c r="AO148" t="inlineStr"/>
+      <c r="AO148" t="n">
+        <v>63.06206896551724</v>
+      </c>
       <c r="AP148" t="inlineStr"/>
       <c r="AQ148" t="inlineStr"/>
       <c r="AR148" t="inlineStr">
@@ -13329,9 +13913,15 @@
       <c r="AA150" t="inlineStr"/>
       <c r="AB150" t="inlineStr"/>
       <c r="AC150" t="inlineStr"/>
-      <c r="AD150" t="inlineStr"/>
-      <c r="AE150" t="inlineStr"/>
-      <c r="AF150" t="inlineStr"/>
+      <c r="AD150" t="n">
+        <v>62.23230490018149</v>
+      </c>
+      <c r="AE150" t="n">
+        <v>62.23230490018149</v>
+      </c>
+      <c r="AF150" t="n">
+        <v>62.23230490018149</v>
+      </c>
       <c r="AG150" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -13360,7 +13950,9 @@
         </is>
       </c>
       <c r="AN150" t="inlineStr"/>
-      <c r="AO150" t="inlineStr"/>
+      <c r="AO150" t="n">
+        <v>62.23230490018149</v>
+      </c>
       <c r="AP150" t="inlineStr"/>
       <c r="AQ150" t="inlineStr"/>
       <c r="AR150" t="inlineStr">
@@ -13499,9 +14091,15 @@
       <c r="AA152" t="inlineStr"/>
       <c r="AB152" t="inlineStr"/>
       <c r="AC152" t="inlineStr"/>
-      <c r="AD152" t="inlineStr"/>
-      <c r="AE152" t="inlineStr"/>
-      <c r="AF152" t="inlineStr"/>
+      <c r="AD152" t="n">
+        <v>60.88560885608856</v>
+      </c>
+      <c r="AE152" t="n">
+        <v>60.88560885608856</v>
+      </c>
+      <c r="AF152" t="n">
+        <v>60.88560885608856</v>
+      </c>
       <c r="AG152" t="inlineStr">
         <is>
           <t>29/10/2025</t>
@@ -13530,7 +14128,9 @@
         </is>
       </c>
       <c r="AN152" t="inlineStr"/>
-      <c r="AO152" t="inlineStr"/>
+      <c r="AO152" t="n">
+        <v>60.88560885608856</v>
+      </c>
       <c r="AP152" t="inlineStr"/>
       <c r="AQ152" t="inlineStr"/>
       <c r="AR152" t="inlineStr">
@@ -13669,9 +14269,15 @@
       <c r="AA154" t="inlineStr"/>
       <c r="AB154" t="inlineStr"/>
       <c r="AC154" t="inlineStr"/>
-      <c r="AD154" t="inlineStr"/>
-      <c r="AE154" t="inlineStr"/>
-      <c r="AF154" t="inlineStr"/>
+      <c r="AD154" t="n">
+        <v>62.8021978021978</v>
+      </c>
+      <c r="AE154" t="n">
+        <v>62.8021978021978</v>
+      </c>
+      <c r="AF154" t="n">
+        <v>62.8021978021978</v>
+      </c>
       <c r="AG154" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -13700,7 +14306,9 @@
         </is>
       </c>
       <c r="AN154" t="inlineStr"/>
-      <c r="AO154" t="inlineStr"/>
+      <c r="AO154" t="n">
+        <v>62.8021978021978</v>
+      </c>
       <c r="AP154" t="inlineStr"/>
       <c r="AQ154" t="inlineStr"/>
       <c r="AR154" t="inlineStr">
@@ -13839,9 +14447,15 @@
       <c r="AA156" t="inlineStr"/>
       <c r="AB156" t="inlineStr"/>
       <c r="AC156" t="inlineStr"/>
-      <c r="AD156" t="inlineStr"/>
-      <c r="AE156" t="inlineStr"/>
-      <c r="AF156" t="inlineStr"/>
+      <c r="AD156" t="n">
+        <v>62.46056782334384</v>
+      </c>
+      <c r="AE156" t="n">
+        <v>62.46056782334384</v>
+      </c>
+      <c r="AF156" t="n">
+        <v>62.46056782334384</v>
+      </c>
       <c r="AG156" t="inlineStr">
         <is>
           <t>22/10/2025</t>
@@ -13870,7 +14484,9 @@
         </is>
       </c>
       <c r="AN156" t="inlineStr"/>
-      <c r="AO156" t="inlineStr"/>
+      <c r="AO156" t="n">
+        <v>62.46056782334384</v>
+      </c>
       <c r="AP156" t="inlineStr"/>
       <c r="AQ156" t="inlineStr"/>
       <c r="AR156" t="inlineStr">
@@ -14009,9 +14625,15 @@
       <c r="AA158" t="inlineStr"/>
       <c r="AB158" t="inlineStr"/>
       <c r="AC158" t="inlineStr"/>
-      <c r="AD158" t="inlineStr"/>
-      <c r="AE158" t="inlineStr"/>
-      <c r="AF158" t="inlineStr"/>
+      <c r="AD158" t="n">
+        <v>60.69895769466586</v>
+      </c>
+      <c r="AE158" t="n">
+        <v>60.69895769466586</v>
+      </c>
+      <c r="AF158" t="n">
+        <v>60.69895769466586</v>
+      </c>
       <c r="AG158" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -14040,7 +14662,9 @@
         </is>
       </c>
       <c r="AN158" t="inlineStr"/>
-      <c r="AO158" t="inlineStr"/>
+      <c r="AO158" t="n">
+        <v>60.69895769466586</v>
+      </c>
       <c r="AP158" t="inlineStr"/>
       <c r="AQ158" t="inlineStr"/>
       <c r="AR158" t="inlineStr">
@@ -14179,9 +14803,15 @@
       <c r="AA160" t="inlineStr"/>
       <c r="AB160" t="inlineStr"/>
       <c r="AC160" t="inlineStr"/>
-      <c r="AD160" t="inlineStr"/>
-      <c r="AE160" t="inlineStr"/>
-      <c r="AF160" t="inlineStr"/>
+      <c r="AD160" t="n">
+        <v>62.52713851498045</v>
+      </c>
+      <c r="AE160" t="n">
+        <v>62.52713851498045</v>
+      </c>
+      <c r="AF160" t="n">
+        <v>62.52713851498045</v>
+      </c>
       <c r="AG160" t="inlineStr">
         <is>
           <t>28/10/2025</t>
@@ -14210,7 +14840,9 @@
         </is>
       </c>
       <c r="AN160" t="inlineStr"/>
-      <c r="AO160" t="inlineStr"/>
+      <c r="AO160" t="n">
+        <v>62.52713851498045</v>
+      </c>
       <c r="AP160" t="inlineStr"/>
       <c r="AQ160" t="inlineStr"/>
       <c r="AR160" t="inlineStr">
@@ -14349,9 +14981,15 @@
       <c r="AA162" t="inlineStr"/>
       <c r="AB162" t="inlineStr"/>
       <c r="AC162" t="inlineStr"/>
-      <c r="AD162" t="inlineStr"/>
-      <c r="AE162" t="inlineStr"/>
-      <c r="AF162" t="inlineStr"/>
+      <c r="AD162" t="n">
+        <v>62.28882833787466</v>
+      </c>
+      <c r="AE162" t="n">
+        <v>62.28882833787466</v>
+      </c>
+      <c r="AF162" t="n">
+        <v>62.28882833787466</v>
+      </c>
       <c r="AG162" t="inlineStr">
         <is>
           <t>17/09/2025</t>
@@ -14380,7 +15018,9 @@
         </is>
       </c>
       <c r="AN162" t="inlineStr"/>
-      <c r="AO162" t="inlineStr"/>
+      <c r="AO162" t="n">
+        <v>62.28882833787466</v>
+      </c>
       <c r="AP162" t="inlineStr"/>
       <c r="AQ162" t="inlineStr"/>
       <c r="AR162" t="inlineStr">
@@ -14657,9 +15297,15 @@
       <c r="AA166" t="inlineStr"/>
       <c r="AB166" t="inlineStr"/>
       <c r="AC166" t="inlineStr"/>
-      <c r="AD166" t="inlineStr"/>
-      <c r="AE166" t="inlineStr"/>
-      <c r="AF166" t="inlineStr"/>
+      <c r="AD166" t="n">
+        <v>62.17203586848224</v>
+      </c>
+      <c r="AE166" t="n">
+        <v>62.17203586848224</v>
+      </c>
+      <c r="AF166" t="n">
+        <v>62.17203586848224</v>
+      </c>
       <c r="AG166" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -14688,7 +15334,9 @@
         </is>
       </c>
       <c r="AN166" t="inlineStr"/>
-      <c r="AO166" t="inlineStr"/>
+      <c r="AO166" t="n">
+        <v>62.17203586848224</v>
+      </c>
       <c r="AP166" t="inlineStr"/>
       <c r="AQ166" t="inlineStr"/>
       <c r="AR166" t="inlineStr">
@@ -14827,9 +15475,15 @@
       <c r="AA168" t="inlineStr"/>
       <c r="AB168" t="inlineStr"/>
       <c r="AC168" t="inlineStr"/>
-      <c r="AD168" t="inlineStr"/>
-      <c r="AE168" t="inlineStr"/>
-      <c r="AF168" t="inlineStr"/>
+      <c r="AD168" t="n">
+        <v>62.74473924977127</v>
+      </c>
+      <c r="AE168" t="n">
+        <v>62.74473924977127</v>
+      </c>
+      <c r="AF168" t="n">
+        <v>62.74473924977127</v>
+      </c>
       <c r="AG168" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -14858,7 +15512,9 @@
         </is>
       </c>
       <c r="AN168" t="inlineStr"/>
-      <c r="AO168" t="inlineStr"/>
+      <c r="AO168" t="n">
+        <v>62.74473924977127</v>
+      </c>
       <c r="AP168" t="inlineStr"/>
       <c r="AQ168" t="inlineStr"/>
       <c r="AR168" t="inlineStr">
@@ -14997,9 +15653,15 @@
       <c r="AA170" t="inlineStr"/>
       <c r="AB170" t="inlineStr"/>
       <c r="AC170" t="inlineStr"/>
-      <c r="AD170" t="inlineStr"/>
-      <c r="AE170" t="inlineStr"/>
-      <c r="AF170" t="inlineStr"/>
+      <c r="AD170" t="n">
+        <v>62.17203586848224</v>
+      </c>
+      <c r="AE170" t="n">
+        <v>62.17203586848224</v>
+      </c>
+      <c r="AF170" t="n">
+        <v>62.17203586848224</v>
+      </c>
       <c r="AG170" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -15028,7 +15690,9 @@
         </is>
       </c>
       <c r="AN170" t="inlineStr"/>
-      <c r="AO170" t="inlineStr"/>
+      <c r="AO170" t="n">
+        <v>62.17203586848224</v>
+      </c>
       <c r="AP170" t="inlineStr"/>
       <c r="AQ170" t="inlineStr"/>
       <c r="AR170" t="inlineStr">
@@ -15167,9 +15831,15 @@
       <c r="AA172" t="inlineStr"/>
       <c r="AB172" t="inlineStr"/>
       <c r="AC172" t="inlineStr"/>
-      <c r="AD172" t="inlineStr"/>
-      <c r="AE172" t="inlineStr"/>
-      <c r="AF172" t="inlineStr"/>
+      <c r="AD172" t="n">
+        <v>61.8392134181608</v>
+      </c>
+      <c r="AE172" t="n">
+        <v>61.8392134181608</v>
+      </c>
+      <c r="AF172" t="n">
+        <v>61.8392134181608</v>
+      </c>
       <c r="AG172" t="inlineStr">
         <is>
           <t>6/10/2025</t>
@@ -15198,7 +15868,9 @@
         </is>
       </c>
       <c r="AN172" t="inlineStr"/>
-      <c r="AO172" t="inlineStr"/>
+      <c r="AO172" t="n">
+        <v>61.8392134181608</v>
+      </c>
       <c r="AP172" t="inlineStr"/>
       <c r="AQ172" t="inlineStr"/>
       <c r="AR172" t="inlineStr">
@@ -15337,9 +16009,15 @@
       <c r="AA174" t="inlineStr"/>
       <c r="AB174" t="inlineStr"/>
       <c r="AC174" t="inlineStr"/>
-      <c r="AD174" t="inlineStr"/>
-      <c r="AE174" t="inlineStr"/>
-      <c r="AF174" t="inlineStr"/>
+      <c r="AD174" t="n">
+        <v>62.8021978021978</v>
+      </c>
+      <c r="AE174" t="n">
+        <v>62.8021978021978</v>
+      </c>
+      <c r="AF174" t="n">
+        <v>62.8021978021978</v>
+      </c>
       <c r="AG174" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -15368,7 +16046,9 @@
         </is>
       </c>
       <c r="AN174" t="inlineStr"/>
-      <c r="AO174" t="inlineStr"/>
+      <c r="AO174" t="n">
+        <v>62.8021978021978</v>
+      </c>
       <c r="AP174" t="inlineStr"/>
       <c r="AQ174" t="inlineStr"/>
       <c r="AR174" t="inlineStr">
@@ -15507,9 +16187,15 @@
       <c r="AA176" t="inlineStr"/>
       <c r="AB176" t="inlineStr"/>
       <c r="AC176" t="inlineStr"/>
-      <c r="AD176" t="inlineStr"/>
-      <c r="AE176" t="inlineStr"/>
-      <c r="AF176" t="inlineStr"/>
+      <c r="AD176" t="n">
+        <v>63.82978723404256</v>
+      </c>
+      <c r="AE176" t="n">
+        <v>63.82978723404256</v>
+      </c>
+      <c r="AF176" t="n">
+        <v>63.82978723404256</v>
+      </c>
       <c r="AG176" t="inlineStr">
         <is>
           <t>30/10/2025</t>
@@ -15538,7 +16224,9 @@
         </is>
       </c>
       <c r="AN176" t="inlineStr"/>
-      <c r="AO176" t="inlineStr"/>
+      <c r="AO176" t="n">
+        <v>63.82978723404256</v>
+      </c>
       <c r="AP176" t="inlineStr"/>
       <c r="AQ176" t="inlineStr"/>
       <c r="AR176" t="inlineStr">
@@ -15677,9 +16365,15 @@
       <c r="AA178" t="inlineStr"/>
       <c r="AB178" t="inlineStr"/>
       <c r="AC178" t="inlineStr"/>
-      <c r="AD178" t="inlineStr"/>
-      <c r="AE178" t="inlineStr"/>
-      <c r="AF178" t="inlineStr"/>
+      <c r="AD178" t="n">
+        <v>62.68738574040219</v>
+      </c>
+      <c r="AE178" t="n">
+        <v>62.68738574040219</v>
+      </c>
+      <c r="AF178" t="n">
+        <v>62.68738574040219</v>
+      </c>
       <c r="AG178" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -15708,7 +16402,9 @@
         </is>
       </c>
       <c r="AN178" t="inlineStr"/>
-      <c r="AO178" t="inlineStr"/>
+      <c r="AO178" t="n">
+        <v>62.68738574040219</v>
+      </c>
       <c r="AP178" t="inlineStr"/>
       <c r="AQ178" t="inlineStr"/>
       <c r="AR178" t="inlineStr">
@@ -15847,9 +16543,15 @@
       <c r="AA180" t="inlineStr"/>
       <c r="AB180" t="inlineStr"/>
       <c r="AC180" t="inlineStr"/>
-      <c r="AD180" t="inlineStr"/>
-      <c r="AE180" t="inlineStr"/>
-      <c r="AF180" t="inlineStr"/>
+      <c r="AD180" t="n">
+        <v>62.97709923664122</v>
+      </c>
+      <c r="AE180" t="n">
+        <v>62.97709923664122</v>
+      </c>
+      <c r="AF180" t="n">
+        <v>62.97709923664122</v>
+      </c>
       <c r="AG180" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -15878,7 +16580,9 @@
         </is>
       </c>
       <c r="AN180" t="inlineStr"/>
-      <c r="AO180" t="inlineStr"/>
+      <c r="AO180" t="n">
+        <v>62.97709923664122</v>
+      </c>
       <c r="AP180" t="inlineStr"/>
       <c r="AQ180" t="inlineStr"/>
       <c r="AR180" t="inlineStr">
@@ -16017,9 +16721,15 @@
       <c r="AA182" t="inlineStr"/>
       <c r="AB182" t="inlineStr"/>
       <c r="AC182" t="inlineStr"/>
-      <c r="AD182" t="inlineStr"/>
-      <c r="AE182" t="inlineStr"/>
-      <c r="AF182" t="inlineStr"/>
+      <c r="AD182" t="n">
+        <v>62.10465784933871</v>
+      </c>
+      <c r="AE182" t="n">
+        <v>62.10465784933871</v>
+      </c>
+      <c r="AF182" t="n">
+        <v>62.10465784933871</v>
+      </c>
       <c r="AG182" t="inlineStr">
         <is>
           <t>3/11/2025</t>
@@ -16048,7 +16758,9 @@
         </is>
       </c>
       <c r="AN182" t="inlineStr"/>
-      <c r="AO182" t="inlineStr"/>
+      <c r="AO182" t="n">
+        <v>62.10465784933871</v>
+      </c>
       <c r="AP182" t="inlineStr"/>
       <c r="AQ182" t="inlineStr"/>
       <c r="AR182" t="inlineStr">
@@ -16124,9 +16836,15 @@
       <c r="AA183" t="inlineStr"/>
       <c r="AB183" t="inlineStr"/>
       <c r="AC183" t="inlineStr"/>
-      <c r="AD183" t="inlineStr"/>
-      <c r="AE183" t="inlineStr"/>
-      <c r="AF183" t="inlineStr"/>
+      <c r="AD183" t="n">
+        <v>62.1195652173913</v>
+      </c>
+      <c r="AE183" t="n">
+        <v>62.1195652173913</v>
+      </c>
+      <c r="AF183" t="n">
+        <v>62.1195652173913</v>
+      </c>
       <c r="AG183" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -16155,7 +16873,9 @@
         </is>
       </c>
       <c r="AN183" t="inlineStr"/>
-      <c r="AO183" t="inlineStr"/>
+      <c r="AO183" t="n">
+        <v>62.1195652173913</v>
+      </c>
       <c r="AP183" t="inlineStr"/>
       <c r="AQ183" t="inlineStr"/>
       <c r="AR183" t="inlineStr">
@@ -16294,9 +17014,15 @@
       <c r="AA185" t="inlineStr"/>
       <c r="AB185" t="inlineStr"/>
       <c r="AC185" t="inlineStr"/>
-      <c r="AD185" t="inlineStr"/>
-      <c r="AE185" t="inlineStr"/>
-      <c r="AF185" t="inlineStr"/>
+      <c r="AD185" t="n">
+        <v>61.94573130377233</v>
+      </c>
+      <c r="AE185" t="n">
+        <v>61.94573130377233</v>
+      </c>
+      <c r="AF185" t="n">
+        <v>61.94573130377233</v>
+      </c>
       <c r="AG185" t="inlineStr">
         <is>
           <t>8/11/2025</t>
@@ -16325,7 +17051,9 @@
         </is>
       </c>
       <c r="AN185" t="inlineStr"/>
-      <c r="AO185" t="inlineStr"/>
+      <c r="AO185" t="n">
+        <v>61.94573130377233</v>
+      </c>
       <c r="AP185" t="inlineStr"/>
       <c r="AQ185" t="inlineStr"/>
       <c r="AR185" t="inlineStr">
@@ -16464,9 +17192,15 @@
       <c r="AA187" t="inlineStr"/>
       <c r="AB187" t="inlineStr"/>
       <c r="AC187" t="inlineStr"/>
-      <c r="AD187" t="inlineStr"/>
-      <c r="AE187" t="inlineStr"/>
-      <c r="AF187" t="inlineStr"/>
+      <c r="AD187" t="n">
+        <v>62.1195652173913</v>
+      </c>
+      <c r="AE187" t="n">
+        <v>62.1195652173913</v>
+      </c>
+      <c r="AF187" t="n">
+        <v>62.1195652173913</v>
+      </c>
       <c r="AG187" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -16495,7 +17229,9 @@
         </is>
       </c>
       <c r="AN187" t="inlineStr"/>
-      <c r="AO187" t="inlineStr"/>
+      <c r="AO187" t="n">
+        <v>62.1195652173913</v>
+      </c>
       <c r="AP187" t="inlineStr"/>
       <c r="AQ187" t="inlineStr"/>
       <c r="AR187" t="inlineStr">
@@ -16634,9 +17370,15 @@
       <c r="AA189" t="inlineStr"/>
       <c r="AB189" t="inlineStr"/>
       <c r="AC189" t="inlineStr"/>
-      <c r="AD189" t="inlineStr"/>
-      <c r="AE189" t="inlineStr"/>
-      <c r="AF189" t="inlineStr"/>
+      <c r="AD189" t="n">
+        <v>62.1195652173913</v>
+      </c>
+      <c r="AE189" t="n">
+        <v>62.1195652173913</v>
+      </c>
+      <c r="AF189" t="n">
+        <v>62.1195652173913</v>
+      </c>
       <c r="AG189" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -16665,7 +17407,9 @@
         </is>
       </c>
       <c r="AN189" t="inlineStr"/>
-      <c r="AO189" t="inlineStr"/>
+      <c r="AO189" t="n">
+        <v>62.1195652173913</v>
+      </c>
       <c r="AP189" t="inlineStr"/>
       <c r="AQ189" t="inlineStr"/>
       <c r="AR189" t="inlineStr">
@@ -16804,9 +17548,15 @@
       <c r="AA191" t="inlineStr"/>
       <c r="AB191" t="inlineStr"/>
       <c r="AC191" t="inlineStr"/>
-      <c r="AD191" t="inlineStr"/>
-      <c r="AE191" t="inlineStr"/>
-      <c r="AF191" t="inlineStr"/>
+      <c r="AD191" t="n">
+        <v>61.78378378378378</v>
+      </c>
+      <c r="AE191" t="n">
+        <v>61.78378378378378</v>
+      </c>
+      <c r="AF191" t="n">
+        <v>61.78378378378378</v>
+      </c>
       <c r="AG191" t="inlineStr">
         <is>
           <t>8/11/2025</t>
@@ -16835,7 +17585,9 @@
         </is>
       </c>
       <c r="AN191" t="inlineStr"/>
-      <c r="AO191" t="inlineStr"/>
+      <c r="AO191" t="n">
+        <v>61.78378378378378</v>
+      </c>
       <c r="AP191" t="inlineStr"/>
       <c r="AQ191" t="inlineStr"/>
       <c r="AR191" t="inlineStr">
@@ -16974,9 +17726,15 @@
       <c r="AA193" t="inlineStr"/>
       <c r="AB193" t="inlineStr"/>
       <c r="AC193" t="inlineStr"/>
-      <c r="AD193" t="inlineStr"/>
-      <c r="AE193" t="inlineStr"/>
-      <c r="AF193" t="inlineStr"/>
+      <c r="AD193" t="n">
+        <v>63.74455732946299</v>
+      </c>
+      <c r="AE193" t="n">
+        <v>63.74455732946299</v>
+      </c>
+      <c r="AF193" t="n">
+        <v>63.74455732946299</v>
+      </c>
       <c r="AG193" t="inlineStr">
         <is>
           <t>7/11/2025</t>
@@ -17005,7 +17763,9 @@
         </is>
       </c>
       <c r="AN193" t="inlineStr"/>
-      <c r="AO193" t="inlineStr"/>
+      <c r="AO193" t="n">
+        <v>63.74455732946299</v>
+      </c>
       <c r="AP193" t="inlineStr"/>
       <c r="AQ193" t="inlineStr"/>
       <c r="AR193" t="inlineStr">
@@ -17144,9 +17904,15 @@
       <c r="AA195" t="inlineStr"/>
       <c r="AB195" t="inlineStr"/>
       <c r="AC195" t="inlineStr"/>
-      <c r="AD195" t="inlineStr"/>
-      <c r="AE195" t="inlineStr"/>
-      <c r="AF195" t="inlineStr"/>
+      <c r="AD195" t="n">
+        <v>62.68738574040219</v>
+      </c>
+      <c r="AE195" t="n">
+        <v>62.68738574040219</v>
+      </c>
+      <c r="AF195" t="n">
+        <v>62.68738574040219</v>
+      </c>
       <c r="AG195" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -17175,7 +17941,9 @@
         </is>
       </c>
       <c r="AN195" t="inlineStr"/>
-      <c r="AO195" t="inlineStr"/>
+      <c r="AO195" t="n">
+        <v>62.68738574040219</v>
+      </c>
       <c r="AP195" t="inlineStr"/>
       <c r="AQ195" t="inlineStr"/>
       <c r="AR195" t="inlineStr">
@@ -17314,9 +18082,15 @@
       <c r="AA197" t="inlineStr"/>
       <c r="AB197" t="inlineStr"/>
       <c r="AC197" t="inlineStr"/>
-      <c r="AD197" t="inlineStr"/>
-      <c r="AE197" t="inlineStr"/>
-      <c r="AF197" t="inlineStr"/>
+      <c r="AD197" t="n">
+        <v>62.23230490018149</v>
+      </c>
+      <c r="AE197" t="n">
+        <v>62.23230490018149</v>
+      </c>
+      <c r="AF197" t="n">
+        <v>62.23230490018149</v>
+      </c>
       <c r="AG197" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -17345,7 +18119,9 @@
         </is>
       </c>
       <c r="AN197" t="inlineStr"/>
-      <c r="AO197" t="inlineStr"/>
+      <c r="AO197" t="n">
+        <v>62.23230490018149</v>
+      </c>
       <c r="AP197" t="inlineStr"/>
       <c r="AQ197" t="inlineStr"/>
       <c r="AR197" t="inlineStr">
@@ -17484,9 +18260,15 @@
       <c r="AA199" t="inlineStr"/>
       <c r="AB199" t="inlineStr"/>
       <c r="AC199" t="inlineStr"/>
-      <c r="AD199" t="inlineStr"/>
-      <c r="AE199" t="inlineStr"/>
-      <c r="AF199" t="inlineStr"/>
+      <c r="AD199" t="n">
+        <v>61.08597285067874</v>
+      </c>
+      <c r="AE199" t="n">
+        <v>61.08597285067874</v>
+      </c>
+      <c r="AF199" t="n">
+        <v>61.08597285067874</v>
+      </c>
       <c r="AG199" t="inlineStr">
         <is>
           <t>3/11/2025</t>
@@ -17515,7 +18297,9 @@
         </is>
       </c>
       <c r="AN199" t="inlineStr"/>
-      <c r="AO199" t="inlineStr"/>
+      <c r="AO199" t="n">
+        <v>61.08597285067874</v>
+      </c>
       <c r="AP199" t="inlineStr"/>
       <c r="AQ199" t="inlineStr"/>
       <c r="AR199" t="inlineStr">
@@ -17654,9 +18438,15 @@
       <c r="AA201" t="inlineStr"/>
       <c r="AB201" t="inlineStr"/>
       <c r="AC201" t="inlineStr"/>
-      <c r="AD201" t="inlineStr"/>
-      <c r="AE201" t="inlineStr"/>
-      <c r="AF201" t="inlineStr"/>
+      <c r="AD201" t="n">
+        <v>62.1195652173913</v>
+      </c>
+      <c r="AE201" t="n">
+        <v>62.1195652173913</v>
+      </c>
+      <c r="AF201" t="n">
+        <v>62.1195652173913</v>
+      </c>
       <c r="AG201" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -17685,7 +18475,9 @@
         </is>
       </c>
       <c r="AN201" t="inlineStr"/>
-      <c r="AO201" t="inlineStr"/>
+      <c r="AO201" t="n">
+        <v>62.1195652173913</v>
+      </c>
       <c r="AP201" t="inlineStr"/>
       <c r="AQ201" t="inlineStr"/>
       <c r="AR201" t="inlineStr">
@@ -17761,9 +18553,15 @@
       <c r="AA202" t="inlineStr"/>
       <c r="AB202" t="inlineStr"/>
       <c r="AC202" t="inlineStr"/>
-      <c r="AD202" t="inlineStr"/>
-      <c r="AE202" t="inlineStr"/>
-      <c r="AF202" t="inlineStr"/>
+      <c r="AD202" t="n">
+        <v>62.1195652173913</v>
+      </c>
+      <c r="AE202" t="n">
+        <v>62.1195652173913</v>
+      </c>
+      <c r="AF202" t="n">
+        <v>62.1195652173913</v>
+      </c>
       <c r="AG202" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -17792,7 +18590,9 @@
         </is>
       </c>
       <c r="AN202" t="inlineStr"/>
-      <c r="AO202" t="inlineStr"/>
+      <c r="AO202" t="n">
+        <v>62.1195652173913</v>
+      </c>
       <c r="AP202" t="inlineStr"/>
       <c r="AQ202" t="inlineStr"/>
       <c r="AR202" t="inlineStr">
@@ -17931,9 +18731,15 @@
       <c r="AA204" t="inlineStr"/>
       <c r="AB204" t="inlineStr"/>
       <c r="AC204" t="inlineStr"/>
-      <c r="AD204" t="inlineStr"/>
-      <c r="AE204" t="inlineStr"/>
-      <c r="AF204" t="inlineStr"/>
+      <c r="AD204" t="n">
+        <v>61.94573130377233</v>
+      </c>
+      <c r="AE204" t="n">
+        <v>61.94573130377233</v>
+      </c>
+      <c r="AF204" t="n">
+        <v>61.94573130377233</v>
+      </c>
       <c r="AG204" t="inlineStr">
         <is>
           <t>8/11/2025</t>
@@ -17962,7 +18768,9 @@
         </is>
       </c>
       <c r="AN204" t="inlineStr"/>
-      <c r="AO204" t="inlineStr"/>
+      <c r="AO204" t="n">
+        <v>61.94573130377233</v>
+      </c>
       <c r="AP204" t="inlineStr"/>
       <c r="AQ204" t="inlineStr"/>
       <c r="AR204" t="inlineStr">
@@ -18101,9 +18909,15 @@
       <c r="AA206" t="inlineStr"/>
       <c r="AB206" t="inlineStr"/>
       <c r="AC206" t="inlineStr"/>
-      <c r="AD206" t="inlineStr"/>
-      <c r="AE206" t="inlineStr"/>
-      <c r="AF206" t="inlineStr"/>
+      <c r="AD206" t="n">
+        <v>62.74473924977127</v>
+      </c>
+      <c r="AE206" t="n">
+        <v>62.74473924977127</v>
+      </c>
+      <c r="AF206" t="n">
+        <v>62.74473924977127</v>
+      </c>
       <c r="AG206" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -18132,7 +18946,9 @@
         </is>
       </c>
       <c r="AN206" t="inlineStr"/>
-      <c r="AO206" t="inlineStr"/>
+      <c r="AO206" t="n">
+        <v>62.74473924977127</v>
+      </c>
       <c r="AP206" t="inlineStr"/>
       <c r="AQ206" t="inlineStr"/>
       <c r="AR206" t="inlineStr">
@@ -18271,9 +19087,15 @@
       <c r="AA208" t="inlineStr"/>
       <c r="AB208" t="inlineStr"/>
       <c r="AC208" t="inlineStr"/>
-      <c r="AD208" t="inlineStr"/>
-      <c r="AE208" t="inlineStr"/>
-      <c r="AF208" t="inlineStr"/>
+      <c r="AD208" t="n">
+        <v>64.02845709204091</v>
+      </c>
+      <c r="AE208" t="n">
+        <v>64.02845709204091</v>
+      </c>
+      <c r="AF208" t="n">
+        <v>64.02845709204091</v>
+      </c>
       <c r="AG208" t="inlineStr">
         <is>
           <t>10/10/2025</t>
@@ -18302,7 +19124,9 @@
         </is>
       </c>
       <c r="AN208" t="inlineStr"/>
-      <c r="AO208" t="inlineStr"/>
+      <c r="AO208" t="n">
+        <v>64.02845709204091</v>
+      </c>
       <c r="AP208" t="inlineStr"/>
       <c r="AQ208" t="inlineStr"/>
       <c r="AR208" t="inlineStr">
@@ -18441,9 +19265,15 @@
       <c r="AA210" t="inlineStr"/>
       <c r="AB210" t="inlineStr"/>
       <c r="AC210" t="inlineStr"/>
-      <c r="AD210" t="inlineStr"/>
-      <c r="AE210" t="inlineStr"/>
-      <c r="AF210" t="inlineStr"/>
+      <c r="AD210" t="n">
+        <v>62.96670030272453</v>
+      </c>
+      <c r="AE210" t="n">
+        <v>62.96670030272453</v>
+      </c>
+      <c r="AF210" t="n">
+        <v>62.96670030272453</v>
+      </c>
       <c r="AG210" t="inlineStr">
         <is>
           <t>1/11/2025</t>
@@ -18472,7 +19302,9 @@
         </is>
       </c>
       <c r="AN210" t="inlineStr"/>
-      <c r="AO210" t="inlineStr"/>
+      <c r="AO210" t="n">
+        <v>62.96670030272453</v>
+      </c>
       <c r="AP210" t="inlineStr"/>
       <c r="AQ210" t="inlineStr"/>
       <c r="AR210" t="inlineStr">
@@ -18611,9 +19443,15 @@
       <c r="AA212" t="inlineStr"/>
       <c r="AB212" t="inlineStr"/>
       <c r="AC212" t="inlineStr"/>
-      <c r="AD212" t="inlineStr"/>
-      <c r="AE212" t="inlineStr"/>
-      <c r="AF212" t="inlineStr"/>
+      <c r="AD212" t="n">
+        <v>62.68738574040219</v>
+      </c>
+      <c r="AE212" t="n">
+        <v>62.68738574040219</v>
+      </c>
+      <c r="AF212" t="n">
+        <v>62.68738574040219</v>
+      </c>
       <c r="AG212" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -18642,7 +19480,9 @@
         </is>
       </c>
       <c r="AN212" t="inlineStr"/>
-      <c r="AO212" t="inlineStr"/>
+      <c r="AO212" t="n">
+        <v>62.68738574040219</v>
+      </c>
       <c r="AP212" t="inlineStr"/>
       <c r="AQ212" t="inlineStr"/>
       <c r="AR212" t="inlineStr">
@@ -18781,9 +19621,15 @@
       <c r="AA214" t="inlineStr"/>
       <c r="AB214" t="inlineStr"/>
       <c r="AC214" t="inlineStr"/>
-      <c r="AD214" t="inlineStr"/>
-      <c r="AE214" t="inlineStr"/>
-      <c r="AF214" t="inlineStr"/>
+      <c r="AD214" t="n">
+        <v>62.23230490018149</v>
+      </c>
+      <c r="AE214" t="n">
+        <v>62.23230490018149</v>
+      </c>
+      <c r="AF214" t="n">
+        <v>62.23230490018149</v>
+      </c>
       <c r="AG214" t="inlineStr">
         <is>
           <t>5/11/2025</t>
@@ -18812,7 +19658,9 @@
         </is>
       </c>
       <c r="AN214" t="inlineStr"/>
-      <c r="AO214" t="inlineStr"/>
+      <c r="AO214" t="n">
+        <v>62.23230490018149</v>
+      </c>
       <c r="AP214" t="inlineStr"/>
       <c r="AQ214" t="inlineStr"/>
       <c r="AR214" t="inlineStr">

</xml_diff>

<commit_message>
Consolidate to single canonical DOCX pipeline - remove all competing parser files
Co-authored-by: danieljohnconstantine-a11y <229551202+danieljohnconstantine-a11y@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/all_dogs_master.xlsx
+++ b/outputs/all_dogs_master.xlsx
@@ -802,7 +802,7 @@
       </c>
       <c r="BF2" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -888,7 +888,7 @@
       </c>
       <c r="BF3" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="BF4" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="BF5" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="BF6" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="BF7" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="BF8" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -1404,7 +1404,7 @@
       </c>
       <c r="BF9" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="BF10" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -1576,7 +1576,7 @@
       </c>
       <c r="BF11" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="BF12" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="BF13" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1834,7 @@
       </c>
       <c r="BF14" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="BF15" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="BF16" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -2092,7 +2092,7 @@
       </c>
       <c r="BF17" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -2178,7 +2178,7 @@
       </c>
       <c r="BF18" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -2264,7 +2264,7 @@
       </c>
       <c r="BF19" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2350,7 @@
       </c>
       <c r="BF20" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="BF21" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="BF22" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="BF23" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="BF24" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -2780,7 +2780,7 @@
       </c>
       <c r="BF25" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="BF26" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="BF27" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="BF28" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -3124,7 +3124,7 @@
       </c>
       <c r="BF29" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="BF30" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="BF31" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -3382,7 +3382,7 @@
       </c>
       <c r="BF32" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -3468,7 +3468,7 @@
       </c>
       <c r="BF33" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3554,7 @@
       </c>
       <c r="BF34" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="BF35" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -3726,7 +3726,7 @@
       </c>
       <c r="BF36" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="BF37" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -3898,7 +3898,7 @@
       </c>
       <c r="BF38" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -3984,7 +3984,7 @@
       </c>
       <c r="BF39" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -4070,7 +4070,7 @@
       </c>
       <c r="BF40" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -4156,7 +4156,7 @@
       </c>
       <c r="BF41" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -4242,7 +4242,7 @@
       </c>
       <c r="BF42" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="BF43" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -4414,7 +4414,7 @@
       </c>
       <c r="BF44" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -4500,7 +4500,7 @@
       </c>
       <c r="BF45" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -4586,7 +4586,7 @@
       </c>
       <c r="BF46" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -4672,7 +4672,7 @@
       </c>
       <c r="BF47" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -4758,7 +4758,7 @@
       </c>
       <c r="BF48" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -4844,7 +4844,7 @@
       </c>
       <c r="BF49" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -4930,7 +4930,7 @@
       </c>
       <c r="BF50" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -5016,7 +5016,7 @@
       </c>
       <c r="BF51" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -5102,7 +5102,7 @@
       </c>
       <c r="BF52" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -5188,7 +5188,7 @@
       </c>
       <c r="BF53" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -5274,7 +5274,7 @@
       </c>
       <c r="BF54" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="BF55" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -5446,7 +5446,7 @@
       </c>
       <c r="BF56" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="BF57" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -5618,7 +5618,7 @@
       </c>
       <c r="BF58" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -5704,7 +5704,7 @@
       </c>
       <c r="BF59" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -5790,7 +5790,7 @@
       </c>
       <c r="BF60" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -5876,7 +5876,7 @@
       </c>
       <c r="BF61" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -5962,7 +5962,7 @@
       </c>
       <c r="BF62" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -6048,7 +6048,7 @@
       </c>
       <c r="BF63" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -6134,7 +6134,7 @@
       </c>
       <c r="BF64" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="BF65" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -6306,7 +6306,7 @@
       </c>
       <c r="BF66" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -6392,7 +6392,7 @@
       </c>
       <c r="BF67" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -6478,7 +6478,7 @@
       </c>
       <c r="BF68" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -6564,7 +6564,7 @@
       </c>
       <c r="BF69" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="BF70" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="BF71" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -6822,7 +6822,7 @@
       </c>
       <c r="BF72" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -6908,7 +6908,7 @@
       </c>
       <c r="BF73" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -6994,7 +6994,7 @@
       </c>
       <c r="BF74" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -7080,7 +7080,7 @@
       </c>
       <c r="BF75" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -7166,7 +7166,7 @@
       </c>
       <c r="BF76" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -7252,7 +7252,7 @@
       </c>
       <c r="BF77" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -7338,7 +7338,7 @@
       </c>
       <c r="BF78" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -7424,7 +7424,7 @@
       </c>
       <c r="BF79" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -7510,7 +7510,7 @@
       </c>
       <c r="BF80" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="BF81" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -7682,7 +7682,7 @@
       </c>
       <c r="BF82" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -7768,7 +7768,7 @@
       </c>
       <c r="BF83" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -7854,7 +7854,7 @@
       </c>
       <c r="BF84" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -7940,7 +7940,7 @@
       </c>
       <c r="BF85" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -8026,7 +8026,7 @@
       </c>
       <c r="BF86" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -8112,7 +8112,7 @@
       </c>
       <c r="BF87" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -8198,7 +8198,7 @@
       </c>
       <c r="BF88" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -8284,7 +8284,7 @@
       </c>
       <c r="BF89" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -8370,7 +8370,7 @@
       </c>
       <c r="BF90" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -8456,7 +8456,7 @@
       </c>
       <c r="BF91" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -8542,7 +8542,7 @@
       </c>
       <c r="BF92" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -8628,7 +8628,7 @@
       </c>
       <c r="BF93" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -8714,7 +8714,7 @@
       </c>
       <c r="BF94" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -8800,7 +8800,7 @@
       </c>
       <c r="BF95" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -8886,7 +8886,7 @@
       </c>
       <c r="BF96" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -8972,7 +8972,7 @@
       </c>
       <c r="BF97" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -9058,7 +9058,7 @@
       </c>
       <c r="BF98" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -9144,7 +9144,7 @@
       </c>
       <c r="BF99" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="BF100" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -9316,7 +9316,7 @@
       </c>
       <c r="BF101" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -9402,7 +9402,7 @@
       </c>
       <c r="BF102" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -9488,7 +9488,7 @@
       </c>
       <c r="BF103" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -9574,7 +9574,7 @@
       </c>
       <c r="BF104" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -9660,7 +9660,7 @@
       </c>
       <c r="BF105" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -9746,7 +9746,7 @@
       </c>
       <c r="BF106" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -9832,7 +9832,7 @@
       </c>
       <c r="BF107" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="BF108" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -10004,7 +10004,7 @@
       </c>
       <c r="BF109" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10090,7 @@
       </c>
       <c r="BF110" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -10176,7 +10176,7 @@
       </c>
       <c r="BF111" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -10262,7 +10262,7 @@
       </c>
       <c r="BF112" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -10348,7 +10348,7 @@
       </c>
       <c r="BF113" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -10434,7 +10434,7 @@
       </c>
       <c r="BF114" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -10520,7 +10520,7 @@
       </c>
       <c r="BF115" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -10606,7 +10606,7 @@
       </c>
       <c r="BF116" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -10692,7 +10692,7 @@
       </c>
       <c r="BF117" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -10778,7 +10778,7 @@
       </c>
       <c r="BF118" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -10864,7 +10864,7 @@
       </c>
       <c r="BF119" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -10950,7 +10950,7 @@
       </c>
       <c r="BF120" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -11036,7 +11036,7 @@
       </c>
       <c r="BF121" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -11122,7 +11122,7 @@
       </c>
       <c r="BF122" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -11208,7 +11208,7 @@
       </c>
       <c r="BF123" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -11294,7 +11294,7 @@
       </c>
       <c r="BF124" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -11380,7 +11380,7 @@
       </c>
       <c r="BF125" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -11466,7 +11466,7 @@
       </c>
       <c r="BF126" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -11552,7 +11552,7 @@
       </c>
       <c r="BF127" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -11638,7 +11638,7 @@
       </c>
       <c r="BF128" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -11724,7 +11724,7 @@
       </c>
       <c r="BF129" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -11810,7 +11810,7 @@
       </c>
       <c r="BF130" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -11896,7 +11896,7 @@
       </c>
       <c r="BF131" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -11982,7 +11982,7 @@
       </c>
       <c r="BF132" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -12068,7 +12068,7 @@
       </c>
       <c r="BF133" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -12154,7 +12154,7 @@
       </c>
       <c r="BF134" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -12240,7 +12240,7 @@
       </c>
       <c r="BF135" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -12326,7 +12326,7 @@
       </c>
       <c r="BF136" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -12412,7 +12412,7 @@
       </c>
       <c r="BF137" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -12498,7 +12498,7 @@
       </c>
       <c r="BF138" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -12584,7 +12584,7 @@
       </c>
       <c r="BF139" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -12670,7 +12670,7 @@
       </c>
       <c r="BF140" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -12756,7 +12756,7 @@
       </c>
       <c r="BF141" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -12842,7 +12842,7 @@
       </c>
       <c r="BF142" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -12928,7 +12928,7 @@
       </c>
       <c r="BF143" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -13014,7 +13014,7 @@
       </c>
       <c r="BF144" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -13100,7 +13100,7 @@
       </c>
       <c r="BF145" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -13186,7 +13186,7 @@
       </c>
       <c r="BF146" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -13272,7 +13272,7 @@
       </c>
       <c r="BF147" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -13358,7 +13358,7 @@
       </c>
       <c r="BF148" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -13444,7 +13444,7 @@
       </c>
       <c r="BF149" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -13530,7 +13530,7 @@
       </c>
       <c r="BF150" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -13616,7 +13616,7 @@
       </c>
       <c r="BF151" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -13702,7 +13702,7 @@
       </c>
       <c r="BF152" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -13788,7 +13788,7 @@
       </c>
       <c r="BF153" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -13874,7 +13874,7 @@
       </c>
       <c r="BF154" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -13960,7 +13960,7 @@
       </c>
       <c r="BF155" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -14046,7 +14046,7 @@
       </c>
       <c r="BF156" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -14132,7 +14132,7 @@
       </c>
       <c r="BF157" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -14218,7 +14218,7 @@
       </c>
       <c r="BF158" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -14304,7 +14304,7 @@
       </c>
       <c r="BF159" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -14390,7 +14390,7 @@
       </c>
       <c r="BF160" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -14476,7 +14476,7 @@
       </c>
       <c r="BF161" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -14562,7 +14562,7 @@
       </c>
       <c r="BF162" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -14648,7 +14648,7 @@
       </c>
       <c r="BF163" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -14734,7 +14734,7 @@
       </c>
       <c r="BF164" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -14820,7 +14820,7 @@
       </c>
       <c r="BF165" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -14906,7 +14906,7 @@
       </c>
       <c r="BF166" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -14992,7 +14992,7 @@
       </c>
       <c r="BF167" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -15078,7 +15078,7 @@
       </c>
       <c r="BF168" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -15164,7 +15164,7 @@
       </c>
       <c r="BF169" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -15250,7 +15250,7 @@
       </c>
       <c r="BF170" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -15336,7 +15336,7 @@
       </c>
       <c r="BF171" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -15422,7 +15422,7 @@
       </c>
       <c r="BF172" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -15508,7 +15508,7 @@
       </c>
       <c r="BF173" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -15594,7 +15594,7 @@
       </c>
       <c r="BF174" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -15680,7 +15680,7 @@
       </c>
       <c r="BF175" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -15766,7 +15766,7 @@
       </c>
       <c r="BF176" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -15852,7 +15852,7 @@
       </c>
       <c r="BF177" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -15938,7 +15938,7 @@
       </c>
       <c r="BF178" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -16024,7 +16024,7 @@
       </c>
       <c r="BF179" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -16110,7 +16110,7 @@
       </c>
       <c r="BF180" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -16196,7 +16196,7 @@
       </c>
       <c r="BF181" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -16282,7 +16282,7 @@
       </c>
       <c r="BF182" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -16368,7 +16368,7 @@
       </c>
       <c r="BF183" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -16454,7 +16454,7 @@
       </c>
       <c r="BF184" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -16540,7 +16540,7 @@
       </c>
       <c r="BF185" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -16626,7 +16626,7 @@
       </c>
       <c r="BF186" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -16712,7 +16712,7 @@
       </c>
       <c r="BF187" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -16798,7 +16798,7 @@
       </c>
       <c r="BF188" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -16884,7 +16884,7 @@
       </c>
       <c r="BF189" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -16970,7 +16970,7 @@
       </c>
       <c r="BF190" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -17056,7 +17056,7 @@
       </c>
       <c r="BF191" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -17142,7 +17142,7 @@
       </c>
       <c r="BF192" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -17228,7 +17228,7 @@
       </c>
       <c r="BF193" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -17314,7 +17314,7 @@
       </c>
       <c r="BF194" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -17400,7 +17400,7 @@
       </c>
       <c r="BF195" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -17486,7 +17486,7 @@
       </c>
       <c r="BF196" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -17572,7 +17572,7 @@
       </c>
       <c r="BF197" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -17658,7 +17658,7 @@
       </c>
       <c r="BF198" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -17744,7 +17744,7 @@
       </c>
       <c r="BF199" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -17830,7 +17830,7 @@
       </c>
       <c r="BF200" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -17916,7 +17916,7 @@
       </c>
       <c r="BF201" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -18002,7 +18002,7 @@
       </c>
       <c r="BF202" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -18088,7 +18088,7 @@
       </c>
       <c r="BF203" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -18174,7 +18174,7 @@
       </c>
       <c r="BF204" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -18260,7 +18260,7 @@
       </c>
       <c r="BF205" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -18346,7 +18346,7 @@
       </c>
       <c r="BF206" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -18432,7 +18432,7 @@
       </c>
       <c r="BF207" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -18518,7 +18518,7 @@
       </c>
       <c r="BF208" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -18604,7 +18604,7 @@
       </c>
       <c r="BF209" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -18690,7 +18690,7 @@
       </c>
       <c r="BF210" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -18776,7 +18776,7 @@
       </c>
       <c r="BF211" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -18862,7 +18862,7 @@
       </c>
       <c r="BF212" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -18948,7 +18948,7 @@
       </c>
       <c r="BF213" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -19034,7 +19034,7 @@
       </c>
       <c r="BF214" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -19120,7 +19120,7 @@
       </c>
       <c r="BF215" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -19206,7 +19206,7 @@
       </c>
       <c r="BF216" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -19292,7 +19292,7 @@
       </c>
       <c r="BF217" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -19378,7 +19378,7 @@
       </c>
       <c r="BF218" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -19464,7 +19464,7 @@
       </c>
       <c r="BF219" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -19550,7 +19550,7 @@
       </c>
       <c r="BF220" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -19636,7 +19636,7 @@
       </c>
       <c r="BF221" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -19722,7 +19722,7 @@
       </c>
       <c r="BF222" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -19808,7 +19808,7 @@
       </c>
       <c r="BF223" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -19894,7 +19894,7 @@
       </c>
       <c r="BF224" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -19980,7 +19980,7 @@
       </c>
       <c r="BF225" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -20066,7 +20066,7 @@
       </c>
       <c r="BF226" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -20152,7 +20152,7 @@
       </c>
       <c r="BF227" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -20238,7 +20238,7 @@
       </c>
       <c r="BF228" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -20324,7 +20324,7 @@
       </c>
       <c r="BF229" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -20410,7 +20410,7 @@
       </c>
       <c r="BF230" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -20496,7 +20496,7 @@
       </c>
       <c r="BF231" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -20582,7 +20582,7 @@
       </c>
       <c r="BF232" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -20668,7 +20668,7 @@
       </c>
       <c r="BF233" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -20754,7 +20754,7 @@
       </c>
       <c r="BF234" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -20840,7 +20840,7 @@
       </c>
       <c r="BF235" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -20926,7 +20926,7 @@
       </c>
       <c r="BF236" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -21012,7 +21012,7 @@
       </c>
       <c r="BF237" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -21098,7 +21098,7 @@
       </c>
       <c r="BF238" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -21184,7 +21184,7 @@
       </c>
       <c r="BF239" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -21270,7 +21270,7 @@
       </c>
       <c r="BF240" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -21356,7 +21356,7 @@
       </c>
       <c r="BF241" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -21442,7 +21442,7 @@
       </c>
       <c r="BF242" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -21528,7 +21528,7 @@
       </c>
       <c r="BF243" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -21614,7 +21614,7 @@
       </c>
       <c r="BF244" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -21700,7 +21700,7 @@
       </c>
       <c r="BF245" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -21786,7 +21786,7 @@
       </c>
       <c r="BF246" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -21872,7 +21872,7 @@
       </c>
       <c r="BF247" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -21958,7 +21958,7 @@
       </c>
       <c r="BF248" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -22044,7 +22044,7 @@
       </c>
       <c r="BF249" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -22130,7 +22130,7 @@
       </c>
       <c r="BF250" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -22216,7 +22216,7 @@
       </c>
       <c r="BF251" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -22302,7 +22302,7 @@
       </c>
       <c r="BF252" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -22388,7 +22388,7 @@
       </c>
       <c r="BF253" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -22474,7 +22474,7 @@
       </c>
       <c r="BF254" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -22560,7 +22560,7 @@
       </c>
       <c r="BF255" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -22646,7 +22646,7 @@
       </c>
       <c r="BF256" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -22732,7 +22732,7 @@
       </c>
       <c r="BF257" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -22818,7 +22818,7 @@
       </c>
       <c r="BF258" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -22904,7 +22904,7 @@
       </c>
       <c r="BF259" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -22990,7 +22990,7 @@
       </c>
       <c r="BF260" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -23076,7 +23076,7 @@
       </c>
       <c r="BF261" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -23162,7 +23162,7 @@
       </c>
       <c r="BF262" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -23248,7 +23248,7 @@
       </c>
       <c r="BF263" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -23334,7 +23334,7 @@
       </c>
       <c r="BF264" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -23420,7 +23420,7 @@
       </c>
       <c r="BF265" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -23506,7 +23506,7 @@
       </c>
       <c r="BF266" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -23592,7 +23592,7 @@
       </c>
       <c r="BF267" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -23678,7 +23678,7 @@
       </c>
       <c r="BF268" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -23764,7 +23764,7 @@
       </c>
       <c r="BF269" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -23850,7 +23850,7 @@
       </c>
       <c r="BF270" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -23936,7 +23936,7 @@
       </c>
       <c r="BF271" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -24022,7 +24022,7 @@
       </c>
       <c r="BF272" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -24108,7 +24108,7 @@
       </c>
       <c r="BF273" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -24194,7 +24194,7 @@
       </c>
       <c r="BF274" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -24280,7 +24280,7 @@
       </c>
       <c r="BF275" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -24366,7 +24366,7 @@
       </c>
       <c r="BF276" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -24452,7 +24452,7 @@
       </c>
       <c r="BF277" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -24538,7 +24538,7 @@
       </c>
       <c r="BF278" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -24624,7 +24624,7 @@
       </c>
       <c r="BF279" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -24710,7 +24710,7 @@
       </c>
       <c r="BF280" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -24796,7 +24796,7 @@
       </c>
       <c r="BF281" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -24882,7 +24882,7 @@
       </c>
       <c r="BF282" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -24968,7 +24968,7 @@
       </c>
       <c r="BF283" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -25054,7 +25054,7 @@
       </c>
       <c r="BF284" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -25140,7 +25140,7 @@
       </c>
       <c r="BF285" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -25226,7 +25226,7 @@
       </c>
       <c r="BF286" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -25312,7 +25312,7 @@
       </c>
       <c r="BF287" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -25398,7 +25398,7 @@
       </c>
       <c r="BF288" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -25484,7 +25484,7 @@
       </c>
       <c r="BF289" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -25570,7 +25570,7 @@
       </c>
       <c r="BF290" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -25656,7 +25656,7 @@
       </c>
       <c r="BF291" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -25742,7 +25742,7 @@
       </c>
       <c r="BF292" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -25828,7 +25828,7 @@
       </c>
       <c r="BF293" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -25914,7 +25914,7 @@
       </c>
       <c r="BF294" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -26000,7 +26000,7 @@
       </c>
       <c r="BF295" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -26086,7 +26086,7 @@
       </c>
       <c r="BF296" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -26172,7 +26172,7 @@
       </c>
       <c r="BF297" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -26258,7 +26258,7 @@
       </c>
       <c r="BF298" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -26344,7 +26344,7 @@
       </c>
       <c r="BF299" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -26430,7 +26430,7 @@
       </c>
       <c r="BF300" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -26516,7 +26516,7 @@
       </c>
       <c r="BF301" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -26602,7 +26602,7 @@
       </c>
       <c r="BF302" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -26688,7 +26688,7 @@
       </c>
       <c r="BF303" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -26774,7 +26774,7 @@
       </c>
       <c r="BF304" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -26860,7 +26860,7 @@
       </c>
       <c r="BF305" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -26946,7 +26946,7 @@
       </c>
       <c r="BF306" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>
@@ -27032,7 +27032,7 @@
       </c>
       <c r="BF307" t="inlineStr">
         <is>
-          <t>2025-11-15T09:56:48.334822</t>
+          <t>2025-11-15T10:55:46.629790</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Final status - 13 fields extracted from DOCX (Track, Race_Date, Trainer, Sire, Dam, Owner, Career_W-P-S, Prize_Money, RTC, DLR, DLW)
Co-authored-by: danieljohnconstantine-a11y <229551202+danieljohnconstantine-a11y@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/all_dogs_master.xlsx
+++ b/outputs/all_dogs_master.xlsx
@@ -826,7 +826,7 @@
       </c>
       <c r="BF2" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="BF3" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="BF4" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1156,7 @@
       </c>
       <c r="BF5" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="BF6" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="BF7" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="BF8" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -1580,7 +1580,7 @@
       </c>
       <c r="BF9" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1686,7 @@
       </c>
       <c r="BF10" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1796,7 @@
       </c>
       <c r="BF11" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1906,7 @@
       </c>
       <c r="BF12" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="BF13" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="BF14" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -2236,7 +2236,7 @@
       </c>
       <c r="BF15" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -2342,7 +2342,7 @@
       </c>
       <c r="BF16" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="BF17" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="BF18" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -2668,7 +2668,7 @@
       </c>
       <c r="BF19" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -2774,7 +2774,7 @@
       </c>
       <c r="BF20" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="BF21" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -2982,7 +2982,7 @@
       </c>
       <c r="BF22" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="BF23" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="BF24" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="BF25" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3418,7 @@
       </c>
       <c r="BF26" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -3528,7 +3528,7 @@
       </c>
       <c r="BF27" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -3638,7 +3638,7 @@
       </c>
       <c r="BF28" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -3744,7 +3744,7 @@
       </c>
       <c r="BF29" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -3846,7 +3846,7 @@
       </c>
       <c r="BF30" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -3952,7 +3952,7 @@
       </c>
       <c r="BF31" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -4058,7 +4058,7 @@
       </c>
       <c r="BF32" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -4160,7 +4160,7 @@
       </c>
       <c r="BF33" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -4270,7 +4270,7 @@
       </c>
       <c r="BF34" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -4380,7 +4380,7 @@
       </c>
       <c r="BF35" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="BF36" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="BF37" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -4690,7 +4690,7 @@
       </c>
       <c r="BF38" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="BF39" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="BF40" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -5012,7 +5012,7 @@
       </c>
       <c r="BF41" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -5122,7 +5122,7 @@
       </c>
       <c r="BF42" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -5228,7 +5228,7 @@
       </c>
       <c r="BF43" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -5334,7 +5334,7 @@
       </c>
       <c r="BF44" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -5444,7 +5444,7 @@
       </c>
       <c r="BF45" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -5554,7 +5554,7 @@
       </c>
       <c r="BF46" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -5664,7 +5664,7 @@
       </c>
       <c r="BF47" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -5762,7 +5762,7 @@
       </c>
       <c r="BF48" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -5872,7 +5872,7 @@
       </c>
       <c r="BF49" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -5978,7 +5978,7 @@
       </c>
       <c r="BF50" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -6084,7 +6084,7 @@
       </c>
       <c r="BF51" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -6190,7 +6190,7 @@
       </c>
       <c r="BF52" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="BF53" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -6398,7 +6398,7 @@
       </c>
       <c r="BF54" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="BF55" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -6614,7 +6614,7 @@
       </c>
       <c r="BF56" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -6720,7 +6720,7 @@
       </c>
       <c r="BF57" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -6830,7 +6830,7 @@
       </c>
       <c r="BF58" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -6940,7 +6940,7 @@
       </c>
       <c r="BF59" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -7050,7 +7050,7 @@
       </c>
       <c r="BF60" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -7160,7 +7160,7 @@
       </c>
       <c r="BF61" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -7258,7 +7258,7 @@
       </c>
       <c r="BF62" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -7360,7 +7360,7 @@
       </c>
       <c r="BF63" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -7470,7 +7470,7 @@
       </c>
       <c r="BF64" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -7572,7 +7572,7 @@
       </c>
       <c r="BF65" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -7658,7 +7658,7 @@
       </c>
       <c r="BF66" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -7768,7 +7768,7 @@
       </c>
       <c r="BF67" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -7870,7 +7870,7 @@
       </c>
       <c r="BF68" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -7980,7 +7980,7 @@
       </c>
       <c r="BF69" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -8086,7 +8086,7 @@
       </c>
       <c r="BF70" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -8184,7 +8184,7 @@
       </c>
       <c r="BF71" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -8290,7 +8290,7 @@
       </c>
       <c r="BF72" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -8392,7 +8392,7 @@
       </c>
       <c r="BF73" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -8490,7 +8490,7 @@
       </c>
       <c r="BF74" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -8596,7 +8596,7 @@
       </c>
       <c r="BF75" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -8706,7 +8706,7 @@
       </c>
       <c r="BF76" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -8808,7 +8808,7 @@
       </c>
       <c r="BF77" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -8918,7 +8918,7 @@
       </c>
       <c r="BF78" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -9024,7 +9024,7 @@
       </c>
       <c r="BF79" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -9134,7 +9134,7 @@
       </c>
       <c r="BF80" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -9240,7 +9240,7 @@
       </c>
       <c r="BF81" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -9346,7 +9346,7 @@
       </c>
       <c r="BF82" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -9456,7 +9456,7 @@
       </c>
       <c r="BF83" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -9566,7 +9566,7 @@
       </c>
       <c r="BF84" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="BF85" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -9738,7 +9738,7 @@
       </c>
       <c r="BF86" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -9824,7 +9824,7 @@
       </c>
       <c r="BF87" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -9910,7 +9910,7 @@
       </c>
       <c r="BF88" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -9996,7 +9996,7 @@
       </c>
       <c r="BF89" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -10082,7 +10082,7 @@
       </c>
       <c r="BF90" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -10168,7 +10168,7 @@
       </c>
       <c r="BF91" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -10254,7 +10254,7 @@
       </c>
       <c r="BF92" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -10340,7 +10340,7 @@
       </c>
       <c r="BF93" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -10426,7 +10426,7 @@
       </c>
       <c r="BF94" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -10512,7 +10512,7 @@
       </c>
       <c r="BF95" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -10598,7 +10598,7 @@
       </c>
       <c r="BF96" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -10684,7 +10684,7 @@
       </c>
       <c r="BF97" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -10770,7 +10770,7 @@
       </c>
       <c r="BF98" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -10856,7 +10856,7 @@
       </c>
       <c r="BF99" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -10942,7 +10942,7 @@
       </c>
       <c r="BF100" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -11028,7 +11028,7 @@
       </c>
       <c r="BF101" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -11114,7 +11114,7 @@
       </c>
       <c r="BF102" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -11216,7 +11216,7 @@
       </c>
       <c r="BF103" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -11326,7 +11326,7 @@
       </c>
       <c r="BF104" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -11436,7 +11436,7 @@
       </c>
       <c r="BF105" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -11546,7 +11546,7 @@
       </c>
       <c r="BF106" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -11656,7 +11656,7 @@
       </c>
       <c r="BF107" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -11766,7 +11766,7 @@
       </c>
       <c r="BF108" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -11876,7 +11876,7 @@
       </c>
       <c r="BF109" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -11986,7 +11986,7 @@
       </c>
       <c r="BF110" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -12092,7 +12092,7 @@
       </c>
       <c r="BF111" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -12198,7 +12198,7 @@
       </c>
       <c r="BF112" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -12308,7 +12308,7 @@
       </c>
       <c r="BF113" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -12418,7 +12418,7 @@
       </c>
       <c r="BF114" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -12528,7 +12528,7 @@
       </c>
       <c r="BF115" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -12638,7 +12638,7 @@
       </c>
       <c r="BF116" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -12748,7 +12748,7 @@
       </c>
       <c r="BF117" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -12854,7 +12854,7 @@
       </c>
       <c r="BF118" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -12960,7 +12960,7 @@
       </c>
       <c r="BF119" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -13066,7 +13066,7 @@
       </c>
       <c r="BF120" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -13172,7 +13172,7 @@
       </c>
       <c r="BF121" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -13258,7 +13258,7 @@
       </c>
       <c r="BF122" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13364,7 @@
       </c>
       <c r="BF123" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -13462,7 +13462,7 @@
       </c>
       <c r="BF124" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -13568,7 +13568,7 @@
       </c>
       <c r="BF125" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -13678,7 +13678,7 @@
       </c>
       <c r="BF126" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -13780,7 +13780,7 @@
       </c>
       <c r="BF127" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -13890,7 +13890,7 @@
       </c>
       <c r="BF128" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -13996,7 +13996,7 @@
       </c>
       <c r="BF129" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -14098,7 +14098,7 @@
       </c>
       <c r="BF130" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -14208,7 +14208,7 @@
       </c>
       <c r="BF131" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -14318,7 +14318,7 @@
       </c>
       <c r="BF132" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -14428,7 +14428,7 @@
       </c>
       <c r="BF133" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -14538,7 +14538,7 @@
       </c>
       <c r="BF134" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -14644,7 +14644,7 @@
       </c>
       <c r="BF135" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -14754,7 +14754,7 @@
       </c>
       <c r="BF136" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -14864,7 +14864,7 @@
       </c>
       <c r="BF137" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -14970,7 +14970,7 @@
       </c>
       <c r="BF138" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -15080,7 +15080,7 @@
       </c>
       <c r="BF139" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -15182,7 +15182,7 @@
       </c>
       <c r="BF140" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -15292,7 +15292,7 @@
       </c>
       <c r="BF141" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -15402,7 +15402,7 @@
       </c>
       <c r="BF142" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -15512,7 +15512,7 @@
       </c>
       <c r="BF143" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -15614,7 +15614,7 @@
       </c>
       <c r="BF144" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -15724,7 +15724,7 @@
       </c>
       <c r="BF145" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -15834,7 +15834,7 @@
       </c>
       <c r="BF146" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -15932,7 +15932,7 @@
       </c>
       <c r="BF147" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -16042,7 +16042,7 @@
       </c>
       <c r="BF148" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -16152,7 +16152,7 @@
       </c>
       <c r="BF149" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -16258,7 +16258,7 @@
       </c>
       <c r="BF150" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -16368,7 +16368,7 @@
       </c>
       <c r="BF151" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -16454,7 +16454,7 @@
       </c>
       <c r="BF152" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -16560,7 +16560,7 @@
       </c>
       <c r="BF153" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -16670,7 +16670,7 @@
       </c>
       <c r="BF154" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -16780,7 +16780,7 @@
       </c>
       <c r="BF155" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -16886,7 +16886,7 @@
       </c>
       <c r="BF156" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -16996,7 +16996,7 @@
       </c>
       <c r="BF157" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -17102,7 +17102,7 @@
       </c>
       <c r="BF158" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -17208,7 +17208,7 @@
       </c>
       <c r="BF159" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -17314,7 +17314,7 @@
       </c>
       <c r="BF160" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -17420,7 +17420,7 @@
       </c>
       <c r="BF161" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -17530,7 +17530,7 @@
       </c>
       <c r="BF162" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -17640,7 +17640,7 @@
       </c>
       <c r="BF163" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -17750,7 +17750,7 @@
       </c>
       <c r="BF164" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -17860,7 +17860,7 @@
       </c>
       <c r="BF165" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -17970,7 +17970,7 @@
       </c>
       <c r="BF166" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -18072,7 +18072,7 @@
       </c>
       <c r="BF167" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -18178,7 +18178,7 @@
       </c>
       <c r="BF168" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -18288,7 +18288,7 @@
       </c>
       <c r="BF169" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -18398,7 +18398,7 @@
       </c>
       <c r="BF170" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -18504,7 +18504,7 @@
       </c>
       <c r="BF171" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -18614,7 +18614,7 @@
       </c>
       <c r="BF172" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -18716,7 +18716,7 @@
       </c>
       <c r="BF173" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -18822,7 +18822,7 @@
       </c>
       <c r="BF174" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -18928,7 +18928,7 @@
       </c>
       <c r="BF175" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -19034,7 +19034,7 @@
       </c>
       <c r="BF176" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -19144,7 +19144,7 @@
       </c>
       <c r="BF177" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -19242,7 +19242,7 @@
       </c>
       <c r="BF178" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -19348,7 +19348,7 @@
       </c>
       <c r="BF179" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -19454,7 +19454,7 @@
       </c>
       <c r="BF180" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -19560,7 +19560,7 @@
       </c>
       <c r="BF181" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -19666,7 +19666,7 @@
       </c>
       <c r="BF182" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -19752,7 +19752,7 @@
       </c>
       <c r="BF183" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -19838,7 +19838,7 @@
       </c>
       <c r="BF184" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -19924,7 +19924,7 @@
       </c>
       <c r="BF185" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -20010,7 +20010,7 @@
       </c>
       <c r="BF186" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -20096,7 +20096,7 @@
       </c>
       <c r="BF187" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -20182,7 +20182,7 @@
       </c>
       <c r="BF188" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -20268,7 +20268,7 @@
       </c>
       <c r="BF189" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -20354,7 +20354,7 @@
       </c>
       <c r="BF190" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -20440,7 +20440,7 @@
       </c>
       <c r="BF191" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -20550,7 +20550,7 @@
       </c>
       <c r="BF192" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -20656,7 +20656,7 @@
       </c>
       <c r="BF193" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -20766,7 +20766,7 @@
       </c>
       <c r="BF194" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -20872,7 +20872,7 @@
       </c>
       <c r="BF195" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -20978,7 +20978,7 @@
       </c>
       <c r="BF196" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -21088,7 +21088,7 @@
       </c>
       <c r="BF197" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -21190,7 +21190,7 @@
       </c>
       <c r="BF198" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -21300,7 +21300,7 @@
       </c>
       <c r="BF199" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -21406,7 +21406,7 @@
       </c>
       <c r="BF200" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -21508,7 +21508,7 @@
       </c>
       <c r="BF201" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -21614,7 +21614,7 @@
       </c>
       <c r="BF202" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -21724,7 +21724,7 @@
       </c>
       <c r="BF203" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -21826,7 +21826,7 @@
       </c>
       <c r="BF204" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -21936,7 +21936,7 @@
       </c>
       <c r="BF205" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -22046,7 +22046,7 @@
       </c>
       <c r="BF206" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -22156,7 +22156,7 @@
       </c>
       <c r="BF207" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -22262,7 +22262,7 @@
       </c>
       <c r="BF208" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -22368,7 +22368,7 @@
       </c>
       <c r="BF209" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -22474,7 +22474,7 @@
       </c>
       <c r="BF210" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -22576,7 +22576,7 @@
       </c>
       <c r="BF211" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -22686,7 +22686,7 @@
       </c>
       <c r="BF212" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -22792,7 +22792,7 @@
       </c>
       <c r="BF213" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -22898,7 +22898,7 @@
       </c>
       <c r="BF214" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -23004,7 +23004,7 @@
       </c>
       <c r="BF215" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -23114,7 +23114,7 @@
       </c>
       <c r="BF216" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -23220,7 +23220,7 @@
       </c>
       <c r="BF217" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -23330,7 +23330,7 @@
       </c>
       <c r="BF218" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -23440,7 +23440,7 @@
       </c>
       <c r="BF219" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -23538,7 +23538,7 @@
       </c>
       <c r="BF220" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -23644,7 +23644,7 @@
       </c>
       <c r="BF221" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -23750,7 +23750,7 @@
       </c>
       <c r="BF222" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -23860,7 +23860,7 @@
       </c>
       <c r="BF223" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -23970,7 +23970,7 @@
       </c>
       <c r="BF224" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -24072,7 +24072,7 @@
       </c>
       <c r="BF225" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -24174,7 +24174,7 @@
       </c>
       <c r="BF226" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -24276,7 +24276,7 @@
       </c>
       <c r="BF227" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -24374,7 +24374,7 @@
       </c>
       <c r="BF228" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -24480,7 +24480,7 @@
       </c>
       <c r="BF229" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -24582,7 +24582,7 @@
       </c>
       <c r="BF230" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -24684,7 +24684,7 @@
       </c>
       <c r="BF231" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -24794,7 +24794,7 @@
       </c>
       <c r="BF232" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -24904,7 +24904,7 @@
       </c>
       <c r="BF233" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -25014,7 +25014,7 @@
       </c>
       <c r="BF234" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -25124,7 +25124,7 @@
       </c>
       <c r="BF235" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -25234,7 +25234,7 @@
       </c>
       <c r="BF236" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -25340,7 +25340,7 @@
       </c>
       <c r="BF237" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -25450,7 +25450,7 @@
       </c>
       <c r="BF238" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -25556,7 +25556,7 @@
       </c>
       <c r="BF239" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -25666,7 +25666,7 @@
       </c>
       <c r="BF240" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -25768,7 +25768,7 @@
       </c>
       <c r="BF241" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -25870,7 +25870,7 @@
       </c>
       <c r="BF242" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -25976,7 +25976,7 @@
       </c>
       <c r="BF243" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -26086,7 +26086,7 @@
       </c>
       <c r="BF244" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -26172,7 +26172,7 @@
       </c>
       <c r="BF245" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -26278,7 +26278,7 @@
       </c>
       <c r="BF246" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -26388,7 +26388,7 @@
       </c>
       <c r="BF247" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -26494,7 +26494,7 @@
       </c>
       <c r="BF248" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -26600,7 +26600,7 @@
       </c>
       <c r="BF249" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -26706,7 +26706,7 @@
       </c>
       <c r="BF250" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -26812,7 +26812,7 @@
       </c>
       <c r="BF251" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -26922,7 +26922,7 @@
       </c>
       <c r="BF252" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -27024,7 +27024,7 @@
       </c>
       <c r="BF253" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -27130,7 +27130,7 @@
       </c>
       <c r="BF254" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -27240,7 +27240,7 @@
       </c>
       <c r="BF255" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -27350,7 +27350,7 @@
       </c>
       <c r="BF256" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -27448,7 +27448,7 @@
       </c>
       <c r="BF257" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -27558,7 +27558,7 @@
       </c>
       <c r="BF258" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -27668,7 +27668,7 @@
       </c>
       <c r="BF259" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -27770,7 +27770,7 @@
       </c>
       <c r="BF260" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -27876,7 +27876,7 @@
       </c>
       <c r="BF261" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -27982,7 +27982,7 @@
       </c>
       <c r="BF262" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -28084,7 +28084,7 @@
       </c>
       <c r="BF263" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -28194,7 +28194,7 @@
       </c>
       <c r="BF264" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -28304,7 +28304,7 @@
       </c>
       <c r="BF265" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -28406,7 +28406,7 @@
       </c>
       <c r="BF266" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -28516,7 +28516,7 @@
       </c>
       <c r="BF267" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -28626,7 +28626,7 @@
       </c>
       <c r="BF268" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -28732,7 +28732,7 @@
       </c>
       <c r="BF269" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -28842,7 +28842,7 @@
       </c>
       <c r="BF270" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -28948,7 +28948,7 @@
       </c>
       <c r="BF271" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -29050,7 +29050,7 @@
       </c>
       <c r="BF272" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -29156,7 +29156,7 @@
       </c>
       <c r="BF273" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -29262,7 +29262,7 @@
       </c>
       <c r="BF274" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -29372,7 +29372,7 @@
       </c>
       <c r="BF275" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -29470,7 +29470,7 @@
       </c>
       <c r="BF276" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -29576,7 +29576,7 @@
       </c>
       <c r="BF277" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -29686,7 +29686,7 @@
       </c>
       <c r="BF278" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -29784,7 +29784,7 @@
       </c>
       <c r="BF279" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -29890,7 +29890,7 @@
       </c>
       <c r="BF280" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -30000,7 +30000,7 @@
       </c>
       <c r="BF281" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -30110,7 +30110,7 @@
       </c>
       <c r="BF282" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -30216,7 +30216,7 @@
       </c>
       <c r="BF283" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -30322,7 +30322,7 @@
       </c>
       <c r="BF284" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -30424,7 +30424,7 @@
       </c>
       <c r="BF285" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -30522,7 +30522,7 @@
       </c>
       <c r="BF286" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -30624,7 +30624,7 @@
       </c>
       <c r="BF287" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -30730,7 +30730,7 @@
       </c>
       <c r="BF288" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -30840,7 +30840,7 @@
       </c>
       <c r="BF289" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -30926,7 +30926,7 @@
       </c>
       <c r="BF290" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -31012,7 +31012,7 @@
       </c>
       <c r="BF291" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -31098,7 +31098,7 @@
       </c>
       <c r="BF292" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -31184,7 +31184,7 @@
       </c>
       <c r="BF293" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -31270,7 +31270,7 @@
       </c>
       <c r="BF294" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -31356,7 +31356,7 @@
       </c>
       <c r="BF295" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -31442,7 +31442,7 @@
       </c>
       <c r="BF296" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -31544,7 +31544,7 @@
       </c>
       <c r="BF297" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -31630,7 +31630,7 @@
       </c>
       <c r="BF298" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -31716,7 +31716,7 @@
       </c>
       <c r="BF299" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -31802,7 +31802,7 @@
       </c>
       <c r="BF300" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -31888,7 +31888,7 @@
       </c>
       <c r="BF301" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -31974,7 +31974,7 @@
       </c>
       <c r="BF302" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -32060,7 +32060,7 @@
       </c>
       <c r="BF303" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -32146,7 +32146,7 @@
       </c>
       <c r="BF304" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -32252,7 +32252,7 @@
       </c>
       <c r="BF305" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -32338,7 +32338,7 @@
       </c>
       <c r="BF306" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>
@@ -32424,7 +32424,7 @@
       </c>
       <c r="BF307" t="inlineStr">
         <is>
-          <t>2025-11-15T23:37:41.662088</t>
+          <t>2025-11-16T02:11:24.063096</t>
         </is>
       </c>
     </row>

</xml_diff>